<commit_message>
Update intent tool: move dropdown to H7, add group collapse for STEP2, fix script text
- Dropdown moved from H5 to H7 (within STEP1 title row)
- Script text: お支払方法 → ご契約方法
- STEP2 ①②/③ sections use row outline grouping (collapsed by default)
- Removed A/B suffixes from STEP2 labels

https://claude.ai/code/session_01AJdG4TQantm5HZTxDeQNzp
</commit_message>
<xml_diff>
--- a/intent_tool.xlsx
+++ b/intent_tool.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="32">
+  <fonts count="31">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -51,14 +51,8 @@
     <font>
       <name val="Meiryo UI"/>
       <b val="1"/>
-      <color rgb="00000000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Meiryo UI"/>
-      <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="10"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Meiryo UI"/>
@@ -86,6 +80,18 @@
     <font>
       <name val="Meiryo UI"/>
       <b val="1"/>
+      <color rgb="00C0392B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Meiryo UI"/>
+      <b val="1"/>
+      <color rgb="00C0392B"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Meiryo UI"/>
+      <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
@@ -99,11 +105,6 @@
       <name val="Meiryo UI"/>
       <color rgb="00404B3A"/>
       <sz val="8"/>
-    </font>
-    <font>
-      <name val="Meiryo UI"/>
-      <color rgb="007A8575"/>
-      <sz val="7"/>
     </font>
     <font>
       <name val="Meiryo UI"/>
@@ -126,12 +127,6 @@
     <font>
       <name val="Meiryo UI"/>
       <b val="1"/>
-      <color rgb="00C0392B"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="Meiryo UI"/>
-      <b val="1"/>
       <color rgb="00B8DEC9"/>
       <sz val="8"/>
     </font>
@@ -143,7 +138,7 @@
     <font>
       <name val="Meiryo UI"/>
       <b val="1"/>
-      <color rgb="002E7D5B"/>
+      <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
@@ -192,16 +187,17 @@
     </font>
     <font>
       <name val="Meiryo UI"/>
-      <color rgb="009B2335"/>
-      <sz val="8"/>
+      <color rgb="0093B8DC"/>
+      <sz val="7"/>
     </font>
     <font>
       <name val="Meiryo UI"/>
-      <color rgb="0093B8DC"/>
-      <sz val="7"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="23">
+  <fills count="24">
     <fill>
       <patternFill/>
     </fill>
@@ -251,6 +247,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00DCE8F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF0F0"/>
       </patternFill>
     </fill>
     <fill>
@@ -314,7 +315,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -347,6 +348,20 @@
         <color rgb="00C0392B"/>
       </top>
       <bottom style="medium">
+        <color rgb="00C0392B"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00C0392B"/>
+      </left>
+      <right style="thin">
+        <color rgb="00C0392B"/>
+      </right>
+      <top style="thin">
+        <color rgb="00C0392B"/>
+      </top>
+      <bottom style="thin">
         <color rgb="00C0392B"/>
       </bottom>
     </border>
@@ -522,7 +537,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="94">
+  <cellXfs count="93">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -540,235 +555,230 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="15" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="23" fillId="5" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="16" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="14" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="29" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="5" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="30" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="18" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="30" fillId="5" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="19" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="30" fillId="5" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="19" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="13" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="13" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="17" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="17" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="21" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="30" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1133,37 +1143,37 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H119"/>
+  <dimension ref="A1:H129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
     <col width="3" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="52" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ■ 自動車保険　意向確認シート（トークスクリプト）</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="22" customHeight="1">
+          <t xml:space="preserve">  ■ 自動車保険　意向確認シート（トークスクリプト型）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ※ 太字部分はお客様に読み上げてください。黄色セルに入力・選択してください。</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="6" customHeight="1">
+          <t xml:space="preserve">  ※ 太字部分はお客様へ読み上げてください。黄色セルを入力・選択し、選択後は対応する下のグループ ＋ を展開してください。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="5" customHeight="1">
       <c r="A3" s="3" t="n"/>
       <c r="B3" s="3" t="n"/>
       <c r="C3" s="3" t="n"/>
@@ -1176,42 +1186,42 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="3" t="n"/>
       <c r="B4" s="3" t="n"/>
-      <c r="C4" s="3" t="n"/>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>日　付</t>
+        </is>
+      </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>日　付</t>
+          <t>担当者名</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>担当者名</t>
+          <t>お客様名</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>お客様名</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
           <t>支店</t>
         </is>
       </c>
+      <c r="G4" s="3" t="n"/>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>契約形態選択 ↓</t>
+          <t>契約方法</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="3" t="n"/>
       <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
+      <c r="C5" s="6" t="n"/>
       <c r="D5" s="6" t="n"/>
       <c r="E5" s="6" t="n"/>
       <c r="F5" s="6" t="n"/>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="7" t="n"/>
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="3" t="n"/>
     </row>
     <row r="6" ht="5" customHeight="1">
       <c r="A6" s="3" t="n"/>
@@ -1223,57 +1233,61 @@
       <c r="G6" s="3" t="n"/>
       <c r="H6" s="3" t="n"/>
     </row>
-    <row r="7" ht="20" customHeight="1">
+    <row r="7" ht="22" customHeight="1">
       <c r="A7" s="3" t="n"/>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  STEP 1　　契約形態の確認　　（まずこちらをお聞きします）</t>
-        </is>
-      </c>
-      <c r="C7" s="9" t="n"/>
-      <c r="D7" s="9" t="n"/>
-      <c r="E7" s="9" t="n"/>
-      <c r="F7" s="9" t="n"/>
-      <c r="G7" s="9" t="n"/>
-      <c r="H7" s="10" t="n"/>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  STEP 1　　契約方法の確認</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="n"/>
+      <c r="D7" s="8" t="n"/>
+      <c r="E7" s="8" t="n"/>
+      <c r="F7" s="8" t="n"/>
+      <c r="G7" s="8" t="n"/>
+      <c r="H7" s="9" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="3" t="n"/>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="10" t="inlineStr">
         <is>
           <t>📋 スクリプト</t>
         </is>
       </c>
-      <c r="C8" s="12" t="n"/>
-      <c r="D8" s="13" t="inlineStr"/>
-      <c r="E8" s="12" t="n"/>
-      <c r="F8" s="12" t="n"/>
-      <c r="G8" s="12" t="n"/>
-      <c r="H8" s="14" t="n"/>
-    </row>
-    <row r="9" ht="72" customHeight="1">
+      <c r="C8" s="11" t="n"/>
+      <c r="D8" s="12" t="inlineStr"/>
+      <c r="E8" s="11" t="n"/>
+      <c r="F8" s="11" t="n"/>
+      <c r="G8" s="11" t="n"/>
+      <c r="H8" s="13" t="n"/>
+    </row>
+    <row r="9" ht="80" customHeight="1">
       <c r="A9" s="3" t="n"/>
-      <c r="B9" s="15" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>📣 読み上げ</t>
         </is>
       </c>
-      <c r="C9" s="12" t="n"/>
-      <c r="D9" s="16" t="inlineStr">
+      <c r="C9" s="11" t="n"/>
+      <c r="D9" s="15" t="inlineStr">
         <is>
           <t>「当社では●社の自動車保険を扱っています。
-そのうち 給与天引きで団体割引が使えるのは 損保ジャパン・三井住友海上・東京海上 の3社です。
-また 通販型のソニー損保 へのお取り次ぎも可能です。
-クレジットカード払いや口座振替をご希望の場合も、一般契約としてご案内できます。
-どのお支払い方法をご希望ですか？」</t>
-        </is>
-      </c>
-      <c r="E9" s="12" t="n"/>
-      <c r="F9" s="12" t="n"/>
-      <c r="G9" s="12" t="n"/>
-      <c r="H9" s="14" t="n"/>
-    </row>
-    <row r="10" ht="18" customHeight="1">
+そのうち 給与天引き（団体割引）が使えるのは 損保ジャパン・三井住友海上・東京海上 の3社です。
+通販型のソニー損保 へのお取り次ぎも可能で、クレジットカード払いや口座振替の一般契約もご案内できます。
+どのご契約方法をご希望ですか？」</t>
+        </is>
+      </c>
+      <c r="E9" s="11" t="n"/>
+      <c r="F9" s="11" t="n"/>
+      <c r="G9" s="11" t="n"/>
+      <c r="H9" s="16" t="inlineStr">
+        <is>
+          <t>← ここで
+選択</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="20" customHeight="1">
       <c r="A10" s="3" t="n"/>
       <c r="B10" s="17" t="inlineStr">
         <is>
@@ -1287,17 +1301,13 @@
       </c>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>損保ジャパン・三井住友海上・東京海上 から選択  →  STEP 2A へ</t>
-        </is>
-      </c>
-      <c r="E10" s="12" t="n"/>
-      <c r="F10" s="12" t="n"/>
-      <c r="G10" s="12" t="n"/>
-      <c r="H10" s="20" t="inlineStr">
-        <is>
-          <t>← H5で選択</t>
-        </is>
-      </c>
+          <t>→ 下のグループ「①②」を展開</t>
+        </is>
+      </c>
+      <c r="E10" s="11" t="n"/>
+      <c r="F10" s="11" t="n"/>
+      <c r="G10" s="11" t="n"/>
+      <c r="H10" s="20" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="3" t="n"/>
@@ -1313,53 +1323,45 @@
       </c>
       <c r="D11" s="23" t="inlineStr">
         <is>
-          <t>同上3社 または その他会社  →  STEP 2A へ</t>
-        </is>
-      </c>
-      <c r="E11" s="12" t="n"/>
-      <c r="F11" s="12" t="n"/>
-      <c r="G11" s="12" t="n"/>
-      <c r="H11" s="20" t="inlineStr">
-        <is>
-          <t>↑H5で選択</t>
-        </is>
-      </c>
+          <t>→ 下のグループ「①②」を展開</t>
+        </is>
+      </c>
+      <c r="E11" s="11" t="n"/>
+      <c r="F11" s="11" t="n"/>
+      <c r="G11" s="11" t="n"/>
+      <c r="H11" s="24" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="3" t="n"/>
-      <c r="B12" s="24" t="inlineStr">
+      <c r="B12" s="25" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C12" s="25" t="inlineStr">
+      <c r="C12" s="26" t="inlineStr">
         <is>
           <t>通販型（ソニー損保）</t>
         </is>
       </c>
-      <c r="D12" s="26" t="inlineStr">
-        <is>
-          <t>ソニー損保へ取り次ぎ  →  STEP 2B へ</t>
-        </is>
-      </c>
-      <c r="E12" s="12" t="n"/>
-      <c r="F12" s="12" t="n"/>
-      <c r="G12" s="12" t="n"/>
-      <c r="H12" s="20" t="inlineStr">
-        <is>
-          <t>↑H5で選択</t>
-        </is>
-      </c>
+      <c r="D12" s="27" t="inlineStr">
+        <is>
+          <t>→ 下のグループ「③」を展開</t>
+        </is>
+      </c>
+      <c r="E12" s="11" t="n"/>
+      <c r="F12" s="11" t="n"/>
+      <c r="G12" s="11" t="n"/>
+      <c r="H12" s="28" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="3" t="n"/>
-      <c r="B13" s="27" t="n"/>
-      <c r="C13" s="28" t="n"/>
-      <c r="D13" s="28" t="n"/>
-      <c r="E13" s="28" t="n"/>
-      <c r="F13" s="28" t="n"/>
-      <c r="G13" s="28" t="n"/>
-      <c r="H13" s="29" t="n"/>
+      <c r="B13" s="29" t="n"/>
+      <c r="C13" s="30" t="n"/>
+      <c r="D13" s="30" t="n"/>
+      <c r="E13" s="30" t="n"/>
+      <c r="F13" s="30" t="n"/>
+      <c r="G13" s="30" t="n"/>
+      <c r="H13" s="31" t="n"/>
     </row>
     <row r="14" ht="5" customHeight="1">
       <c r="A14" s="3" t="n"/>
@@ -1371,361 +1373,358 @@
       <c r="G14" s="3" t="n"/>
       <c r="H14" s="3" t="n"/>
     </row>
-    <row r="15" ht="14" customHeight="1">
+    <row r="15" ht="20" customHeight="1">
       <c r="A15" s="3" t="n"/>
-      <c r="B15" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ▼ ①② 給与天引き・一般契約 の場合 ─────────────────────── STEP 2A へ</t>
-        </is>
-      </c>
-      <c r="F15" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ▼ ③ 通販型 の場合 ─── STEP 2B へ</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="4" customHeight="1">
+      <c r="B15" s="32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ▼  ①② 給与天引き・一般契約 ─── 下のグループ「＋」で展開</t>
+        </is>
+      </c>
+      <c r="F15" s="33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ▼  ③ 通販型 ─── 下のグループ「＋」で展開</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" hidden="1" outlineLevel="1" ht="22" customHeight="1">
       <c r="A16" s="3" t="n"/>
-      <c r="B16" s="3" t="n"/>
-      <c r="C16" s="3" t="n"/>
-      <c r="D16" s="3" t="n"/>
-      <c r="E16" s="3" t="n"/>
-      <c r="F16" s="3" t="n"/>
-      <c r="G16" s="3" t="n"/>
-      <c r="H16" s="3" t="n"/>
-    </row>
-    <row r="17" ht="20" customHeight="1">
+      <c r="B16" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  STEP 2　　意向確認（重視事項）　　給与天引き・一般契約の方</t>
+        </is>
+      </c>
+      <c r="C16" s="8" t="n"/>
+      <c r="D16" s="8" t="n"/>
+      <c r="E16" s="8" t="n"/>
+      <c r="F16" s="8" t="n"/>
+      <c r="G16" s="8" t="n"/>
+      <c r="H16" s="35" t="n"/>
+    </row>
+    <row r="17" hidden="1" outlineLevel="1" ht="18" customHeight="1">
       <c r="A17" s="3" t="n"/>
-      <c r="B17" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  STEP 2A　　意向確認（重視事項の確認）　　①② 給与天引き・一般契約の方</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="n"/>
-      <c r="D17" s="9" t="n"/>
-      <c r="E17" s="9" t="n"/>
-      <c r="F17" s="33" t="n"/>
-      <c r="G17" s="33" t="n"/>
-      <c r="H17" s="34" t="n"/>
-    </row>
-    <row r="18" ht="18" customHeight="1">
+      <c r="B17" s="36" t="inlineStr">
+        <is>
+          <t>📋 スクリプト</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="n"/>
+      <c r="D17" s="37" t="inlineStr"/>
+      <c r="E17" s="11" t="n"/>
+      <c r="F17" s="11" t="n"/>
+      <c r="G17" s="11" t="n"/>
+      <c r="H17" s="13" t="n"/>
+    </row>
+    <row r="18" hidden="1" outlineLevel="1" ht="60" customHeight="1">
       <c r="A18" s="3" t="n"/>
-      <c r="B18" s="35" t="inlineStr">
-        <is>
-          <t>📋 スクリプト</t>
-        </is>
-      </c>
-      <c r="C18" s="12" t="n"/>
-      <c r="D18" s="36" t="inlineStr"/>
-      <c r="E18" s="12" t="n"/>
-      <c r="F18" s="12" t="n"/>
-      <c r="G18" s="12" t="n"/>
-      <c r="H18" s="14" t="n"/>
-    </row>
-    <row r="19" ht="60" customHeight="1">
+      <c r="B18" s="38" t="inlineStr">
+        <is>
+          <t>📣 読み上げ</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="n"/>
+      <c r="D18" s="39" t="inlineStr">
+        <is>
+          <t>「自動車保険でいちばん大切にしていることを教えていただけますか？
+いくつかお伺いしてもよいでしょうか？当てはまるものに○をつけてください。（複数回答可）」</t>
+        </is>
+      </c>
+      <c r="E18" s="11" t="n"/>
+      <c r="F18" s="11" t="n"/>
+      <c r="G18" s="11" t="n"/>
+      <c r="H18" s="13" t="n"/>
+    </row>
+    <row r="19" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A19" s="3" t="n"/>
-      <c r="B19" s="37" t="inlineStr">
-        <is>
-          <t>📣 読み上げ</t>
-        </is>
-      </c>
-      <c r="C19" s="12" t="n"/>
-      <c r="D19" s="38" t="inlineStr">
-        <is>
-          <t>「自動車保険でいちばん大切にしていることを教えていただけますか？
-いくつかお伺いしてもよいですか？　当てはまるものに○をつけてください。
-（複数回答可）」</t>
-        </is>
-      </c>
-      <c r="E19" s="12" t="n"/>
-      <c r="F19" s="12" t="n"/>
-      <c r="G19" s="12" t="n"/>
-      <c r="H19" s="14" t="n"/>
-    </row>
-    <row r="20" ht="18" customHeight="1">
+      <c r="B19" s="36" t="inlineStr">
+        <is>
+          <t>重視項目</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="n"/>
+      <c r="D19" s="40" t="inlineStr">
+        <is>
+          <t>お客様選択</t>
+        </is>
+      </c>
+      <c r="E19" s="11" t="n"/>
+      <c r="F19" s="40" t="inlineStr">
+        <is>
+          <t>各社の強み（参考）</t>
+        </is>
+      </c>
+      <c r="G19" s="11" t="n"/>
+      <c r="H19" s="13" t="n"/>
+    </row>
+    <row r="20" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A20" s="3" t="n"/>
-      <c r="B20" s="35" t="inlineStr">
-        <is>
-          <t>✏️ 重視項目
-（複数可）</t>
-        </is>
-      </c>
-      <c r="C20" s="12" t="n"/>
-      <c r="D20" s="39" t="inlineStr">
-        <is>
-          <t>お客様の選択</t>
-        </is>
-      </c>
-      <c r="E20" s="12" t="n"/>
-      <c r="F20" s="39" t="inlineStr">
-        <is>
-          <t>各社の強み（参考）</t>
-        </is>
-      </c>
-      <c r="G20" s="12" t="n"/>
-      <c r="H20" s="14" t="n"/>
-    </row>
-    <row r="21" ht="20" customHeight="1">
+      <c r="B20" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ①</t>
+        </is>
+      </c>
+      <c r="C20" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  保険料をできるだけ抑えたい</t>
+        </is>
+      </c>
+      <c r="D20" s="11" t="n"/>
+      <c r="E20" s="11" t="n"/>
+      <c r="F20" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  損保ジャパン（多様なプラン）／三井住友海上（ネット割引あり）</t>
+        </is>
+      </c>
+      <c r="G20" s="11" t="n"/>
+      <c r="H20" s="44" t="n"/>
+    </row>
+    <row r="21" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A21" s="3" t="n"/>
-      <c r="B21" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ①</t>
-        </is>
-      </c>
-      <c r="C21" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  保険料をできるだけ抑えたい</t>
-        </is>
-      </c>
-      <c r="D21" s="12" t="n"/>
-      <c r="E21" s="42" t="n"/>
+      <c r="B21" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ②</t>
+        </is>
+      </c>
+      <c r="C21" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  補償をしっかり充実させたい</t>
+        </is>
+      </c>
+      <c r="D21" s="11" t="n"/>
+      <c r="E21" s="11" t="n"/>
       <c r="F21" s="43" t="inlineStr">
         <is>
-          <t xml:space="preserve">  損保ジャパン（多様なプラン）／三井住友海上（ネット割引）</t>
-        </is>
-      </c>
-      <c r="G21" s="12" t="n"/>
-      <c r="H21" s="14" t="n"/>
-    </row>
-    <row r="22" ht="20" customHeight="1">
+          <t xml:space="preserve">  東京海上（総合型・特約充実）／損保ジャパン（幅広い特約）</t>
+        </is>
+      </c>
+      <c r="G21" s="11" t="n"/>
+      <c r="H21" s="44" t="n"/>
+    </row>
+    <row r="22" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A22" s="3" t="n"/>
-      <c r="B22" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ②</t>
-        </is>
-      </c>
-      <c r="C22" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  万一の補償をしっかり充実させたい</t>
-        </is>
-      </c>
-      <c r="D22" s="12" t="n"/>
-      <c r="E22" s="42" t="n"/>
+      <c r="B22" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ③</t>
+        </is>
+      </c>
+      <c r="C22" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  事故時の対応・サポートを重視したい</t>
+        </is>
+      </c>
+      <c r="D22" s="11" t="n"/>
+      <c r="E22" s="11" t="n"/>
       <c r="F22" s="43" t="inlineStr">
         <is>
-          <t xml:space="preserve">  東京海上（総合型・特約充実）／損保ジャパン（幅広い特約）</t>
-        </is>
-      </c>
-      <c r="G22" s="12" t="n"/>
-      <c r="H22" s="14" t="n"/>
-    </row>
-    <row r="23" ht="20" customHeight="1">
+          <t xml:space="preserve">  三井住友海上（示談交渉◎）／東京海上（専任担当）</t>
+        </is>
+      </c>
+      <c r="G22" s="11" t="n"/>
+      <c r="H22" s="44" t="n"/>
+    </row>
+    <row r="23" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A23" s="3" t="n"/>
-      <c r="B23" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ③</t>
-        </is>
-      </c>
-      <c r="C23" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  事故時の対応・サポートを重視したい</t>
-        </is>
-      </c>
-      <c r="D23" s="12" t="n"/>
-      <c r="E23" s="42" t="n"/>
+      <c r="B23" s="41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ④</t>
+        </is>
+      </c>
+      <c r="C23" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  手続きが簡単・わかりやすいものがいい</t>
+        </is>
+      </c>
+      <c r="D23" s="11" t="n"/>
+      <c r="E23" s="11" t="n"/>
       <c r="F23" s="43" t="inlineStr">
         <is>
-          <t xml:space="preserve">  三井住友海上（示談交渉サービス）／東京海上（専任担当）</t>
-        </is>
-      </c>
-      <c r="G23" s="12" t="n"/>
-      <c r="H23" s="14" t="n"/>
-    </row>
-    <row r="24" ht="20" customHeight="1">
+          <t xml:space="preserve">  三井住友海上（シンプル設計・見積り速い）</t>
+        </is>
+      </c>
+      <c r="G23" s="11" t="n"/>
+      <c r="H23" s="44" t="n"/>
+    </row>
+    <row r="24" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A24" s="3" t="n"/>
-      <c r="B24" s="40" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ④</t>
-        </is>
-      </c>
-      <c r="C24" s="41" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  手続きが簡単・わかりやすいものがいい</t>
-        </is>
-      </c>
-      <c r="D24" s="12" t="n"/>
-      <c r="E24" s="42" t="n"/>
-      <c r="F24" s="43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  三井住友海上（シンプル設計・見積り◎）</t>
-        </is>
-      </c>
-      <c r="G24" s="12" t="n"/>
-      <c r="H24" s="14" t="n"/>
-    </row>
-    <row r="25" ht="20" customHeight="1">
+      <c r="B24" s="45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ⑤</t>
+        </is>
+      </c>
+      <c r="C24" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  担当者に相談しながら決めたい</t>
+        </is>
+      </c>
+      <c r="D24" s="47" t="n"/>
+      <c r="E24" s="47" t="n"/>
+      <c r="F24" s="48" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  3社すべて対応可。担当者によるサポートが手厚い</t>
+        </is>
+      </c>
+      <c r="G24" s="47" t="n"/>
+      <c r="H24" s="49" t="n"/>
+    </row>
+    <row r="25" hidden="1" outlineLevel="1" ht="18" customHeight="1">
       <c r="A25" s="3" t="n"/>
-      <c r="B25" s="44" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ⑤</t>
-        </is>
-      </c>
-      <c r="C25" s="45" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  担当者に相談しながら決めたい</t>
-        </is>
-      </c>
-      <c r="D25" s="46" t="n"/>
-      <c r="E25" s="47" t="n"/>
-      <c r="F25" s="48" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  対面での丁寧なサポートが可能な3社すべて</t>
-        </is>
-      </c>
-      <c r="G25" s="46" t="n"/>
-      <c r="H25" s="49" t="n"/>
-    </row>
-    <row r="26" ht="20" customHeight="1">
+      <c r="B25" s="3" t="n"/>
+      <c r="C25" s="3" t="n"/>
+      <c r="D25" s="3" t="n"/>
+      <c r="E25" s="3" t="n"/>
+      <c r="F25" s="3" t="n"/>
+      <c r="G25" s="3" t="n"/>
+      <c r="H25" s="3" t="n"/>
+    </row>
+    <row r="26" hidden="1" outlineLevel="1" ht="22" customHeight="1">
       <c r="A26" s="3" t="n"/>
-      <c r="B26" s="3" t="n"/>
-      <c r="C26" s="3" t="n"/>
-      <c r="D26" s="3" t="n"/>
-      <c r="E26" s="3" t="n"/>
-      <c r="F26" s="3" t="n"/>
-      <c r="G26" s="3" t="n"/>
-      <c r="H26" s="3" t="n"/>
-    </row>
-    <row r="27" ht="5" customHeight="1">
+      <c r="B26" s="50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  STEP 2-2　　3社ご提案（意向確認結果をふまえて）</t>
+        </is>
+      </c>
+      <c r="C26" s="8" t="n"/>
+      <c r="D26" s="8" t="n"/>
+      <c r="E26" s="8" t="n"/>
+      <c r="F26" s="8" t="n"/>
+      <c r="G26" s="8" t="n"/>
+      <c r="H26" s="35" t="n"/>
+    </row>
+    <row r="27" hidden="1" outlineLevel="1" ht="18" customHeight="1">
       <c r="A27" s="3" t="n"/>
-      <c r="B27" s="3" t="n"/>
-      <c r="C27" s="3" t="n"/>
-      <c r="D27" s="3" t="n"/>
-      <c r="E27" s="3" t="n"/>
-      <c r="F27" s="3" t="n"/>
-      <c r="G27" s="3" t="n"/>
-      <c r="H27" s="3" t="n"/>
-    </row>
-    <row r="28" ht="20" customHeight="1">
+      <c r="B27" s="36" t="inlineStr">
+        <is>
+          <t>📣 読み上げ
++ ポイント</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="n"/>
+      <c r="D27" s="51" t="inlineStr">
+        <is>
+          <t>「ありがとうございます。いただいたご希望をもとに、損保ジャパン・三井住友海上・東京海上 の3社でお見積りをご用意します。
+─── 募集人ポイント ────────────────────────────────────────────────────────────
+三井住友海上はシンプル設計で見積り・手続きが速く、担当者の手間が少ないです。
+お客様には保険料もご提示しやすい選択肢です。必ず3社セットでお見せしましょう。
+────────────────────────────────────────────────────────────────────────────」</t>
+        </is>
+      </c>
+      <c r="E27" s="11" t="n"/>
+      <c r="F27" s="11" t="n"/>
+      <c r="G27" s="11" t="n"/>
+      <c r="H27" s="13" t="n"/>
+    </row>
+    <row r="28" hidden="1" outlineLevel="1" ht="60" customHeight="1">
       <c r="A28" s="3" t="n"/>
-      <c r="B28" s="50" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  STEP 2A-2　　3社ご提案（意向確認の結果をふまえて）</t>
-        </is>
-      </c>
-      <c r="C28" s="9" t="n"/>
-      <c r="D28" s="9" t="n"/>
-      <c r="E28" s="9" t="n"/>
-      <c r="F28" s="9" t="n"/>
-      <c r="G28" s="9" t="n"/>
-      <c r="H28" s="10" t="n"/>
-    </row>
-    <row r="29" ht="68" customHeight="1">
+      <c r="B28" s="52" t="inlineStr">
+        <is>
+          <t>会　社</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="n"/>
+      <c r="D28" s="53" t="inlineStr">
+        <is>
+          <t>主な強み・特徴</t>
+        </is>
+      </c>
+      <c r="E28" s="11" t="n"/>
+      <c r="F28" s="53" t="inlineStr">
+        <is>
+          <t>MSI提案の一言</t>
+        </is>
+      </c>
+      <c r="G28" s="11" t="n"/>
+      <c r="H28" s="54" t="inlineStr">
+        <is>
+          <t>提案</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" hidden="1" outlineLevel="1" ht="18" customHeight="1">
       <c r="A29" s="3" t="n"/>
-      <c r="B29" s="35" t="inlineStr">
-        <is>
-          <t>📣 読み上げ
-+ポイント</t>
-        </is>
-      </c>
-      <c r="C29" s="12" t="n"/>
-      <c r="D29" s="51" t="inlineStr">
-        <is>
-          <t>「ありがとうございます。いただいたご希望をもとに、損保ジャパン・三井住友海上・東京海上
-の3社でお見積りをご用意します。
-─── ここがポイント ───────────────────────────────────────────────────
-三井住友海上は見積り・手続きがシンプルで、担当者の手間も少ないです。
-ご予算重視のお客様にもお伝えしやすい選択肢です。ぜひ一緒に比べてみましょう。
-────────────────────────────────────────────────────────────────」</t>
-        </is>
-      </c>
-      <c r="E29" s="12" t="n"/>
-      <c r="F29" s="12" t="n"/>
-      <c r="G29" s="12" t="n"/>
-      <c r="H29" s="14" t="n"/>
-    </row>
-    <row r="30" ht="20" customHeight="1">
+      <c r="B29" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  損保ジャパン</t>
+        </is>
+      </c>
+      <c r="C29" s="11" t="n"/>
+      <c r="D29" s="27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  取引歴が長く慣れている。多彩なプラン・特約</t>
+        </is>
+      </c>
+      <c r="E29" s="11" t="n"/>
+      <c r="F29" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  慣れ親しんだ会社。実績・信頼で推せます</t>
+        </is>
+      </c>
+      <c r="G29" s="11" t="n"/>
+      <c r="H29" s="57" t="n"/>
+    </row>
+    <row r="30" hidden="1" outlineLevel="1" ht="18" customHeight="1">
       <c r="A30" s="3" t="n"/>
-      <c r="B30" s="52" t="inlineStr">
-        <is>
-          <t>会　社</t>
-        </is>
-      </c>
-      <c r="C30" s="12" t="n"/>
-      <c r="D30" s="53" t="inlineStr">
-        <is>
-          <t>主な強み・特徴</t>
-        </is>
-      </c>
-      <c r="E30" s="12" t="n"/>
-      <c r="F30" s="53" t="inlineStr">
-        <is>
-          <t>MSI提案時の一言</t>
-        </is>
-      </c>
-      <c r="G30" s="12" t="n"/>
-      <c r="H30" s="54" t="inlineStr">
-        <is>
-          <t>提案する</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="18" customHeight="1">
+      <c r="B30" s="58" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  三井住友海上</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="n"/>
+      <c r="D30" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  シンプル設計・見積り速い・ネット割引あり</t>
+        </is>
+      </c>
+      <c r="E30" s="11" t="n"/>
+      <c r="F30" s="56" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  手続きが楽で保険料も競争力あり。比較必須</t>
+        </is>
+      </c>
+      <c r="G30" s="11" t="n"/>
+      <c r="H30" s="59" t="n"/>
+    </row>
+    <row r="31" hidden="1" outlineLevel="1" ht="18" customHeight="1">
       <c r="A31" s="3" t="n"/>
-      <c r="B31" s="55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  損保ジャパン</t>
-        </is>
-      </c>
-      <c r="C31" s="12" t="n"/>
-      <c r="D31" s="26" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  取引歴が長く慣れている。多彩なプラン・特約</t>
-        </is>
-      </c>
-      <c r="E31" s="12" t="n"/>
+      <c r="B31" s="60" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  東京海上日動</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="n"/>
+      <c r="D31" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  業界最大手。補償・サービスの充実度が高い</t>
+        </is>
+      </c>
+      <c r="E31" s="11" t="n"/>
       <c r="F31" s="56" t="inlineStr">
         <is>
-          <t xml:space="preserve">  お客様のご状況を最もよく把握している1社</t>
-        </is>
-      </c>
-      <c r="G31" s="12" t="n"/>
-      <c r="H31" s="57" t="n"/>
-    </row>
-    <row r="32" ht="18" customHeight="1">
+          <t xml:space="preserve">  手厚い補償を重視するお客様に有効</t>
+        </is>
+      </c>
+      <c r="G31" s="11" t="n"/>
+      <c r="H31" s="61" t="n"/>
+    </row>
+    <row r="32" hidden="1" outlineLevel="1" ht="18" customHeight="1">
       <c r="A32" s="3" t="n"/>
-      <c r="B32" s="58" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  三井住友海上</t>
-        </is>
-      </c>
-      <c r="C32" s="12" t="n"/>
-      <c r="D32" s="19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  シンプル設計・見積りが速い・ネット割引あり</t>
-        </is>
-      </c>
-      <c r="E32" s="12" t="n"/>
-      <c r="F32" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  手続きが楽で保険料も競争力あり。ぜひ比較を</t>
-        </is>
-      </c>
-      <c r="G32" s="12" t="n"/>
-      <c r="H32" s="59" t="n"/>
-    </row>
-    <row r="33" ht="18" customHeight="1">
+      <c r="B32" s="62" t="n"/>
+      <c r="C32" s="63" t="n"/>
+      <c r="D32" s="63" t="n"/>
+      <c r="E32" s="63" t="n"/>
+      <c r="F32" s="63" t="n"/>
+      <c r="G32" s="63" t="n"/>
+      <c r="H32" s="64" t="n"/>
+    </row>
+    <row r="33" hidden="1" outlineLevel="1" ht="18" customHeight="1">
       <c r="A33" s="3" t="n"/>
-      <c r="B33" s="60" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  東京海上日動</t>
-        </is>
-      </c>
-      <c r="C33" s="46" t="n"/>
-      <c r="D33" s="61" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  業界最大手。補償・サービスの充実度が高い</t>
-        </is>
-      </c>
-      <c r="E33" s="46" t="n"/>
-      <c r="F33" s="62" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  手厚い補償を求めるお客様に刺さります</t>
-        </is>
-      </c>
-      <c r="G33" s="46" t="n"/>
-      <c r="H33" s="63" t="n"/>
-    </row>
-    <row r="34" ht="5" customHeight="1">
+      <c r="B33" s="29" t="n"/>
+      <c r="C33" s="30" t="n"/>
+      <c r="D33" s="30" t="n"/>
+      <c r="E33" s="30" t="n"/>
+      <c r="F33" s="30" t="n"/>
+      <c r="G33" s="30" t="n"/>
+      <c r="H33" s="31" t="n"/>
+    </row>
+    <row r="34" hidden="1" outlineLevel="1" ht="5" customHeight="1">
       <c r="A34" s="3" t="n"/>
       <c r="B34" s="3" t="n"/>
       <c r="C34" s="3" t="n"/>
@@ -1735,128 +1734,123 @@
       <c r="G34" s="3" t="n"/>
       <c r="H34" s="3" t="n"/>
     </row>
-    <row r="35" ht="20" customHeight="1">
+    <row r="35" ht="5" customHeight="1">
       <c r="A35" s="3" t="n"/>
-      <c r="B35" s="64" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  STEP 2B　　ソニー損保ご案内　　③ 通販型をご希望の方</t>
-        </is>
-      </c>
-      <c r="C35" s="9" t="n"/>
-      <c r="D35" s="9" t="n"/>
-      <c r="E35" s="9" t="n"/>
-      <c r="F35" s="9" t="n"/>
-      <c r="G35" s="9" t="n"/>
-      <c r="H35" s="10" t="n"/>
-    </row>
-    <row r="36" ht="18" customHeight="1">
+      <c r="B35" s="3" t="n"/>
+      <c r="C35" s="3" t="n"/>
+      <c r="D35" s="3" t="n"/>
+      <c r="E35" s="3" t="n"/>
+      <c r="F35" s="3" t="n"/>
+      <c r="G35" s="3" t="n"/>
+      <c r="H35" s="3" t="n"/>
+    </row>
+    <row r="36" hidden="1" outlineLevel="1" ht="22" customHeight="1">
       <c r="A36" s="3" t="n"/>
       <c r="B36" s="65" t="inlineStr">
         <is>
+          <t xml:space="preserve">  STEP 2　　ソニー損保ご案内　　通販型をご希望の方</t>
+        </is>
+      </c>
+      <c r="C36" s="8" t="n"/>
+      <c r="D36" s="8" t="n"/>
+      <c r="E36" s="8" t="n"/>
+      <c r="F36" s="8" t="n"/>
+      <c r="G36" s="8" t="n"/>
+      <c r="H36" s="35" t="n"/>
+    </row>
+    <row r="37" hidden="1" outlineLevel="1" ht="18" customHeight="1">
+      <c r="A37" s="3" t="n"/>
+      <c r="B37" s="66" t="inlineStr">
+        <is>
           <t>📋 スクリプト</t>
         </is>
       </c>
-      <c r="C36" s="12" t="n"/>
-      <c r="D36" s="66" t="inlineStr"/>
-      <c r="E36" s="12" t="n"/>
-      <c r="F36" s="12" t="n"/>
-      <c r="G36" s="12" t="n"/>
-      <c r="H36" s="14" t="n"/>
-    </row>
-    <row r="37" ht="65" customHeight="1">
-      <c r="A37" s="3" t="n"/>
-      <c r="B37" s="67" t="inlineStr">
+      <c r="C37" s="11" t="n"/>
+      <c r="D37" s="67" t="inlineStr"/>
+      <c r="E37" s="11" t="n"/>
+      <c r="F37" s="11" t="n"/>
+      <c r="G37" s="11" t="n"/>
+      <c r="H37" s="13" t="n"/>
+    </row>
+    <row r="38" hidden="1" outlineLevel="1" ht="65" customHeight="1">
+      <c r="A38" s="3" t="n"/>
+      <c r="B38" s="68" t="inlineStr">
         <is>
           <t>📣 読み上げ①</t>
         </is>
       </c>
-      <c r="C37" s="12" t="n"/>
-      <c r="D37" s="68" t="inlineStr">
+      <c r="C38" s="11" t="n"/>
+      <c r="D38" s="69" t="inlineStr">
         <is>
           <t>「それではソニー損保をご案内しますので、お客様のご状況を確認させてください。
-ソニー損保はインターネットで直接ご契約いただく通販型です。
-お手続きはお客様ご自身にインターネットでしていただく形となりますが、よろしいでしょうか？」</t>
-        </is>
-      </c>
-      <c r="E37" s="12" t="n"/>
-      <c r="F37" s="12" t="n"/>
-      <c r="G37" s="12" t="n"/>
-      <c r="H37" s="14" t="n"/>
-    </row>
-    <row r="38" ht="65" customHeight="1">
-      <c r="A38" s="3" t="n"/>
-      <c r="B38" s="67" t="inlineStr">
+ソニー損保はインターネットでお客様ご自身に直接ご契約いただく通販型です。手続きはお客様側のご対応となりますが、よろしいでしょうか？」</t>
+        </is>
+      </c>
+      <c r="E38" s="11" t="n"/>
+      <c r="F38" s="11" t="n"/>
+      <c r="G38" s="11" t="n"/>
+      <c r="H38" s="13" t="n"/>
+    </row>
+    <row r="39" hidden="1" outlineLevel="1" ht="65" customHeight="1">
+      <c r="A39" s="3" t="n"/>
+      <c r="B39" s="68" t="inlineStr">
         <is>
           <t>📣 読み上げ②
-（留意点の説明）</t>
-        </is>
-      </c>
-      <c r="C38" s="12" t="n"/>
-      <c r="D38" s="68" t="inlineStr">
-        <is>
-          <t>「保険料の面ではメリットが大きい場合もありますが、事故時のサポートはコールセンター対応が
-基本となります。当社担当者が直接サポートすることは難しくなる点もご了承ください。
-それでもよろしければ、ソニー損保のサイトをご一緒に確認しながら手続きをご案内します。」</t>
-        </is>
-      </c>
-      <c r="E38" s="12" t="n"/>
-      <c r="F38" s="12" t="n"/>
-      <c r="G38" s="12" t="n"/>
-      <c r="H38" s="14" t="n"/>
-    </row>
-    <row r="39" ht="65" customHeight="1">
-      <c r="A39" s="3" t="n"/>
-      <c r="B39" s="69" t="inlineStr">
+（留意点）</t>
+        </is>
+      </c>
+      <c r="C39" s="11" t="n"/>
+      <c r="D39" s="69" t="inlineStr">
+        <is>
+          <t>「保険料面ではメリットが出る場合もありますが、事故時のサポートはコールセンター対応が基本となります。
+当社担当者が直接サポートすることは難しくなりますが、それでもよろしいでしょうか？
+ご希望でしたら、ソニー損保のサイトをご一緒に確認しながら手続きをご案内します。」</t>
+        </is>
+      </c>
+      <c r="E39" s="11" t="n"/>
+      <c r="F39" s="11" t="n"/>
+      <c r="G39" s="11" t="n"/>
+      <c r="H39" s="13" t="n"/>
+    </row>
+    <row r="40" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A40" s="3" t="n"/>
+      <c r="B40" s="66" t="inlineStr">
         <is>
           <t>✏️ お客様の意向</t>
         </is>
       </c>
-      <c r="C39" s="46" t="n"/>
-      <c r="D39" s="70" t="inlineStr">
+      <c r="C40" s="11" t="n"/>
+      <c r="D40" s="70" t="inlineStr">
         <is>
           <t>ソニー損保で進める</t>
         </is>
       </c>
-      <c r="E39" s="46" t="n"/>
-      <c r="F39" s="71" t="n"/>
-      <c r="G39" s="72" t="inlineStr">
-        <is>
-          <t>← 選択してください</t>
-        </is>
-      </c>
-      <c r="H39" s="49" t="n"/>
-    </row>
-    <row r="40" ht="20" customHeight="1">
-      <c r="A40" s="3" t="n"/>
-      <c r="B40" s="3" t="n"/>
-      <c r="C40" s="3" t="n"/>
-      <c r="D40" s="3" t="n"/>
-      <c r="E40" s="3" t="n"/>
-      <c r="F40" s="3" t="n"/>
-      <c r="G40" s="3" t="n"/>
-      <c r="H40" s="3" t="n"/>
-    </row>
-    <row r="41" ht="18" customHeight="1">
+      <c r="E40" s="11" t="n"/>
+      <c r="F40" s="11" t="n"/>
+      <c r="G40" s="11" t="n"/>
+      <c r="H40" s="57" t="n"/>
+    </row>
+    <row r="41" hidden="1" outlineLevel="1" ht="18" customHeight="1">
       <c r="A41" s="3" t="n"/>
-      <c r="B41" s="3" t="n"/>
-      <c r="C41" s="3" t="n"/>
-      <c r="D41" s="3" t="n"/>
-      <c r="E41" s="3" t="n"/>
-      <c r="F41" s="3" t="n"/>
-      <c r="G41" s="3" t="n"/>
-      <c r="H41" s="3" t="n"/>
-    </row>
-    <row r="42" ht="18" customHeight="1">
+      <c r="B41" s="71" t="inlineStr"/>
+      <c r="C41" s="11" t="n"/>
+      <c r="D41" s="63" t="n"/>
+      <c r="E41" s="63" t="n"/>
+      <c r="F41" s="63" t="n"/>
+      <c r="G41" s="63" t="n"/>
+      <c r="H41" s="64" t="n"/>
+    </row>
+    <row r="42" hidden="1" outlineLevel="1" ht="18" customHeight="1">
       <c r="A42" s="3" t="n"/>
-      <c r="B42" s="3" t="n"/>
-      <c r="C42" s="3" t="n"/>
-      <c r="D42" s="3" t="n"/>
-      <c r="E42" s="3" t="n"/>
-      <c r="F42" s="3" t="n"/>
-      <c r="G42" s="3" t="n"/>
-      <c r="H42" s="3" t="n"/>
-    </row>
-    <row r="43" ht="5" customHeight="1">
+      <c r="B42" s="72" t="inlineStr"/>
+      <c r="C42" s="47" t="n"/>
+      <c r="D42" s="30" t="n"/>
+      <c r="E42" s="30" t="n"/>
+      <c r="F42" s="30" t="n"/>
+      <c r="G42" s="30" t="n"/>
+      <c r="H42" s="31" t="n"/>
+    </row>
+    <row r="43" hidden="1" outlineLevel="1" ht="5" customHeight="1">
       <c r="A43" s="3" t="n"/>
       <c r="B43" s="3" t="n"/>
       <c r="C43" s="3" t="n"/>
@@ -1866,83 +1860,85 @@
       <c r="G43" s="3" t="n"/>
       <c r="H43" s="3" t="n"/>
     </row>
-    <row r="44" ht="20" customHeight="1">
+    <row r="44" hidden="1" outlineLevel="1" ht="16" customHeight="1">
       <c r="A44" s="3" t="n"/>
-      <c r="B44" s="73" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  📝 面談メモ・次回アクション</t>
-        </is>
-      </c>
-      <c r="C44" s="9" t="n"/>
-      <c r="D44" s="9" t="n"/>
-      <c r="E44" s="9" t="n"/>
-      <c r="F44" s="9" t="n"/>
-      <c r="G44" s="9" t="n"/>
-      <c r="H44" s="10" t="n"/>
-    </row>
-    <row r="45" ht="80" customHeight="1">
+      <c r="B44" s="3" t="n"/>
+      <c r="C44" s="3" t="n"/>
+      <c r="D44" s="3" t="n"/>
+      <c r="E44" s="3" t="n"/>
+      <c r="F44" s="3" t="n"/>
+      <c r="G44" s="3" t="n"/>
+      <c r="H44" s="3" t="n"/>
+    </row>
+    <row r="45" ht="16" customHeight="1">
       <c r="A45" s="3" t="n"/>
-      <c r="B45" s="74" t="inlineStr"/>
-      <c r="C45" s="12" t="n"/>
-      <c r="D45" s="12" t="n"/>
-      <c r="E45" s="12" t="n"/>
-      <c r="F45" s="12" t="n"/>
-      <c r="G45" s="12" t="n"/>
-      <c r="H45" s="14" t="n"/>
-    </row>
-    <row r="46" ht="5" customHeight="1">
+      <c r="B45" s="3" t="n"/>
+      <c r="C45" s="3" t="n"/>
+      <c r="D45" s="3" t="n"/>
+      <c r="E45" s="3" t="n"/>
+      <c r="F45" s="3" t="n"/>
+      <c r="G45" s="3" t="n"/>
+      <c r="H45" s="3" t="n"/>
+    </row>
+    <row r="46" ht="20" customHeight="1">
       <c r="A46" s="3" t="n"/>
-      <c r="B46" s="75" t="n"/>
-      <c r="C46" s="76" t="n"/>
-      <c r="D46" s="76" t="n"/>
-      <c r="E46" s="76" t="n"/>
-      <c r="F46" s="76" t="n"/>
-      <c r="G46" s="76" t="n"/>
-      <c r="H46" s="77" t="n"/>
-    </row>
-    <row r="47" ht="20" customHeight="1">
+      <c r="B46" s="73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  📝 面談メモ・お客様の声</t>
+        </is>
+      </c>
+      <c r="C46" s="8" t="n"/>
+      <c r="D46" s="8" t="n"/>
+      <c r="E46" s="8" t="n"/>
+      <c r="F46" s="8" t="n"/>
+      <c r="G46" s="8" t="n"/>
+      <c r="H46" s="35" t="n"/>
+    </row>
+    <row r="47" ht="80" customHeight="1">
       <c r="A47" s="3" t="n"/>
-      <c r="B47" s="78" t="inlineStr">
+      <c r="B47" s="74" t="n"/>
+      <c r="C47" s="11" t="n"/>
+      <c r="D47" s="11" t="n"/>
+      <c r="E47" s="11" t="n"/>
+      <c r="F47" s="11" t="n"/>
+      <c r="G47" s="11" t="n"/>
+      <c r="H47" s="13" t="n"/>
+    </row>
+    <row r="48" ht="5" customHeight="1">
+      <c r="A48" s="3" t="n"/>
+      <c r="B48" s="62" t="n"/>
+      <c r="C48" s="63" t="n"/>
+      <c r="D48" s="63" t="n"/>
+      <c r="E48" s="63" t="n"/>
+      <c r="F48" s="63" t="n"/>
+      <c r="G48" s="63" t="n"/>
+      <c r="H48" s="64" t="n"/>
+    </row>
+    <row r="49" ht="20" customHeight="1">
+      <c r="A49" s="3" t="n"/>
+      <c r="B49" s="75" t="inlineStr">
         <is>
           <t xml:space="preserve">  📌 次回アクション</t>
         </is>
       </c>
-      <c r="C47" s="12" t="n"/>
-      <c r="D47" s="12" t="n"/>
-      <c r="E47" s="12" t="n"/>
-      <c r="F47" s="12" t="n"/>
-      <c r="G47" s="12" t="n"/>
-      <c r="H47" s="14" t="n"/>
-    </row>
-    <row r="48" ht="30" customHeight="1">
-      <c r="A48" s="3" t="n"/>
-      <c r="B48" s="79" t="inlineStr"/>
-      <c r="C48" s="46" t="n"/>
-      <c r="D48" s="46" t="n"/>
-      <c r="E48" s="46" t="n"/>
-      <c r="F48" s="46" t="n"/>
-      <c r="G48" s="46" t="n"/>
-      <c r="H48" s="49" t="n"/>
-    </row>
-    <row r="49" ht="5" customHeight="1">
-      <c r="A49" s="3" t="n"/>
-      <c r="B49" s="3" t="n"/>
-      <c r="C49" s="3" t="n"/>
-      <c r="D49" s="3" t="n"/>
-      <c r="E49" s="3" t="n"/>
-      <c r="F49" s="3" t="n"/>
-      <c r="G49" s="3" t="n"/>
-      <c r="H49" s="3" t="n"/>
-    </row>
-    <row r="50" ht="16" customHeight="1">
+      <c r="C49" s="11" t="n"/>
+      <c r="D49" s="11" t="n"/>
+      <c r="E49" s="11" t="n"/>
+      <c r="F49" s="11" t="n"/>
+      <c r="G49" s="11" t="n"/>
+      <c r="H49" s="13" t="n"/>
+    </row>
+    <row r="50" ht="30" customHeight="1">
       <c r="A50" s="3" t="n"/>
-      <c r="B50" s="80" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ＊本シートは比較推奨規制対応の意向確認記録としてご活用ください。　面談後にファイルを保存・アーカイブしてください。</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="18" customHeight="1">
+      <c r="B50" s="76" t="n"/>
+      <c r="C50" s="47" t="n"/>
+      <c r="D50" s="47" t="n"/>
+      <c r="E50" s="47" t="n"/>
+      <c r="F50" s="47" t="n"/>
+      <c r="G50" s="47" t="n"/>
+      <c r="H50" s="77" t="n"/>
+    </row>
+    <row r="51" ht="5" customHeight="1">
       <c r="A51" s="3" t="n"/>
       <c r="B51" s="3" t="n"/>
       <c r="C51" s="3" t="n"/>
@@ -1954,13 +1950,11 @@
     </row>
     <row r="52" ht="16" customHeight="1">
       <c r="A52" s="3" t="n"/>
-      <c r="B52" s="3" t="n"/>
-      <c r="C52" s="3" t="n"/>
-      <c r="D52" s="3" t="n"/>
-      <c r="E52" s="3" t="n"/>
-      <c r="F52" s="3" t="n"/>
-      <c r="G52" s="3" t="n"/>
-      <c r="H52" s="3" t="n"/>
+      <c r="B52" s="78" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ＊本シートは比較推奨規制対応の意向確認記録として活用してください。面談後は保存・アーカイブをお願いします。</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="16" customHeight="1">
       <c r="A53" s="3" t="n"/>
@@ -2632,81 +2626,182 @@
       <c r="G119" s="3" t="n"/>
       <c r="H119" s="3" t="n"/>
     </row>
+    <row r="120" ht="16" customHeight="1">
+      <c r="A120" s="3" t="n"/>
+      <c r="B120" s="3" t="n"/>
+      <c r="C120" s="3" t="n"/>
+      <c r="D120" s="3" t="n"/>
+      <c r="E120" s="3" t="n"/>
+      <c r="F120" s="3" t="n"/>
+      <c r="G120" s="3" t="n"/>
+      <c r="H120" s="3" t="n"/>
+    </row>
+    <row r="121" ht="16" customHeight="1">
+      <c r="A121" s="3" t="n"/>
+      <c r="B121" s="3" t="n"/>
+      <c r="C121" s="3" t="n"/>
+      <c r="D121" s="3" t="n"/>
+      <c r="E121" s="3" t="n"/>
+      <c r="F121" s="3" t="n"/>
+      <c r="G121" s="3" t="n"/>
+      <c r="H121" s="3" t="n"/>
+    </row>
+    <row r="122" ht="16" customHeight="1">
+      <c r="A122" s="3" t="n"/>
+      <c r="B122" s="3" t="n"/>
+      <c r="C122" s="3" t="n"/>
+      <c r="D122" s="3" t="n"/>
+      <c r="E122" s="3" t="n"/>
+      <c r="F122" s="3" t="n"/>
+      <c r="G122" s="3" t="n"/>
+      <c r="H122" s="3" t="n"/>
+    </row>
+    <row r="123" ht="16" customHeight="1">
+      <c r="A123" s="3" t="n"/>
+      <c r="B123" s="3" t="n"/>
+      <c r="C123" s="3" t="n"/>
+      <c r="D123" s="3" t="n"/>
+      <c r="E123" s="3" t="n"/>
+      <c r="F123" s="3" t="n"/>
+      <c r="G123" s="3" t="n"/>
+      <c r="H123" s="3" t="n"/>
+    </row>
+    <row r="124" ht="16" customHeight="1">
+      <c r="A124" s="3" t="n"/>
+      <c r="B124" s="3" t="n"/>
+      <c r="C124" s="3" t="n"/>
+      <c r="D124" s="3" t="n"/>
+      <c r="E124" s="3" t="n"/>
+      <c r="F124" s="3" t="n"/>
+      <c r="G124" s="3" t="n"/>
+      <c r="H124" s="3" t="n"/>
+    </row>
+    <row r="125" ht="16" customHeight="1">
+      <c r="A125" s="3" t="n"/>
+      <c r="B125" s="3" t="n"/>
+      <c r="C125" s="3" t="n"/>
+      <c r="D125" s="3" t="n"/>
+      <c r="E125" s="3" t="n"/>
+      <c r="F125" s="3" t="n"/>
+      <c r="G125" s="3" t="n"/>
+      <c r="H125" s="3" t="n"/>
+    </row>
+    <row r="126" ht="16" customHeight="1">
+      <c r="A126" s="3" t="n"/>
+      <c r="B126" s="3" t="n"/>
+      <c r="C126" s="3" t="n"/>
+      <c r="D126" s="3" t="n"/>
+      <c r="E126" s="3" t="n"/>
+      <c r="F126" s="3" t="n"/>
+      <c r="G126" s="3" t="n"/>
+      <c r="H126" s="3" t="n"/>
+    </row>
+    <row r="127" ht="16" customHeight="1">
+      <c r="A127" s="3" t="n"/>
+      <c r="B127" s="3" t="n"/>
+      <c r="C127" s="3" t="n"/>
+      <c r="D127" s="3" t="n"/>
+      <c r="E127" s="3" t="n"/>
+      <c r="F127" s="3" t="n"/>
+      <c r="G127" s="3" t="n"/>
+      <c r="H127" s="3" t="n"/>
+    </row>
+    <row r="128" ht="16" customHeight="1">
+      <c r="A128" s="3" t="n"/>
+      <c r="B128" s="3" t="n"/>
+      <c r="C128" s="3" t="n"/>
+      <c r="D128" s="3" t="n"/>
+      <c r="E128" s="3" t="n"/>
+      <c r="F128" s="3" t="n"/>
+      <c r="G128" s="3" t="n"/>
+      <c r="H128" s="3" t="n"/>
+    </row>
+    <row r="129" ht="16" customHeight="1">
+      <c r="A129" s="3" t="n"/>
+      <c r="B129" s="3" t="n"/>
+      <c r="C129" s="3" t="n"/>
+      <c r="D129" s="3" t="n"/>
+      <c r="E129" s="3" t="n"/>
+      <c r="F129" s="3" t="n"/>
+      <c r="G129" s="3" t="n"/>
+      <c r="H129" s="3" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="60">
+  <mergeCells count="61">
     <mergeCell ref="F20:H20"/>
-    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="D9:G9"/>
+    <mergeCell ref="C20:E20"/>
     <mergeCell ref="F21:H21"/>
-    <mergeCell ref="C24:D24"/>
+    <mergeCell ref="F29:G29"/>
     <mergeCell ref="D12:G12"/>
-    <mergeCell ref="D19:H19"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="B49:H49"/>
+    <mergeCell ref="C22:E22"/>
     <mergeCell ref="B15:E15"/>
     <mergeCell ref="B31:C31"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="B18:C18"/>
+    <mergeCell ref="C21:E21"/>
+    <mergeCell ref="B27:C27"/>
     <mergeCell ref="D31:E31"/>
-    <mergeCell ref="D36:H36"/>
-    <mergeCell ref="G39:H39"/>
-    <mergeCell ref="B45:H45"/>
     <mergeCell ref="F23:H23"/>
+    <mergeCell ref="B36:H36"/>
     <mergeCell ref="B39:C39"/>
     <mergeCell ref="B50:H50"/>
     <mergeCell ref="F30:G30"/>
     <mergeCell ref="F22:H22"/>
-    <mergeCell ref="B35:H35"/>
-    <mergeCell ref="C25:D25"/>
-    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="B26:H26"/>
+    <mergeCell ref="C23:E23"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="D27:H27"/>
     <mergeCell ref="B47:H47"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="B7:H7"/>
-    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="B16:H16"/>
+    <mergeCell ref="B17:C17"/>
     <mergeCell ref="D10:G10"/>
     <mergeCell ref="B8:C8"/>
+    <mergeCell ref="D17:H17"/>
+    <mergeCell ref="B46:H46"/>
+    <mergeCell ref="D40:G40"/>
     <mergeCell ref="B38:C38"/>
-    <mergeCell ref="C21:D21"/>
     <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B52:H52"/>
     <mergeCell ref="B19:C19"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B28:C28"/>
     <mergeCell ref="F31:G31"/>
+    <mergeCell ref="D28:E28"/>
     <mergeCell ref="D37:H37"/>
-    <mergeCell ref="B48:H48"/>
+    <mergeCell ref="F28:G28"/>
     <mergeCell ref="D11:G11"/>
+    <mergeCell ref="B40:C40"/>
     <mergeCell ref="B9:C9"/>
-    <mergeCell ref="C23:D23"/>
     <mergeCell ref="D18:H18"/>
-    <mergeCell ref="D9:H9"/>
-    <mergeCell ref="F25:H25"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="B17:E17"/>
-    <mergeCell ref="B28:H28"/>
+    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="C24:E24"/>
+    <mergeCell ref="B30:C30"/>
     <mergeCell ref="D8:H8"/>
-    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="D39:H39"/>
+    <mergeCell ref="F19:H19"/>
     <mergeCell ref="D30:E30"/>
-    <mergeCell ref="B33:C33"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="B44:H44"/>
-    <mergeCell ref="B20:C20"/>
-    <mergeCell ref="D29:H29"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="D29:E29"/>
     <mergeCell ref="D38:H38"/>
+    <mergeCell ref="B41:C41"/>
     <mergeCell ref="F15:H15"/>
     <mergeCell ref="F24:H24"/>
   </mergeCells>
   <dataValidations count="4">
-    <dataValidation sqref="H5" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="STEP1 選択" prompt="契約方法を選択してください" type="list">
       <formula1>"①給与天引き（団体割引）,②一般契約（クレカ・口振）,③通販型（ソニー損保）"</formula1>
     </dataValidation>
-    <dataValidation sqref="E21 E22 E23 E24 E25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H20 H21 H22 H23 H24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"○,−"</formula1>
     </dataValidation>
-    <dataValidation sqref="H31 H32 H33" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H29 H30 H31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"◎提案する,○提案する,△保留,×見送り"</formula1>
     </dataValidation>
-    <dataValidation sqref="F39" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"はい（取り次ぎ確定）,再検討（給与天引きも比較）,見送り"</formula1>
+    <dataValidation sqref="H40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"はい（取り次ぎ確定）,再検討（3社も比較）,見送り"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2719,16 +2814,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="4" customWidth="1" min="2" max="2"/>
-    <col width="42" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -2741,534 +2836,624 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  面談前後に確認し、すべて「済」になっていることを確認してください。</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="16" customHeight="1">
-      <c r="A3" s="81" t="n"/>
-      <c r="B3" s="81" t="n"/>
-      <c r="C3" s="82" t="inlineStr">
+          <t xml:space="preserve">  面談前後に確認し、すべて「✅ 済」になっていることを確認してください。</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="79" t="n"/>
+      <c r="B3" s="79" t="n"/>
+      <c r="C3" s="80" t="inlineStr">
         <is>
           <t xml:space="preserve">  確認項目</t>
         </is>
       </c>
-      <c r="E3" s="83" t="inlineStr">
+      <c r="E3" s="81" t="inlineStr">
         <is>
           <t>SJ</t>
         </is>
       </c>
-      <c r="F3" s="83" t="inlineStr">
+      <c r="F3" s="81" t="inlineStr">
         <is>
           <t>MSI</t>
         </is>
       </c>
-      <c r="G3" s="83" t="inlineStr">
+      <c r="G3" s="81" t="inlineStr">
         <is>
           <t>TN</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="81" t="n"/>
-      <c r="B4" s="84" t="inlineStr">
+      <c r="A4" s="79" t="n"/>
+      <c r="B4" s="82" t="inlineStr">
         <is>
           <t xml:space="preserve">  【 事前確認 】</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="81" t="n"/>
-      <c r="B5" s="85" t="inlineStr">
+      <c r="A5" s="79" t="n"/>
+      <c r="B5" s="83" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C5" s="86" t="inlineStr">
+      <c r="C5" s="84" t="inlineStr">
         <is>
           <t xml:space="preserve">  お客様の意向（重視事項）を確認した</t>
         </is>
       </c>
-      <c r="E5" s="87" t="n"/>
-      <c r="F5" s="88" t="n"/>
-      <c r="G5" s="88" t="n"/>
+      <c r="E5" s="85" t="n"/>
+      <c r="F5" s="86" t="n"/>
+      <c r="G5" s="86" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="81" t="n"/>
-      <c r="B6" s="85" t="inlineStr">
+      <c r="A6" s="79" t="n"/>
+      <c r="B6" s="83" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C6" s="86" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  複数社（原則3社以上）の見積りを取得した</t>
-        </is>
-      </c>
-      <c r="E6" s="87" t="n"/>
-      <c r="F6" s="88" t="n"/>
-      <c r="G6" s="88" t="n"/>
+      <c r="C6" s="84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  複数社（原則3社）の見積りを取得した</t>
+        </is>
+      </c>
+      <c r="E6" s="85" t="n"/>
+      <c r="F6" s="86" t="n"/>
+      <c r="G6" s="86" t="n"/>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="81" t="n"/>
-      <c r="B7" s="85" t="inlineStr">
+      <c r="A7" s="79" t="n"/>
+      <c r="B7" s="83" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C7" s="86" t="inlineStr">
+      <c r="C7" s="84" t="inlineStr">
         <is>
           <t xml:space="preserve">  各社の保険料・補償内容を比較説明した</t>
         </is>
       </c>
-      <c r="E7" s="87" t="n"/>
-      <c r="F7" s="88" t="n"/>
-      <c r="G7" s="88" t="n"/>
+      <c r="E7" s="85" t="n"/>
+      <c r="F7" s="86" t="n"/>
+      <c r="G7" s="86" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="81" t="n"/>
-      <c r="B8" s="85" t="inlineStr">
+      <c r="A8" s="79" t="n"/>
+      <c r="B8" s="83" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C8" s="86" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  比較に用いた基準・理由を説明できる状態にある</t>
-        </is>
-      </c>
-      <c r="E8" s="87" t="n"/>
-      <c r="F8" s="88" t="n"/>
-      <c r="G8" s="88" t="n"/>
+      <c r="C8" s="84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  比較に用いた基準・理由を説明できる</t>
+        </is>
+      </c>
+      <c r="E8" s="85" t="n"/>
+      <c r="F8" s="86" t="n"/>
+      <c r="G8" s="86" t="n"/>
     </row>
     <row r="9" ht="4" customHeight="1">
-      <c r="A9" s="81" t="n"/>
-      <c r="B9" s="81" t="n"/>
-      <c r="C9" s="81" t="n"/>
-      <c r="D9" s="81" t="n"/>
-      <c r="E9" s="81" t="n"/>
-      <c r="F9" s="81" t="n"/>
-      <c r="G9" s="81" t="n"/>
+      <c r="A9" s="79" t="n"/>
+      <c r="B9" s="79" t="n"/>
+      <c r="C9" s="79" t="n"/>
+      <c r="D9" s="79" t="n"/>
+      <c r="E9" s="79" t="n"/>
+      <c r="F9" s="79" t="n"/>
+      <c r="G9" s="79" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="81" t="n"/>
-      <c r="B10" s="84" t="inlineStr">
+      <c r="A10" s="79" t="n"/>
+      <c r="B10" s="82" t="inlineStr">
         <is>
           <t xml:space="preserve">  【 三井住友海上の提案 】</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="81" t="n"/>
-      <c r="B11" s="89" t="inlineStr">
+      <c r="A11" s="79" t="n"/>
+      <c r="B11" s="87" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C11" s="86" t="inlineStr">
+      <c r="C11" s="84" t="inlineStr">
         <is>
           <t xml:space="preserve">  三井住友海上の見積りを必ず含めた</t>
         </is>
       </c>
-      <c r="E11" s="90" t="n"/>
-      <c r="F11" s="88" t="n"/>
-      <c r="G11" s="88" t="n"/>
+      <c r="E11" s="88" t="n"/>
+      <c r="F11" s="86" t="n"/>
+      <c r="G11" s="86" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="81" t="n"/>
-      <c r="B12" s="89" t="inlineStr">
+      <c r="A12" s="79" t="n"/>
+      <c r="B12" s="87" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C12" s="86" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  損保ジャパンとの比較ポイントをお客様に説明した</t>
-        </is>
-      </c>
-      <c r="E12" s="90" t="n"/>
-      <c r="F12" s="88" t="n"/>
-      <c r="G12" s="88" t="n"/>
+      <c r="C12" s="84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  損保ジャパンとの比較ポイントを説明した</t>
+        </is>
+      </c>
+      <c r="E12" s="88" t="n"/>
+      <c r="F12" s="86" t="n"/>
+      <c r="G12" s="86" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="81" t="n"/>
-      <c r="B13" s="89" t="inlineStr">
+      <c r="A13" s="79" t="n"/>
+      <c r="B13" s="87" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C13" s="86" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  お客様が三井住友海上を選ばない理由を記録した（選ばない場合）</t>
-        </is>
-      </c>
-      <c r="E13" s="90" t="n"/>
-      <c r="F13" s="88" t="n"/>
-      <c r="G13" s="88" t="n"/>
+      <c r="C13" s="84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  MSIを選ばない場合、理由を記録した</t>
+        </is>
+      </c>
+      <c r="E13" s="88" t="n"/>
+      <c r="F13" s="86" t="n"/>
+      <c r="G13" s="86" t="n"/>
     </row>
     <row r="14" ht="4" customHeight="1">
-      <c r="A14" s="81" t="n"/>
-      <c r="B14" s="81" t="n"/>
-      <c r="C14" s="81" t="n"/>
-      <c r="D14" s="81" t="n"/>
-      <c r="E14" s="81" t="n"/>
-      <c r="F14" s="81" t="n"/>
-      <c r="G14" s="81" t="n"/>
+      <c r="A14" s="79" t="n"/>
+      <c r="B14" s="79" t="n"/>
+      <c r="C14" s="79" t="n"/>
+      <c r="D14" s="79" t="n"/>
+      <c r="E14" s="79" t="n"/>
+      <c r="F14" s="79" t="n"/>
+      <c r="G14" s="79" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="81" t="n"/>
-      <c r="B15" s="84" t="inlineStr">
+      <c r="A15" s="79" t="n"/>
+      <c r="B15" s="82" t="inlineStr">
         <is>
           <t xml:space="preserve">  【 推奨根拠の記録 】</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="81" t="n"/>
-      <c r="B16" s="91" t="inlineStr">
+      <c r="A16" s="79" t="n"/>
+      <c r="B16" s="89" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C16" s="86" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  推奨する商品・会社とその理由を記録した</t>
-        </is>
-      </c>
-      <c r="E16" s="92" t="n"/>
-      <c r="F16" s="88" t="n"/>
-      <c r="G16" s="88" t="n"/>
+      <c r="C16" s="84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  推奨する会社・商品とその理由を記録した</t>
+        </is>
+      </c>
+      <c r="E16" s="90" t="n"/>
+      <c r="F16" s="86" t="n"/>
+      <c r="G16" s="86" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="81" t="n"/>
-      <c r="B17" s="91" t="inlineStr">
+      <c r="A17" s="79" t="n"/>
+      <c r="B17" s="89" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C17" s="86" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  お客様が最終的に選んだ商品・会社を記録した</t>
-        </is>
-      </c>
-      <c r="E17" s="92" t="n"/>
-      <c r="F17" s="88" t="n"/>
-      <c r="G17" s="88" t="n"/>
+      <c r="C17" s="84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  お客様が選んだ会社・商品を記録した</t>
+        </is>
+      </c>
+      <c r="E17" s="90" t="n"/>
+      <c r="F17" s="86" t="n"/>
+      <c r="G17" s="86" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="81" t="n"/>
-      <c r="B18" s="91" t="inlineStr">
+      <c r="A18" s="79" t="n"/>
+      <c r="B18" s="89" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C18" s="86" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  意向と選択が異なる場合、その経緯を記録した</t>
-        </is>
-      </c>
-      <c r="E18" s="92" t="n"/>
-      <c r="F18" s="88" t="n"/>
-      <c r="G18" s="88" t="n"/>
+      <c r="C18" s="84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  意向と選択が異なる場合、経緯を記録した</t>
+        </is>
+      </c>
+      <c r="E18" s="90" t="n"/>
+      <c r="F18" s="86" t="n"/>
+      <c r="G18" s="86" t="n"/>
     </row>
     <row r="19" ht="4" customHeight="1">
-      <c r="A19" s="81" t="n"/>
-      <c r="B19" s="81" t="n"/>
-      <c r="C19" s="81" t="n"/>
-      <c r="D19" s="81" t="n"/>
-      <c r="E19" s="81" t="n"/>
-      <c r="F19" s="81" t="n"/>
-      <c r="G19" s="81" t="n"/>
+      <c r="A19" s="79" t="n"/>
+      <c r="B19" s="79" t="n"/>
+      <c r="C19" s="79" t="n"/>
+      <c r="D19" s="79" t="n"/>
+      <c r="E19" s="79" t="n"/>
+      <c r="F19" s="79" t="n"/>
+      <c r="G19" s="79" t="n"/>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="81" t="n"/>
-      <c r="B20" s="84" t="inlineStr">
+      <c r="A20" s="79" t="n"/>
+      <c r="B20" s="82" t="inlineStr">
         <is>
           <t xml:space="preserve">  【 コンプライアンス 】</t>
         </is>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="81" t="n"/>
-      <c r="B21" s="93" t="inlineStr">
+      <c r="A21" s="79" t="n"/>
+      <c r="B21" s="91" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C21" s="86" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  特定の会社を誘導した事実はない</t>
-        </is>
-      </c>
-      <c r="E21" s="7" t="n"/>
-      <c r="F21" s="88" t="n"/>
-      <c r="G21" s="88" t="n"/>
+      <c r="C21" s="84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  特定会社への誘導はない</t>
+        </is>
+      </c>
+      <c r="E21" s="92" t="n"/>
+      <c r="F21" s="86" t="n"/>
+      <c r="G21" s="86" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="81" t="n"/>
-      <c r="B22" s="93" t="inlineStr">
+      <c r="A22" s="79" t="n"/>
+      <c r="B22" s="91" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C22" s="86" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  お客様から意向確認の同意を得た</t>
-        </is>
-      </c>
-      <c r="E22" s="7" t="n"/>
-      <c r="F22" s="88" t="n"/>
-      <c r="G22" s="88" t="n"/>
+      <c r="C22" s="84" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  意向確認の同意を得た</t>
+        </is>
+      </c>
+      <c r="E22" s="92" t="n"/>
+      <c r="F22" s="86" t="n"/>
+      <c r="G22" s="86" t="n"/>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="81" t="n"/>
-      <c r="B23" s="93" t="inlineStr">
+      <c r="A23" s="79" t="n"/>
+      <c r="B23" s="91" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C23" s="86" t="inlineStr">
+      <c r="C23" s="84" t="inlineStr">
         <is>
           <t xml:space="preserve">  本シートを保管・アーカイブ予定</t>
         </is>
       </c>
-      <c r="E23" s="7" t="n"/>
-      <c r="F23" s="88" t="n"/>
-      <c r="G23" s="88" t="n"/>
+      <c r="E23" s="92" t="n"/>
+      <c r="F23" s="86" t="n"/>
+      <c r="G23" s="86" t="n"/>
     </row>
     <row r="24" ht="4" customHeight="1">
-      <c r="A24" s="81" t="n"/>
-      <c r="B24" s="81" t="n"/>
-      <c r="C24" s="81" t="n"/>
-      <c r="D24" s="81" t="n"/>
-      <c r="E24" s="81" t="n"/>
-      <c r="F24" s="81" t="n"/>
-      <c r="G24" s="81" t="n"/>
+      <c r="A24" s="79" t="n"/>
+      <c r="B24" s="79" t="n"/>
+      <c r="C24" s="79" t="n"/>
+      <c r="D24" s="79" t="n"/>
+      <c r="E24" s="79" t="n"/>
+      <c r="F24" s="79" t="n"/>
+      <c r="G24" s="79" t="n"/>
     </row>
     <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="81" t="n"/>
-      <c r="B25" s="81" t="n"/>
-      <c r="C25" s="81" t="n"/>
-      <c r="D25" s="81" t="n"/>
-      <c r="E25" s="81" t="n"/>
-      <c r="F25" s="81" t="n"/>
-      <c r="G25" s="81" t="n"/>
+      <c r="A25" s="79" t="n"/>
+      <c r="B25" s="79" t="n"/>
+      <c r="C25" s="79" t="n"/>
+      <c r="D25" s="79" t="n"/>
+      <c r="E25" s="79" t="n"/>
+      <c r="F25" s="79" t="n"/>
+      <c r="G25" s="79" t="n"/>
     </row>
     <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="81" t="n"/>
-      <c r="B26" s="81" t="n"/>
-      <c r="C26" s="81" t="n"/>
-      <c r="D26" s="81" t="n"/>
-      <c r="E26" s="81" t="n"/>
-      <c r="F26" s="81" t="n"/>
-      <c r="G26" s="81" t="n"/>
+      <c r="A26" s="79" t="n"/>
+      <c r="B26" s="79" t="n"/>
+      <c r="C26" s="79" t="n"/>
+      <c r="D26" s="79" t="n"/>
+      <c r="E26" s="79" t="n"/>
+      <c r="F26" s="79" t="n"/>
+      <c r="G26" s="79" t="n"/>
     </row>
     <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="81" t="n"/>
-      <c r="B27" s="81" t="n"/>
-      <c r="C27" s="81" t="n"/>
-      <c r="D27" s="81" t="n"/>
-      <c r="E27" s="81" t="n"/>
-      <c r="F27" s="81" t="n"/>
-      <c r="G27" s="81" t="n"/>
+      <c r="A27" s="79" t="n"/>
+      <c r="B27" s="79" t="n"/>
+      <c r="C27" s="79" t="n"/>
+      <c r="D27" s="79" t="n"/>
+      <c r="E27" s="79" t="n"/>
+      <c r="F27" s="79" t="n"/>
+      <c r="G27" s="79" t="n"/>
     </row>
     <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="81" t="n"/>
-      <c r="B28" s="81" t="n"/>
-      <c r="C28" s="81" t="n"/>
-      <c r="D28" s="81" t="n"/>
-      <c r="E28" s="81" t="n"/>
-      <c r="F28" s="81" t="n"/>
-      <c r="G28" s="81" t="n"/>
+      <c r="A28" s="79" t="n"/>
+      <c r="B28" s="79" t="n"/>
+      <c r="C28" s="79" t="n"/>
+      <c r="D28" s="79" t="n"/>
+      <c r="E28" s="79" t="n"/>
+      <c r="F28" s="79" t="n"/>
+      <c r="G28" s="79" t="n"/>
     </row>
     <row r="29" ht="16" customHeight="1">
-      <c r="A29" s="81" t="n"/>
-      <c r="B29" s="81" t="n"/>
-      <c r="C29" s="81" t="n"/>
-      <c r="D29" s="81" t="n"/>
-      <c r="E29" s="81" t="n"/>
-      <c r="F29" s="81" t="n"/>
-      <c r="G29" s="81" t="n"/>
+      <c r="A29" s="79" t="n"/>
+      <c r="B29" s="79" t="n"/>
+      <c r="C29" s="79" t="n"/>
+      <c r="D29" s="79" t="n"/>
+      <c r="E29" s="79" t="n"/>
+      <c r="F29" s="79" t="n"/>
+      <c r="G29" s="79" t="n"/>
     </row>
     <row r="30" ht="16" customHeight="1">
-      <c r="A30" s="81" t="n"/>
-      <c r="B30" s="81" t="n"/>
-      <c r="C30" s="81" t="n"/>
-      <c r="D30" s="81" t="n"/>
-      <c r="E30" s="81" t="n"/>
-      <c r="F30" s="81" t="n"/>
-      <c r="G30" s="81" t="n"/>
+      <c r="A30" s="79" t="n"/>
+      <c r="B30" s="79" t="n"/>
+      <c r="C30" s="79" t="n"/>
+      <c r="D30" s="79" t="n"/>
+      <c r="E30" s="79" t="n"/>
+      <c r="F30" s="79" t="n"/>
+      <c r="G30" s="79" t="n"/>
     </row>
     <row r="31" ht="16" customHeight="1">
-      <c r="A31" s="81" t="n"/>
-      <c r="B31" s="81" t="n"/>
-      <c r="C31" s="81" t="n"/>
-      <c r="D31" s="81" t="n"/>
-      <c r="E31" s="81" t="n"/>
-      <c r="F31" s="81" t="n"/>
-      <c r="G31" s="81" t="n"/>
+      <c r="A31" s="79" t="n"/>
+      <c r="B31" s="79" t="n"/>
+      <c r="C31" s="79" t="n"/>
+      <c r="D31" s="79" t="n"/>
+      <c r="E31" s="79" t="n"/>
+      <c r="F31" s="79" t="n"/>
+      <c r="G31" s="79" t="n"/>
     </row>
     <row r="32" ht="16" customHeight="1">
-      <c r="A32" s="81" t="n"/>
-      <c r="B32" s="81" t="n"/>
-      <c r="C32" s="81" t="n"/>
-      <c r="D32" s="81" t="n"/>
-      <c r="E32" s="81" t="n"/>
-      <c r="F32" s="81" t="n"/>
-      <c r="G32" s="81" t="n"/>
+      <c r="A32" s="79" t="n"/>
+      <c r="B32" s="79" t="n"/>
+      <c r="C32" s="79" t="n"/>
+      <c r="D32" s="79" t="n"/>
+      <c r="E32" s="79" t="n"/>
+      <c r="F32" s="79" t="n"/>
+      <c r="G32" s="79" t="n"/>
     </row>
     <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="81" t="n"/>
-      <c r="B33" s="81" t="n"/>
-      <c r="C33" s="81" t="n"/>
-      <c r="D33" s="81" t="n"/>
-      <c r="E33" s="81" t="n"/>
-      <c r="F33" s="81" t="n"/>
-      <c r="G33" s="81" t="n"/>
+      <c r="A33" s="79" t="n"/>
+      <c r="B33" s="79" t="n"/>
+      <c r="C33" s="79" t="n"/>
+      <c r="D33" s="79" t="n"/>
+      <c r="E33" s="79" t="n"/>
+      <c r="F33" s="79" t="n"/>
+      <c r="G33" s="79" t="n"/>
     </row>
     <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="81" t="n"/>
-      <c r="B34" s="81" t="n"/>
-      <c r="C34" s="81" t="n"/>
-      <c r="D34" s="81" t="n"/>
-      <c r="E34" s="81" t="n"/>
-      <c r="F34" s="81" t="n"/>
-      <c r="G34" s="81" t="n"/>
+      <c r="A34" s="79" t="n"/>
+      <c r="B34" s="79" t="n"/>
+      <c r="C34" s="79" t="n"/>
+      <c r="D34" s="79" t="n"/>
+      <c r="E34" s="79" t="n"/>
+      <c r="F34" s="79" t="n"/>
+      <c r="G34" s="79" t="n"/>
     </row>
     <row r="35" ht="16" customHeight="1">
-      <c r="A35" s="81" t="n"/>
-      <c r="B35" s="81" t="n"/>
-      <c r="C35" s="81" t="n"/>
-      <c r="D35" s="81" t="n"/>
-      <c r="E35" s="81" t="n"/>
-      <c r="F35" s="81" t="n"/>
-      <c r="G35" s="81" t="n"/>
+      <c r="A35" s="79" t="n"/>
+      <c r="B35" s="79" t="n"/>
+      <c r="C35" s="79" t="n"/>
+      <c r="D35" s="79" t="n"/>
+      <c r="E35" s="79" t="n"/>
+      <c r="F35" s="79" t="n"/>
+      <c r="G35" s="79" t="n"/>
     </row>
     <row r="36" ht="16" customHeight="1">
-      <c r="A36" s="81" t="n"/>
-      <c r="B36" s="81" t="n"/>
-      <c r="C36" s="81" t="n"/>
-      <c r="D36" s="81" t="n"/>
-      <c r="E36" s="81" t="n"/>
-      <c r="F36" s="81" t="n"/>
-      <c r="G36" s="81" t="n"/>
+      <c r="A36" s="79" t="n"/>
+      <c r="B36" s="79" t="n"/>
+      <c r="C36" s="79" t="n"/>
+      <c r="D36" s="79" t="n"/>
+      <c r="E36" s="79" t="n"/>
+      <c r="F36" s="79" t="n"/>
+      <c r="G36" s="79" t="n"/>
     </row>
     <row r="37" ht="16" customHeight="1">
-      <c r="A37" s="81" t="n"/>
-      <c r="B37" s="81" t="n"/>
-      <c r="C37" s="81" t="n"/>
-      <c r="D37" s="81" t="n"/>
-      <c r="E37" s="81" t="n"/>
-      <c r="F37" s="81" t="n"/>
-      <c r="G37" s="81" t="n"/>
+      <c r="A37" s="79" t="n"/>
+      <c r="B37" s="79" t="n"/>
+      <c r="C37" s="79" t="n"/>
+      <c r="D37" s="79" t="n"/>
+      <c r="E37" s="79" t="n"/>
+      <c r="F37" s="79" t="n"/>
+      <c r="G37" s="79" t="n"/>
     </row>
     <row r="38" ht="16" customHeight="1">
-      <c r="A38" s="81" t="n"/>
-      <c r="B38" s="81" t="n"/>
-      <c r="C38" s="81" t="n"/>
-      <c r="D38" s="81" t="n"/>
-      <c r="E38" s="81" t="n"/>
-      <c r="F38" s="81" t="n"/>
-      <c r="G38" s="81" t="n"/>
+      <c r="A38" s="79" t="n"/>
+      <c r="B38" s="79" t="n"/>
+      <c r="C38" s="79" t="n"/>
+      <c r="D38" s="79" t="n"/>
+      <c r="E38" s="79" t="n"/>
+      <c r="F38" s="79" t="n"/>
+      <c r="G38" s="79" t="n"/>
     </row>
     <row r="39" ht="16" customHeight="1">
-      <c r="A39" s="81" t="n"/>
-      <c r="B39" s="81" t="n"/>
-      <c r="C39" s="81" t="n"/>
-      <c r="D39" s="81" t="n"/>
-      <c r="E39" s="81" t="n"/>
-      <c r="F39" s="81" t="n"/>
-      <c r="G39" s="81" t="n"/>
+      <c r="A39" s="79" t="n"/>
+      <c r="B39" s="79" t="n"/>
+      <c r="C39" s="79" t="n"/>
+      <c r="D39" s="79" t="n"/>
+      <c r="E39" s="79" t="n"/>
+      <c r="F39" s="79" t="n"/>
+      <c r="G39" s="79" t="n"/>
     </row>
     <row r="40" ht="16" customHeight="1">
-      <c r="A40" s="81" t="n"/>
-      <c r="B40" s="81" t="n"/>
-      <c r="C40" s="81" t="n"/>
-      <c r="D40" s="81" t="n"/>
-      <c r="E40" s="81" t="n"/>
-      <c r="F40" s="81" t="n"/>
-      <c r="G40" s="81" t="n"/>
+      <c r="A40" s="79" t="n"/>
+      <c r="B40" s="79" t="n"/>
+      <c r="C40" s="79" t="n"/>
+      <c r="D40" s="79" t="n"/>
+      <c r="E40" s="79" t="n"/>
+      <c r="F40" s="79" t="n"/>
+      <c r="G40" s="79" t="n"/>
     </row>
     <row r="41" ht="16" customHeight="1">
-      <c r="A41" s="81" t="n"/>
-      <c r="B41" s="81" t="n"/>
-      <c r="C41" s="81" t="n"/>
-      <c r="D41" s="81" t="n"/>
-      <c r="E41" s="81" t="n"/>
-      <c r="F41" s="81" t="n"/>
-      <c r="G41" s="81" t="n"/>
+      <c r="A41" s="79" t="n"/>
+      <c r="B41" s="79" t="n"/>
+      <c r="C41" s="79" t="n"/>
+      <c r="D41" s="79" t="n"/>
+      <c r="E41" s="79" t="n"/>
+      <c r="F41" s="79" t="n"/>
+      <c r="G41" s="79" t="n"/>
     </row>
     <row r="42" ht="16" customHeight="1">
-      <c r="A42" s="81" t="n"/>
-      <c r="B42" s="81" t="n"/>
-      <c r="C42" s="81" t="n"/>
-      <c r="D42" s="81" t="n"/>
-      <c r="E42" s="81" t="n"/>
-      <c r="F42" s="81" t="n"/>
-      <c r="G42" s="81" t="n"/>
+      <c r="A42" s="79" t="n"/>
+      <c r="B42" s="79" t="n"/>
+      <c r="C42" s="79" t="n"/>
+      <c r="D42" s="79" t="n"/>
+      <c r="E42" s="79" t="n"/>
+      <c r="F42" s="79" t="n"/>
+      <c r="G42" s="79" t="n"/>
     </row>
     <row r="43" ht="16" customHeight="1">
-      <c r="A43" s="81" t="n"/>
-      <c r="B43" s="81" t="n"/>
-      <c r="C43" s="81" t="n"/>
-      <c r="D43" s="81" t="n"/>
-      <c r="E43" s="81" t="n"/>
-      <c r="F43" s="81" t="n"/>
-      <c r="G43" s="81" t="n"/>
+      <c r="A43" s="79" t="n"/>
+      <c r="B43" s="79" t="n"/>
+      <c r="C43" s="79" t="n"/>
+      <c r="D43" s="79" t="n"/>
+      <c r="E43" s="79" t="n"/>
+      <c r="F43" s="79" t="n"/>
+      <c r="G43" s="79" t="n"/>
     </row>
     <row r="44" ht="16" customHeight="1">
-      <c r="A44" s="81" t="n"/>
-      <c r="B44" s="81" t="n"/>
-      <c r="C44" s="81" t="n"/>
-      <c r="D44" s="81" t="n"/>
-      <c r="E44" s="81" t="n"/>
-      <c r="F44" s="81" t="n"/>
-      <c r="G44" s="81" t="n"/>
+      <c r="A44" s="79" t="n"/>
+      <c r="B44" s="79" t="n"/>
+      <c r="C44" s="79" t="n"/>
+      <c r="D44" s="79" t="n"/>
+      <c r="E44" s="79" t="n"/>
+      <c r="F44" s="79" t="n"/>
+      <c r="G44" s="79" t="n"/>
     </row>
     <row r="45" ht="16" customHeight="1">
-      <c r="A45" s="81" t="n"/>
-      <c r="B45" s="81" t="n"/>
-      <c r="C45" s="81" t="n"/>
-      <c r="D45" s="81" t="n"/>
-      <c r="E45" s="81" t="n"/>
-      <c r="F45" s="81" t="n"/>
-      <c r="G45" s="81" t="n"/>
+      <c r="A45" s="79" t="n"/>
+      <c r="B45" s="79" t="n"/>
+      <c r="C45" s="79" t="n"/>
+      <c r="D45" s="79" t="n"/>
+      <c r="E45" s="79" t="n"/>
+      <c r="F45" s="79" t="n"/>
+      <c r="G45" s="79" t="n"/>
     </row>
     <row r="46" ht="16" customHeight="1">
-      <c r="A46" s="81" t="n"/>
-      <c r="B46" s="81" t="n"/>
-      <c r="C46" s="81" t="n"/>
-      <c r="D46" s="81" t="n"/>
-      <c r="E46" s="81" t="n"/>
-      <c r="F46" s="81" t="n"/>
-      <c r="G46" s="81" t="n"/>
+      <c r="A46" s="79" t="n"/>
+      <c r="B46" s="79" t="n"/>
+      <c r="C46" s="79" t="n"/>
+      <c r="D46" s="79" t="n"/>
+      <c r="E46" s="79" t="n"/>
+      <c r="F46" s="79" t="n"/>
+      <c r="G46" s="79" t="n"/>
     </row>
     <row r="47" ht="16" customHeight="1">
-      <c r="A47" s="81" t="n"/>
-      <c r="B47" s="81" t="n"/>
-      <c r="C47" s="81" t="n"/>
-      <c r="D47" s="81" t="n"/>
-      <c r="E47" s="81" t="n"/>
-      <c r="F47" s="81" t="n"/>
-      <c r="G47" s="81" t="n"/>
+      <c r="A47" s="79" t="n"/>
+      <c r="B47" s="79" t="n"/>
+      <c r="C47" s="79" t="n"/>
+      <c r="D47" s="79" t="n"/>
+      <c r="E47" s="79" t="n"/>
+      <c r="F47" s="79" t="n"/>
+      <c r="G47" s="79" t="n"/>
     </row>
     <row r="48" ht="16" customHeight="1">
-      <c r="A48" s="81" t="n"/>
-      <c r="B48" s="81" t="n"/>
-      <c r="C48" s="81" t="n"/>
-      <c r="D48" s="81" t="n"/>
-      <c r="E48" s="81" t="n"/>
-      <c r="F48" s="81" t="n"/>
-      <c r="G48" s="81" t="n"/>
+      <c r="A48" s="79" t="n"/>
+      <c r="B48" s="79" t="n"/>
+      <c r="C48" s="79" t="n"/>
+      <c r="D48" s="79" t="n"/>
+      <c r="E48" s="79" t="n"/>
+      <c r="F48" s="79" t="n"/>
+      <c r="G48" s="79" t="n"/>
     </row>
     <row r="49" ht="16" customHeight="1">
-      <c r="A49" s="81" t="n"/>
-      <c r="B49" s="81" t="n"/>
-      <c r="C49" s="81" t="n"/>
-      <c r="D49" s="81" t="n"/>
-      <c r="E49" s="81" t="n"/>
-      <c r="F49" s="81" t="n"/>
-      <c r="G49" s="81" t="n"/>
+      <c r="A49" s="79" t="n"/>
+      <c r="B49" s="79" t="n"/>
+      <c r="C49" s="79" t="n"/>
+      <c r="D49" s="79" t="n"/>
+      <c r="E49" s="79" t="n"/>
+      <c r="F49" s="79" t="n"/>
+      <c r="G49" s="79" t="n"/>
+    </row>
+    <row r="50" ht="16" customHeight="1">
+      <c r="A50" s="79" t="n"/>
+      <c r="B50" s="79" t="n"/>
+      <c r="C50" s="79" t="n"/>
+      <c r="D50" s="79" t="n"/>
+      <c r="E50" s="79" t="n"/>
+      <c r="F50" s="79" t="n"/>
+      <c r="G50" s="79" t="n"/>
+    </row>
+    <row r="51" ht="16" customHeight="1">
+      <c r="A51" s="79" t="n"/>
+      <c r="B51" s="79" t="n"/>
+      <c r="C51" s="79" t="n"/>
+      <c r="D51" s="79" t="n"/>
+      <c r="E51" s="79" t="n"/>
+      <c r="F51" s="79" t="n"/>
+      <c r="G51" s="79" t="n"/>
+    </row>
+    <row r="52" ht="16" customHeight="1">
+      <c r="A52" s="79" t="n"/>
+      <c r="B52" s="79" t="n"/>
+      <c r="C52" s="79" t="n"/>
+      <c r="D52" s="79" t="n"/>
+      <c r="E52" s="79" t="n"/>
+      <c r="F52" s="79" t="n"/>
+      <c r="G52" s="79" t="n"/>
+    </row>
+    <row r="53" ht="16" customHeight="1">
+      <c r="A53" s="79" t="n"/>
+      <c r="B53" s="79" t="n"/>
+      <c r="C53" s="79" t="n"/>
+      <c r="D53" s="79" t="n"/>
+      <c r="E53" s="79" t="n"/>
+      <c r="F53" s="79" t="n"/>
+      <c r="G53" s="79" t="n"/>
+    </row>
+    <row r="54" ht="16" customHeight="1">
+      <c r="A54" s="79" t="n"/>
+      <c r="B54" s="79" t="n"/>
+      <c r="C54" s="79" t="n"/>
+      <c r="D54" s="79" t="n"/>
+      <c r="E54" s="79" t="n"/>
+      <c r="F54" s="79" t="n"/>
+      <c r="G54" s="79" t="n"/>
+    </row>
+    <row r="55" ht="16" customHeight="1">
+      <c r="A55" s="79" t="n"/>
+      <c r="B55" s="79" t="n"/>
+      <c r="C55" s="79" t="n"/>
+      <c r="D55" s="79" t="n"/>
+      <c r="E55" s="79" t="n"/>
+      <c r="F55" s="79" t="n"/>
+      <c r="G55" s="79" t="n"/>
+    </row>
+    <row r="56" ht="16" customHeight="1">
+      <c r="A56" s="79" t="n"/>
+      <c r="B56" s="79" t="n"/>
+      <c r="C56" s="79" t="n"/>
+      <c r="D56" s="79" t="n"/>
+      <c r="E56" s="79" t="n"/>
+      <c r="F56" s="79" t="n"/>
+      <c r="G56" s="79" t="n"/>
+    </row>
+    <row r="57" ht="16" customHeight="1">
+      <c r="A57" s="79" t="n"/>
+      <c r="B57" s="79" t="n"/>
+      <c r="C57" s="79" t="n"/>
+      <c r="D57" s="79" t="n"/>
+      <c r="E57" s="79" t="n"/>
+      <c r="F57" s="79" t="n"/>
+      <c r="G57" s="79" t="n"/>
+    </row>
+    <row r="58" ht="16" customHeight="1">
+      <c r="A58" s="79" t="n"/>
+      <c r="B58" s="79" t="n"/>
+      <c r="C58" s="79" t="n"/>
+      <c r="D58" s="79" t="n"/>
+      <c r="E58" s="79" t="n"/>
+      <c r="F58" s="79" t="n"/>
+      <c r="G58" s="79" t="n"/>
+    </row>
+    <row r="59" ht="16" customHeight="1">
+      <c r="A59" s="79" t="n"/>
+      <c r="B59" s="79" t="n"/>
+      <c r="C59" s="79" t="n"/>
+      <c r="D59" s="79" t="n"/>
+      <c r="E59" s="79" t="n"/>
+      <c r="F59" s="79" t="n"/>
+      <c r="G59" s="79" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="20">
@@ -3284,8 +3469,8 @@
     <mergeCell ref="C21:D21"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="B4:G4"/>
+    <mergeCell ref="C17:D17"/>
     <mergeCell ref="C23:D23"/>
-    <mergeCell ref="C17:D17"/>
     <mergeCell ref="C8:D8"/>
     <mergeCell ref="C7:D7"/>
     <mergeCell ref="A2:G2"/>

</xml_diff>

<commit_message>
Fix H7 dropdown: remove empty string value causing inlineStr type conflict
- H7 and H10 now have no pre-set value (type=n/empty), resolving the
  data validation interference caused by inlineStr cell type
- Apply frame borders first, then override H7/H10 with red medium border
- Split STEP1 header to B7:F7, add G7 label "契約方法を選択 ▼"
- Add H10 as second prominent dropdown target in the dedicated input row

https://claude.ai/code/session_01AJdG4TQantm5HZTxDeQNzp
</commit_message>
<xml_diff>
--- a/intent_tool.xlsx
+++ b/intent_tool.xlsx
@@ -57,6 +57,12 @@
     <font>
       <name val="Meiryo UI"/>
       <b val="1"/>
+      <color rgb="001C3557"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Meiryo UI"/>
+      <b val="1"/>
       <color rgb="00C5D8F5"/>
       <sz val="8"/>
     </font>
@@ -81,13 +87,7 @@
       <name val="Meiryo UI"/>
       <b val="1"/>
       <color rgb="00C0392B"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Meiryo UI"/>
-      <b val="1"/>
-      <color rgb="00C0392B"/>
-      <sz val="8"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Meiryo UI"/>
@@ -115,13 +115,13 @@
     <font>
       <name val="Meiryo UI"/>
       <b val="1"/>
-      <color rgb="00C0392B"/>
-      <sz val="9"/>
+      <color rgb="002E7D5B"/>
+      <sz val="8"/>
     </font>
     <font>
       <name val="Meiryo UI"/>
       <b val="1"/>
-      <color rgb="002E7D5B"/>
+      <color rgb="00C0392B"/>
       <sz val="8"/>
     </font>
     <font>
@@ -251,7 +251,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF0F0"/>
+        <fgColor rgb="00FFF8E1"/>
       </patternFill>
     </fill>
     <fill>
@@ -315,7 +315,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -335,34 +335,6 @@
       </top>
       <bottom style="thin">
         <color rgb="00BFC5BB"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="00C0392B"/>
-      </left>
-      <right style="medium">
-        <color rgb="00C0392B"/>
-      </right>
-      <top style="medium">
-        <color rgb="00C0392B"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="00C0392B"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="00C0392B"/>
-      </left>
-      <right style="thin">
-        <color rgb="00C0392B"/>
-      </right>
-      <top style="thin">
-        <color rgb="00C0392B"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00C0392B"/>
       </bottom>
     </border>
     <border>
@@ -479,6 +451,20 @@
     </border>
     <border>
       <left style="medium">
+        <color rgb="00C0392B"/>
+      </left>
+      <right style="medium">
+        <color rgb="00C0392B"/>
+      </right>
+      <top style="medium">
+        <color rgb="00C0392B"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00C0392B"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
         <color rgb="002E7D5B"/>
       </left>
       <right style="medium">
@@ -537,7 +523,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -555,162 +541,171 @@
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="15" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="15" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="19" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="13" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="20" fillId="12" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="20" fillId="12" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="17" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="17" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="18" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="20" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="20" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="14" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -719,25 +714,25 @@
     <xf numFmtId="0" fontId="28" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="27" fillId="20" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="20" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="18" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="29" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -757,28 +752,28 @@
     <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="30" fillId="5" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="5" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="30" fillId="5" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="5" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="5" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="30" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1244,32 +1239,36 @@
       <c r="D7" s="8" t="n"/>
       <c r="E7" s="8" t="n"/>
       <c r="F7" s="8" t="n"/>
-      <c r="G7" s="8" t="n"/>
-      <c r="H7" s="9" t="inlineStr"/>
+      <c r="G7" s="9" t="inlineStr">
+        <is>
+          <t>契約方法を選択 ▼</t>
+        </is>
+      </c>
+      <c r="H7" s="10" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="3" t="n"/>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>📋 スクリプト</t>
         </is>
       </c>
-      <c r="C8" s="11" t="n"/>
-      <c r="D8" s="12" t="inlineStr"/>
-      <c r="E8" s="11" t="n"/>
-      <c r="F8" s="11" t="n"/>
-      <c r="G8" s="11" t="n"/>
-      <c r="H8" s="13" t="n"/>
+      <c r="C8" s="12" t="n"/>
+      <c r="D8" s="13" t="inlineStr"/>
+      <c r="E8" s="12" t="n"/>
+      <c r="F8" s="12" t="n"/>
+      <c r="G8" s="12" t="n"/>
+      <c r="H8" s="14" t="n"/>
     </row>
     <row r="9" ht="80" customHeight="1">
       <c r="A9" s="3" t="n"/>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B9" s="15" t="inlineStr">
         <is>
           <t>📣 読み上げ</t>
         </is>
       </c>
-      <c r="C9" s="11" t="n"/>
-      <c r="D9" s="15" t="inlineStr">
+      <c r="C9" s="12" t="n"/>
+      <c r="D9" s="16" t="inlineStr">
         <is>
           <t>「当社では●社の自動車保険を扱っています。
 そのうち 給与天引き（団体割引）が使えるのは 損保ジャパン・三井住友海上・東京海上 の3社です。
@@ -1277,87 +1276,90 @@
 どのご契約方法をご希望ですか？」</t>
         </is>
       </c>
-      <c r="E9" s="11" t="n"/>
-      <c r="F9" s="11" t="n"/>
-      <c r="G9" s="11" t="n"/>
-      <c r="H9" s="16" t="inlineStr">
-        <is>
-          <t>← ここで
-選択</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="20" customHeight="1">
+      <c r="E9" s="12" t="n"/>
+      <c r="F9" s="12" t="n"/>
+      <c r="G9" s="12" t="n"/>
+      <c r="H9" s="14" t="n"/>
+    </row>
+    <row r="10" ht="26" customHeight="1">
       <c r="A10" s="3" t="n"/>
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>①</t>
-        </is>
-      </c>
-      <c r="C10" s="18" t="inlineStr">
-        <is>
-          <t>給与天引き（団体割引）</t>
-        </is>
-      </c>
-      <c r="D10" s="19" t="inlineStr">
-        <is>
-          <t>→ 下のグループ「①②」を展開</t>
-        </is>
-      </c>
-      <c r="E10" s="11" t="n"/>
-      <c r="F10" s="11" t="n"/>
-      <c r="G10" s="11" t="n"/>
-      <c r="H10" s="20" t="n"/>
+          <t xml:space="preserve">  ▶ お客様のご希望の契約方法（右の黄色セルで選択してください）</t>
+        </is>
+      </c>
+      <c r="C10" s="12" t="n"/>
+      <c r="D10" s="12" t="n"/>
+      <c r="E10" s="12" t="n"/>
+      <c r="F10" s="12" t="n"/>
+      <c r="G10" s="18" t="inlineStr">
+        <is>
+          <t>契約方法 →</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="3" t="n"/>
-      <c r="B11" s="21" t="inlineStr">
-        <is>
-          <t>②</t>
-        </is>
-      </c>
-      <c r="C11" s="22" t="inlineStr">
-        <is>
-          <t>一般契約（クレカ・口振）</t>
-        </is>
-      </c>
-      <c r="D11" s="23" t="inlineStr">
+      <c r="B11" s="19" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C11" s="20" t="inlineStr">
+        <is>
+          <t>給与天引き（団体割引）</t>
+        </is>
+      </c>
+      <c r="D11" s="21" t="inlineStr">
         <is>
           <t>→ 下のグループ「①②」を展開</t>
         </is>
       </c>
-      <c r="E11" s="11" t="n"/>
-      <c r="F11" s="11" t="n"/>
-      <c r="G11" s="11" t="n"/>
-      <c r="H11" s="24" t="n"/>
+      <c r="E11" s="12" t="n"/>
+      <c r="F11" s="12" t="n"/>
+      <c r="G11" s="12" t="n"/>
+      <c r="H11" s="22" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="3" t="n"/>
-      <c r="B12" s="25" t="inlineStr">
-        <is>
-          <t>③</t>
-        </is>
-      </c>
-      <c r="C12" s="26" t="inlineStr">
-        <is>
-          <t>通販型（ソニー損保）</t>
-        </is>
-      </c>
-      <c r="D12" s="27" t="inlineStr">
-        <is>
-          <t>→ 下のグループ「③」を展開</t>
-        </is>
-      </c>
-      <c r="E12" s="11" t="n"/>
-      <c r="F12" s="11" t="n"/>
-      <c r="G12" s="11" t="n"/>
-      <c r="H12" s="28" t="n"/>
+      <c r="B12" s="23" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C12" s="24" t="inlineStr">
+        <is>
+          <t>一般契約（クレカ・口振）</t>
+        </is>
+      </c>
+      <c r="D12" s="25" t="inlineStr">
+        <is>
+          <t>→ 下のグループ「①②」を展開</t>
+        </is>
+      </c>
+      <c r="E12" s="12" t="n"/>
+      <c r="F12" s="12" t="n"/>
+      <c r="G12" s="12" t="n"/>
+      <c r="H12" s="26" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="3" t="n"/>
-      <c r="B13" s="29" t="n"/>
-      <c r="C13" s="30" t="n"/>
-      <c r="D13" s="30" t="n"/>
+      <c r="B13" s="27" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C13" s="28" t="inlineStr">
+        <is>
+          <t>通販型（ソニー損保）</t>
+        </is>
+      </c>
+      <c r="D13" s="29" t="inlineStr">
+        <is>
+          <t>→ 下のグループ「③」を展開</t>
+        </is>
+      </c>
       <c r="E13" s="30" t="n"/>
       <c r="F13" s="30" t="n"/>
       <c r="G13" s="30" t="n"/>
@@ -1407,12 +1409,12 @@
           <t>📋 スクリプト</t>
         </is>
       </c>
-      <c r="C17" s="11" t="n"/>
+      <c r="C17" s="12" t="n"/>
       <c r="D17" s="37" t="inlineStr"/>
-      <c r="E17" s="11" t="n"/>
-      <c r="F17" s="11" t="n"/>
-      <c r="G17" s="11" t="n"/>
-      <c r="H17" s="13" t="n"/>
+      <c r="E17" s="12" t="n"/>
+      <c r="F17" s="12" t="n"/>
+      <c r="G17" s="12" t="n"/>
+      <c r="H17" s="14" t="n"/>
     </row>
     <row r="18" hidden="1" outlineLevel="1" ht="60" customHeight="1">
       <c r="A18" s="3" t="n"/>
@@ -1421,17 +1423,17 @@
           <t>📣 読み上げ</t>
         </is>
       </c>
-      <c r="C18" s="11" t="n"/>
+      <c r="C18" s="12" t="n"/>
       <c r="D18" s="39" t="inlineStr">
         <is>
           <t>「自動車保険でいちばん大切にしていることを教えていただけますか？
 いくつかお伺いしてもよいでしょうか？当てはまるものに○をつけてください。（複数回答可）」</t>
         </is>
       </c>
-      <c r="E18" s="11" t="n"/>
-      <c r="F18" s="11" t="n"/>
-      <c r="G18" s="11" t="n"/>
-      <c r="H18" s="13" t="n"/>
+      <c r="E18" s="12" t="n"/>
+      <c r="F18" s="12" t="n"/>
+      <c r="G18" s="12" t="n"/>
+      <c r="H18" s="14" t="n"/>
     </row>
     <row r="19" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A19" s="3" t="n"/>
@@ -1440,20 +1442,20 @@
           <t>重視項目</t>
         </is>
       </c>
-      <c r="C19" s="11" t="n"/>
+      <c r="C19" s="12" t="n"/>
       <c r="D19" s="40" t="inlineStr">
         <is>
           <t>お客様選択</t>
         </is>
       </c>
-      <c r="E19" s="11" t="n"/>
+      <c r="E19" s="12" t="n"/>
       <c r="F19" s="40" t="inlineStr">
         <is>
           <t>各社の強み（参考）</t>
         </is>
       </c>
-      <c r="G19" s="11" t="n"/>
-      <c r="H19" s="13" t="n"/>
+      <c r="G19" s="12" t="n"/>
+      <c r="H19" s="14" t="n"/>
     </row>
     <row r="20" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A20" s="3" t="n"/>
@@ -1467,14 +1469,14 @@
           <t xml:space="preserve">  保険料をできるだけ抑えたい</t>
         </is>
       </c>
-      <c r="D20" s="11" t="n"/>
-      <c r="E20" s="11" t="n"/>
+      <c r="D20" s="12" t="n"/>
+      <c r="E20" s="12" t="n"/>
       <c r="F20" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">  損保ジャパン（多様なプラン）／三井住友海上（ネット割引あり）</t>
         </is>
       </c>
-      <c r="G20" s="11" t="n"/>
+      <c r="G20" s="12" t="n"/>
       <c r="H20" s="44" t="n"/>
     </row>
     <row r="21" hidden="1" outlineLevel="1" ht="20" customHeight="1">
@@ -1489,14 +1491,14 @@
           <t xml:space="preserve">  補償をしっかり充実させたい</t>
         </is>
       </c>
-      <c r="D21" s="11" t="n"/>
-      <c r="E21" s="11" t="n"/>
+      <c r="D21" s="12" t="n"/>
+      <c r="E21" s="12" t="n"/>
       <c r="F21" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">  東京海上（総合型・特約充実）／損保ジャパン（幅広い特約）</t>
         </is>
       </c>
-      <c r="G21" s="11" t="n"/>
+      <c r="G21" s="12" t="n"/>
       <c r="H21" s="44" t="n"/>
     </row>
     <row r="22" hidden="1" outlineLevel="1" ht="20" customHeight="1">
@@ -1511,14 +1513,14 @@
           <t xml:space="preserve">  事故時の対応・サポートを重視したい</t>
         </is>
       </c>
-      <c r="D22" s="11" t="n"/>
-      <c r="E22" s="11" t="n"/>
+      <c r="D22" s="12" t="n"/>
+      <c r="E22" s="12" t="n"/>
       <c r="F22" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">  三井住友海上（示談交渉◎）／東京海上（専任担当）</t>
         </is>
       </c>
-      <c r="G22" s="11" t="n"/>
+      <c r="G22" s="12" t="n"/>
       <c r="H22" s="44" t="n"/>
     </row>
     <row r="23" hidden="1" outlineLevel="1" ht="20" customHeight="1">
@@ -1533,14 +1535,14 @@
           <t xml:space="preserve">  手続きが簡単・わかりやすいものがいい</t>
         </is>
       </c>
-      <c r="D23" s="11" t="n"/>
-      <c r="E23" s="11" t="n"/>
+      <c r="D23" s="12" t="n"/>
+      <c r="E23" s="12" t="n"/>
       <c r="F23" s="43" t="inlineStr">
         <is>
           <t xml:space="preserve">  三井住友海上（シンプル設計・見積り速い）</t>
         </is>
       </c>
-      <c r="G23" s="11" t="n"/>
+      <c r="G23" s="12" t="n"/>
       <c r="H23" s="44" t="n"/>
     </row>
     <row r="24" hidden="1" outlineLevel="1" ht="20" customHeight="1">
@@ -1555,15 +1557,15 @@
           <t xml:space="preserve">  担当者に相談しながら決めたい</t>
         </is>
       </c>
-      <c r="D24" s="47" t="n"/>
-      <c r="E24" s="47" t="n"/>
-      <c r="F24" s="48" t="inlineStr">
+      <c r="D24" s="30" t="n"/>
+      <c r="E24" s="30" t="n"/>
+      <c r="F24" s="47" t="inlineStr">
         <is>
           <t xml:space="preserve">  3社すべて対応可。担当者によるサポートが手厚い</t>
         </is>
       </c>
-      <c r="G24" s="47" t="n"/>
-      <c r="H24" s="49" t="n"/>
+      <c r="G24" s="30" t="n"/>
+      <c r="H24" s="48" t="n"/>
     </row>
     <row r="25" hidden="1" outlineLevel="1" ht="18" customHeight="1">
       <c r="A25" s="3" t="n"/>
@@ -1577,7 +1579,7 @@
     </row>
     <row r="26" hidden="1" outlineLevel="1" ht="22" customHeight="1">
       <c r="A26" s="3" t="n"/>
-      <c r="B26" s="50" t="inlineStr">
+      <c r="B26" s="49" t="inlineStr">
         <is>
           <t xml:space="preserve">  STEP 2-2　　3社ご提案（意向確認結果をふまえて）</t>
         </is>
@@ -1597,8 +1599,8 @@
 + ポイント</t>
         </is>
       </c>
-      <c r="C27" s="11" t="n"/>
-      <c r="D27" s="51" t="inlineStr">
+      <c r="C27" s="12" t="n"/>
+      <c r="D27" s="50" t="inlineStr">
         <is>
           <t>「ありがとうございます。いただいたご希望をもとに、損保ジャパン・三井住友海上・東京海上 の3社でお見積りをご用意します。
 ─── 募集人ポイント ────────────────────────────────────────────────────────────
@@ -1607,32 +1609,32 @@
 ────────────────────────────────────────────────────────────────────────────」</t>
         </is>
       </c>
-      <c r="E27" s="11" t="n"/>
-      <c r="F27" s="11" t="n"/>
-      <c r="G27" s="11" t="n"/>
-      <c r="H27" s="13" t="n"/>
+      <c r="E27" s="12" t="n"/>
+      <c r="F27" s="12" t="n"/>
+      <c r="G27" s="12" t="n"/>
+      <c r="H27" s="14" t="n"/>
     </row>
     <row r="28" hidden="1" outlineLevel="1" ht="60" customHeight="1">
       <c r="A28" s="3" t="n"/>
-      <c r="B28" s="52" t="inlineStr">
+      <c r="B28" s="51" t="inlineStr">
         <is>
           <t>会　社</t>
         </is>
       </c>
-      <c r="C28" s="11" t="n"/>
-      <c r="D28" s="53" t="inlineStr">
+      <c r="C28" s="12" t="n"/>
+      <c r="D28" s="52" t="inlineStr">
         <is>
           <t>主な強み・特徴</t>
         </is>
       </c>
-      <c r="E28" s="11" t="n"/>
-      <c r="F28" s="53" t="inlineStr">
+      <c r="E28" s="12" t="n"/>
+      <c r="F28" s="52" t="inlineStr">
         <is>
           <t>MSI提案の一言</t>
         </is>
       </c>
-      <c r="G28" s="11" t="n"/>
-      <c r="H28" s="54" t="inlineStr">
+      <c r="G28" s="12" t="n"/>
+      <c r="H28" s="53" t="inlineStr">
         <is>
           <t>提案</t>
         </is>
@@ -1640,24 +1642,24 @@
     </row>
     <row r="29" hidden="1" outlineLevel="1" ht="18" customHeight="1">
       <c r="A29" s="3" t="n"/>
-      <c r="B29" s="55" t="inlineStr">
+      <c r="B29" s="54" t="inlineStr">
         <is>
           <t xml:space="preserve">  損保ジャパン</t>
         </is>
       </c>
-      <c r="C29" s="11" t="n"/>
-      <c r="D29" s="27" t="inlineStr">
+      <c r="C29" s="12" t="n"/>
+      <c r="D29" s="55" t="inlineStr">
         <is>
           <t xml:space="preserve">  取引歴が長く慣れている。多彩なプラン・特約</t>
         </is>
       </c>
-      <c r="E29" s="11" t="n"/>
+      <c r="E29" s="12" t="n"/>
       <c r="F29" s="56" t="inlineStr">
         <is>
           <t xml:space="preserve">  慣れ親しんだ会社。実績・信頼で推せます</t>
         </is>
       </c>
-      <c r="G29" s="11" t="n"/>
+      <c r="G29" s="12" t="n"/>
       <c r="H29" s="57" t="n"/>
     </row>
     <row r="30" hidden="1" outlineLevel="1" ht="18" customHeight="1">
@@ -1667,19 +1669,19 @@
           <t xml:space="preserve">  三井住友海上</t>
         </is>
       </c>
-      <c r="C30" s="11" t="n"/>
-      <c r="D30" s="19" t="inlineStr">
+      <c r="C30" s="12" t="n"/>
+      <c r="D30" s="21" t="inlineStr">
         <is>
           <t xml:space="preserve">  シンプル設計・見積り速い・ネット割引あり</t>
         </is>
       </c>
-      <c r="E30" s="11" t="n"/>
+      <c r="E30" s="12" t="n"/>
       <c r="F30" s="56" t="inlineStr">
         <is>
           <t xml:space="preserve">  手続きが楽で保険料も競争力あり。比較必須</t>
         </is>
       </c>
-      <c r="G30" s="11" t="n"/>
+      <c r="G30" s="12" t="n"/>
       <c r="H30" s="59" t="n"/>
     </row>
     <row r="31" hidden="1" outlineLevel="1" ht="18" customHeight="1">
@@ -1689,19 +1691,19 @@
           <t xml:space="preserve">  東京海上日動</t>
         </is>
       </c>
-      <c r="C31" s="11" t="n"/>
-      <c r="D31" s="23" t="inlineStr">
+      <c r="C31" s="12" t="n"/>
+      <c r="D31" s="25" t="inlineStr">
         <is>
           <t xml:space="preserve">  業界最大手。補償・サービスの充実度が高い</t>
         </is>
       </c>
-      <c r="E31" s="11" t="n"/>
+      <c r="E31" s="12" t="n"/>
       <c r="F31" s="56" t="inlineStr">
         <is>
           <t xml:space="preserve">  手厚い補償を重視するお客様に有効</t>
         </is>
       </c>
-      <c r="G31" s="11" t="n"/>
+      <c r="G31" s="12" t="n"/>
       <c r="H31" s="61" t="n"/>
     </row>
     <row r="32" hidden="1" outlineLevel="1" ht="18" customHeight="1">
@@ -1716,13 +1718,13 @@
     </row>
     <row r="33" hidden="1" outlineLevel="1" ht="18" customHeight="1">
       <c r="A33" s="3" t="n"/>
-      <c r="B33" s="29" t="n"/>
-      <c r="C33" s="30" t="n"/>
-      <c r="D33" s="30" t="n"/>
-      <c r="E33" s="30" t="n"/>
-      <c r="F33" s="30" t="n"/>
-      <c r="G33" s="30" t="n"/>
-      <c r="H33" s="31" t="n"/>
+      <c r="B33" s="65" t="n"/>
+      <c r="C33" s="66" t="n"/>
+      <c r="D33" s="66" t="n"/>
+      <c r="E33" s="66" t="n"/>
+      <c r="F33" s="66" t="n"/>
+      <c r="G33" s="66" t="n"/>
+      <c r="H33" s="67" t="n"/>
     </row>
     <row r="34" hidden="1" outlineLevel="1" ht="5" customHeight="1">
       <c r="A34" s="3" t="n"/>
@@ -1746,7 +1748,7 @@
     </row>
     <row r="36" hidden="1" outlineLevel="1" ht="22" customHeight="1">
       <c r="A36" s="3" t="n"/>
-      <c r="B36" s="65" t="inlineStr">
+      <c r="B36" s="68" t="inlineStr">
         <is>
           <t xml:space="preserve">  STEP 2　　ソニー損保ご案内　　通販型をご希望の方</t>
         </is>
@@ -1760,80 +1762,80 @@
     </row>
     <row r="37" hidden="1" outlineLevel="1" ht="18" customHeight="1">
       <c r="A37" s="3" t="n"/>
-      <c r="B37" s="66" t="inlineStr">
+      <c r="B37" s="69" t="inlineStr">
         <is>
           <t>📋 スクリプト</t>
         </is>
       </c>
-      <c r="C37" s="11" t="n"/>
-      <c r="D37" s="67" t="inlineStr"/>
-      <c r="E37" s="11" t="n"/>
-      <c r="F37" s="11" t="n"/>
-      <c r="G37" s="11" t="n"/>
-      <c r="H37" s="13" t="n"/>
+      <c r="C37" s="12" t="n"/>
+      <c r="D37" s="70" t="inlineStr"/>
+      <c r="E37" s="12" t="n"/>
+      <c r="F37" s="12" t="n"/>
+      <c r="G37" s="12" t="n"/>
+      <c r="H37" s="14" t="n"/>
     </row>
     <row r="38" hidden="1" outlineLevel="1" ht="65" customHeight="1">
       <c r="A38" s="3" t="n"/>
-      <c r="B38" s="68" t="inlineStr">
+      <c r="B38" s="71" t="inlineStr">
         <is>
           <t>📣 読み上げ①</t>
         </is>
       </c>
-      <c r="C38" s="11" t="n"/>
-      <c r="D38" s="69" t="inlineStr">
+      <c r="C38" s="12" t="n"/>
+      <c r="D38" s="72" t="inlineStr">
         <is>
           <t>「それではソニー損保をご案内しますので、お客様のご状況を確認させてください。
 ソニー損保はインターネットでお客様ご自身に直接ご契約いただく通販型です。手続きはお客様側のご対応となりますが、よろしいでしょうか？」</t>
         </is>
       </c>
-      <c r="E38" s="11" t="n"/>
-      <c r="F38" s="11" t="n"/>
-      <c r="G38" s="11" t="n"/>
-      <c r="H38" s="13" t="n"/>
+      <c r="E38" s="12" t="n"/>
+      <c r="F38" s="12" t="n"/>
+      <c r="G38" s="12" t="n"/>
+      <c r="H38" s="14" t="n"/>
     </row>
     <row r="39" hidden="1" outlineLevel="1" ht="65" customHeight="1">
       <c r="A39" s="3" t="n"/>
-      <c r="B39" s="68" t="inlineStr">
+      <c r="B39" s="71" t="inlineStr">
         <is>
           <t>📣 読み上げ②
 （留意点）</t>
         </is>
       </c>
-      <c r="C39" s="11" t="n"/>
-      <c r="D39" s="69" t="inlineStr">
+      <c r="C39" s="12" t="n"/>
+      <c r="D39" s="72" t="inlineStr">
         <is>
           <t>「保険料面ではメリットが出る場合もありますが、事故時のサポートはコールセンター対応が基本となります。
 当社担当者が直接サポートすることは難しくなりますが、それでもよろしいでしょうか？
 ご希望でしたら、ソニー損保のサイトをご一緒に確認しながら手続きをご案内します。」</t>
         </is>
       </c>
-      <c r="E39" s="11" t="n"/>
-      <c r="F39" s="11" t="n"/>
-      <c r="G39" s="11" t="n"/>
-      <c r="H39" s="13" t="n"/>
+      <c r="E39" s="12" t="n"/>
+      <c r="F39" s="12" t="n"/>
+      <c r="G39" s="12" t="n"/>
+      <c r="H39" s="14" t="n"/>
     </row>
     <row r="40" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A40" s="3" t="n"/>
-      <c r="B40" s="66" t="inlineStr">
+      <c r="B40" s="69" t="inlineStr">
         <is>
           <t>✏️ お客様の意向</t>
         </is>
       </c>
-      <c r="C40" s="11" t="n"/>
-      <c r="D40" s="70" t="inlineStr">
+      <c r="C40" s="12" t="n"/>
+      <c r="D40" s="73" t="inlineStr">
         <is>
           <t>ソニー損保で進める</t>
         </is>
       </c>
-      <c r="E40" s="11" t="n"/>
-      <c r="F40" s="11" t="n"/>
-      <c r="G40" s="11" t="n"/>
+      <c r="E40" s="12" t="n"/>
+      <c r="F40" s="12" t="n"/>
+      <c r="G40" s="12" t="n"/>
       <c r="H40" s="57" t="n"/>
     </row>
     <row r="41" hidden="1" outlineLevel="1" ht="18" customHeight="1">
       <c r="A41" s="3" t="n"/>
-      <c r="B41" s="71" t="inlineStr"/>
-      <c r="C41" s="11" t="n"/>
+      <c r="B41" s="74" t="inlineStr"/>
+      <c r="C41" s="12" t="n"/>
       <c r="D41" s="63" t="n"/>
       <c r="E41" s="63" t="n"/>
       <c r="F41" s="63" t="n"/>
@@ -1842,13 +1844,13 @@
     </row>
     <row r="42" hidden="1" outlineLevel="1" ht="18" customHeight="1">
       <c r="A42" s="3" t="n"/>
-      <c r="B42" s="72" t="inlineStr"/>
-      <c r="C42" s="47" t="n"/>
-      <c r="D42" s="30" t="n"/>
-      <c r="E42" s="30" t="n"/>
-      <c r="F42" s="30" t="n"/>
-      <c r="G42" s="30" t="n"/>
-      <c r="H42" s="31" t="n"/>
+      <c r="B42" s="75" t="inlineStr"/>
+      <c r="C42" s="30" t="n"/>
+      <c r="D42" s="66" t="n"/>
+      <c r="E42" s="66" t="n"/>
+      <c r="F42" s="66" t="n"/>
+      <c r="G42" s="66" t="n"/>
+      <c r="H42" s="67" t="n"/>
     </row>
     <row r="43" hidden="1" outlineLevel="1" ht="5" customHeight="1">
       <c r="A43" s="3" t="n"/>
@@ -1882,7 +1884,7 @@
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="3" t="n"/>
-      <c r="B46" s="73" t="inlineStr">
+      <c r="B46" s="76" t="inlineStr">
         <is>
           <t xml:space="preserve">  📝 面談メモ・お客様の声</t>
         </is>
@@ -1896,13 +1898,13 @@
     </row>
     <row r="47" ht="80" customHeight="1">
       <c r="A47" s="3" t="n"/>
-      <c r="B47" s="74" t="n"/>
-      <c r="C47" s="11" t="n"/>
-      <c r="D47" s="11" t="n"/>
-      <c r="E47" s="11" t="n"/>
-      <c r="F47" s="11" t="n"/>
-      <c r="G47" s="11" t="n"/>
-      <c r="H47" s="13" t="n"/>
+      <c r="B47" s="77" t="n"/>
+      <c r="C47" s="12" t="n"/>
+      <c r="D47" s="12" t="n"/>
+      <c r="E47" s="12" t="n"/>
+      <c r="F47" s="12" t="n"/>
+      <c r="G47" s="12" t="n"/>
+      <c r="H47" s="14" t="n"/>
     </row>
     <row r="48" ht="5" customHeight="1">
       <c r="A48" s="3" t="n"/>
@@ -1916,27 +1918,27 @@
     </row>
     <row r="49" ht="20" customHeight="1">
       <c r="A49" s="3" t="n"/>
-      <c r="B49" s="75" t="inlineStr">
+      <c r="B49" s="78" t="inlineStr">
         <is>
           <t xml:space="preserve">  📌 次回アクション</t>
         </is>
       </c>
-      <c r="C49" s="11" t="n"/>
-      <c r="D49" s="11" t="n"/>
-      <c r="E49" s="11" t="n"/>
-      <c r="F49" s="11" t="n"/>
-      <c r="G49" s="11" t="n"/>
-      <c r="H49" s="13" t="n"/>
+      <c r="C49" s="12" t="n"/>
+      <c r="D49" s="12" t="n"/>
+      <c r="E49" s="12" t="n"/>
+      <c r="F49" s="12" t="n"/>
+      <c r="G49" s="12" t="n"/>
+      <c r="H49" s="14" t="n"/>
     </row>
     <row r="50" ht="30" customHeight="1">
       <c r="A50" s="3" t="n"/>
-      <c r="B50" s="76" t="n"/>
-      <c r="C50" s="47" t="n"/>
-      <c r="D50" s="47" t="n"/>
-      <c r="E50" s="47" t="n"/>
-      <c r="F50" s="47" t="n"/>
-      <c r="G50" s="47" t="n"/>
-      <c r="H50" s="77" t="n"/>
+      <c r="B50" s="79" t="n"/>
+      <c r="C50" s="30" t="n"/>
+      <c r="D50" s="30" t="n"/>
+      <c r="E50" s="30" t="n"/>
+      <c r="F50" s="30" t="n"/>
+      <c r="G50" s="30" t="n"/>
+      <c r="H50" s="80" t="n"/>
     </row>
     <row r="51" ht="5" customHeight="1">
       <c r="A51" s="3" t="n"/>
@@ -1950,7 +1952,7 @@
     </row>
     <row r="52" ht="16" customHeight="1">
       <c r="A52" s="3" t="n"/>
-      <c r="B52" s="78" t="inlineStr">
+      <c r="B52" s="81" t="inlineStr">
         <is>
           <t xml:space="preserve">  ＊本シートは比較推奨規制対応の意向確認記録として活用してください。面談後は保存・アーカイブをお願いします。</t>
         </is>
@@ -2727,9 +2729,9 @@
       <c r="H129" s="3" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="61">
+  <mergeCells count="63">
     <mergeCell ref="F20:H20"/>
-    <mergeCell ref="D9:G9"/>
+    <mergeCell ref="B7:F7"/>
     <mergeCell ref="C20:E20"/>
     <mergeCell ref="F21:H21"/>
     <mergeCell ref="F29:G29"/>
@@ -2757,7 +2759,6 @@
     <mergeCell ref="B47:H47"/>
     <mergeCell ref="B16:H16"/>
     <mergeCell ref="B17:C17"/>
-    <mergeCell ref="D10:G10"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="D17:H17"/>
     <mergeCell ref="B46:H46"/>
@@ -2765,8 +2766,9 @@
     <mergeCell ref="B38:C38"/>
     <mergeCell ref="B29:C29"/>
     <mergeCell ref="B52:H52"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="A2:H2"/>
     <mergeCell ref="B19:C19"/>
-    <mergeCell ref="A2:H2"/>
     <mergeCell ref="B37:C37"/>
     <mergeCell ref="B28:C28"/>
     <mergeCell ref="F31:G31"/>
@@ -2774,10 +2776,12 @@
     <mergeCell ref="D37:H37"/>
     <mergeCell ref="F28:G28"/>
     <mergeCell ref="D11:G11"/>
+    <mergeCell ref="D13:G13"/>
+    <mergeCell ref="B9:C9"/>
     <mergeCell ref="B40:C40"/>
-    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="G10"/>
     <mergeCell ref="D18:H18"/>
-    <mergeCell ref="B7:G7"/>
+    <mergeCell ref="D9:H9"/>
     <mergeCell ref="C24:E24"/>
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="D8:H8"/>
@@ -2791,7 +2795,7 @@
     <mergeCell ref="F24:H24"/>
   </mergeCells>
   <dataValidations count="4">
-    <dataValidation sqref="H7" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="STEP1 選択" prompt="契約方法を選択してください" type="list">
+    <dataValidation sqref="H7 H10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"①給与天引き（団体割引）,②一般契約（クレカ・口振）,③通販型（ソニー損保）"</formula1>
     </dataValidation>
     <dataValidation sqref="H20 H21 H22 H23 H24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
@@ -2841,619 +2845,619 @@
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="79" t="n"/>
-      <c r="B3" s="79" t="n"/>
-      <c r="C3" s="80" t="inlineStr">
+      <c r="A3" s="82" t="n"/>
+      <c r="B3" s="82" t="n"/>
+      <c r="C3" s="83" t="inlineStr">
         <is>
           <t xml:space="preserve">  確認項目</t>
         </is>
       </c>
-      <c r="E3" s="81" t="inlineStr">
+      <c r="E3" s="84" t="inlineStr">
         <is>
           <t>SJ</t>
         </is>
       </c>
-      <c r="F3" s="81" t="inlineStr">
+      <c r="F3" s="84" t="inlineStr">
         <is>
           <t>MSI</t>
         </is>
       </c>
-      <c r="G3" s="81" t="inlineStr">
+      <c r="G3" s="84" t="inlineStr">
         <is>
           <t>TN</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="79" t="n"/>
-      <c r="B4" s="82" t="inlineStr">
+      <c r="A4" s="82" t="n"/>
+      <c r="B4" s="85" t="inlineStr">
         <is>
           <t xml:space="preserve">  【 事前確認 】</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="79" t="n"/>
-      <c r="B5" s="83" t="inlineStr">
+      <c r="A5" s="82" t="n"/>
+      <c r="B5" s="86" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C5" s="84" t="inlineStr">
+      <c r="C5" s="87" t="inlineStr">
         <is>
           <t xml:space="preserve">  お客様の意向（重視事項）を確認した</t>
         </is>
       </c>
-      <c r="E5" s="85" t="n"/>
-      <c r="F5" s="86" t="n"/>
-      <c r="G5" s="86" t="n"/>
+      <c r="E5" s="88" t="n"/>
+      <c r="F5" s="89" t="n"/>
+      <c r="G5" s="89" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="79" t="n"/>
-      <c r="B6" s="83" t="inlineStr">
+      <c r="A6" s="82" t="n"/>
+      <c r="B6" s="86" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C6" s="84" t="inlineStr">
+      <c r="C6" s="87" t="inlineStr">
         <is>
           <t xml:space="preserve">  複数社（原則3社）の見積りを取得した</t>
         </is>
       </c>
-      <c r="E6" s="85" t="n"/>
-      <c r="F6" s="86" t="n"/>
-      <c r="G6" s="86" t="n"/>
+      <c r="E6" s="88" t="n"/>
+      <c r="F6" s="89" t="n"/>
+      <c r="G6" s="89" t="n"/>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="79" t="n"/>
-      <c r="B7" s="83" t="inlineStr">
+      <c r="A7" s="82" t="n"/>
+      <c r="B7" s="86" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C7" s="84" t="inlineStr">
+      <c r="C7" s="87" t="inlineStr">
         <is>
           <t xml:space="preserve">  各社の保険料・補償内容を比較説明した</t>
         </is>
       </c>
-      <c r="E7" s="85" t="n"/>
-      <c r="F7" s="86" t="n"/>
-      <c r="G7" s="86" t="n"/>
+      <c r="E7" s="88" t="n"/>
+      <c r="F7" s="89" t="n"/>
+      <c r="G7" s="89" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="79" t="n"/>
-      <c r="B8" s="83" t="inlineStr">
+      <c r="A8" s="82" t="n"/>
+      <c r="B8" s="86" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C8" s="84" t="inlineStr">
+      <c r="C8" s="87" t="inlineStr">
         <is>
           <t xml:space="preserve">  比較に用いた基準・理由を説明できる</t>
         </is>
       </c>
-      <c r="E8" s="85" t="n"/>
-      <c r="F8" s="86" t="n"/>
-      <c r="G8" s="86" t="n"/>
+      <c r="E8" s="88" t="n"/>
+      <c r="F8" s="89" t="n"/>
+      <c r="G8" s="89" t="n"/>
     </row>
     <row r="9" ht="4" customHeight="1">
-      <c r="A9" s="79" t="n"/>
-      <c r="B9" s="79" t="n"/>
-      <c r="C9" s="79" t="n"/>
-      <c r="D9" s="79" t="n"/>
-      <c r="E9" s="79" t="n"/>
-      <c r="F9" s="79" t="n"/>
-      <c r="G9" s="79" t="n"/>
+      <c r="A9" s="82" t="n"/>
+      <c r="B9" s="82" t="n"/>
+      <c r="C9" s="82" t="n"/>
+      <c r="D9" s="82" t="n"/>
+      <c r="E9" s="82" t="n"/>
+      <c r="F9" s="82" t="n"/>
+      <c r="G9" s="82" t="n"/>
     </row>
     <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="79" t="n"/>
-      <c r="B10" s="82" t="inlineStr">
+      <c r="A10" s="82" t="n"/>
+      <c r="B10" s="85" t="inlineStr">
         <is>
           <t xml:space="preserve">  【 三井住友海上の提案 】</t>
         </is>
       </c>
     </row>
     <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="79" t="n"/>
-      <c r="B11" s="87" t="inlineStr">
+      <c r="A11" s="82" t="n"/>
+      <c r="B11" s="90" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C11" s="84" t="inlineStr">
+      <c r="C11" s="87" t="inlineStr">
         <is>
           <t xml:space="preserve">  三井住友海上の見積りを必ず含めた</t>
         </is>
       </c>
-      <c r="E11" s="88" t="n"/>
-      <c r="F11" s="86" t="n"/>
-      <c r="G11" s="86" t="n"/>
+      <c r="E11" s="91" t="n"/>
+      <c r="F11" s="89" t="n"/>
+      <c r="G11" s="89" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="79" t="n"/>
-      <c r="B12" s="87" t="inlineStr">
+      <c r="A12" s="82" t="n"/>
+      <c r="B12" s="90" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C12" s="84" t="inlineStr">
+      <c r="C12" s="87" t="inlineStr">
         <is>
           <t xml:space="preserve">  損保ジャパンとの比較ポイントを説明した</t>
         </is>
       </c>
-      <c r="E12" s="88" t="n"/>
-      <c r="F12" s="86" t="n"/>
-      <c r="G12" s="86" t="n"/>
+      <c r="E12" s="91" t="n"/>
+      <c r="F12" s="89" t="n"/>
+      <c r="G12" s="89" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="79" t="n"/>
-      <c r="B13" s="87" t="inlineStr">
+      <c r="A13" s="82" t="n"/>
+      <c r="B13" s="90" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C13" s="84" t="inlineStr">
+      <c r="C13" s="87" t="inlineStr">
         <is>
           <t xml:space="preserve">  MSIを選ばない場合、理由を記録した</t>
         </is>
       </c>
-      <c r="E13" s="88" t="n"/>
-      <c r="F13" s="86" t="n"/>
-      <c r="G13" s="86" t="n"/>
+      <c r="E13" s="91" t="n"/>
+      <c r="F13" s="89" t="n"/>
+      <c r="G13" s="89" t="n"/>
     </row>
     <row r="14" ht="4" customHeight="1">
-      <c r="A14" s="79" t="n"/>
-      <c r="B14" s="79" t="n"/>
-      <c r="C14" s="79" t="n"/>
-      <c r="D14" s="79" t="n"/>
-      <c r="E14" s="79" t="n"/>
-      <c r="F14" s="79" t="n"/>
-      <c r="G14" s="79" t="n"/>
+      <c r="A14" s="82" t="n"/>
+      <c r="B14" s="82" t="n"/>
+      <c r="C14" s="82" t="n"/>
+      <c r="D14" s="82" t="n"/>
+      <c r="E14" s="82" t="n"/>
+      <c r="F14" s="82" t="n"/>
+      <c r="G14" s="82" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="79" t="n"/>
-      <c r="B15" s="82" t="inlineStr">
+      <c r="A15" s="82" t="n"/>
+      <c r="B15" s="85" t="inlineStr">
         <is>
           <t xml:space="preserve">  【 推奨根拠の記録 】</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="79" t="n"/>
-      <c r="B16" s="89" t="inlineStr">
+      <c r="A16" s="82" t="n"/>
+      <c r="B16" s="92" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C16" s="84" t="inlineStr">
+      <c r="C16" s="87" t="inlineStr">
         <is>
           <t xml:space="preserve">  推奨する会社・商品とその理由を記録した</t>
         </is>
       </c>
-      <c r="E16" s="90" t="n"/>
-      <c r="F16" s="86" t="n"/>
-      <c r="G16" s="86" t="n"/>
+      <c r="E16" s="93" t="n"/>
+      <c r="F16" s="89" t="n"/>
+      <c r="G16" s="89" t="n"/>
     </row>
     <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="79" t="n"/>
-      <c r="B17" s="89" t="inlineStr">
+      <c r="A17" s="82" t="n"/>
+      <c r="B17" s="92" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C17" s="84" t="inlineStr">
+      <c r="C17" s="87" t="inlineStr">
         <is>
           <t xml:space="preserve">  お客様が選んだ会社・商品を記録した</t>
         </is>
       </c>
-      <c r="E17" s="90" t="n"/>
-      <c r="F17" s="86" t="n"/>
-      <c r="G17" s="86" t="n"/>
+      <c r="E17" s="93" t="n"/>
+      <c r="F17" s="89" t="n"/>
+      <c r="G17" s="89" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="79" t="n"/>
-      <c r="B18" s="89" t="inlineStr">
+      <c r="A18" s="82" t="n"/>
+      <c r="B18" s="92" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C18" s="84" t="inlineStr">
+      <c r="C18" s="87" t="inlineStr">
         <is>
           <t xml:space="preserve">  意向と選択が異なる場合、経緯を記録した</t>
         </is>
       </c>
-      <c r="E18" s="90" t="n"/>
-      <c r="F18" s="86" t="n"/>
-      <c r="G18" s="86" t="n"/>
+      <c r="E18" s="93" t="n"/>
+      <c r="F18" s="89" t="n"/>
+      <c r="G18" s="89" t="n"/>
     </row>
     <row r="19" ht="4" customHeight="1">
-      <c r="A19" s="79" t="n"/>
-      <c r="B19" s="79" t="n"/>
-      <c r="C19" s="79" t="n"/>
-      <c r="D19" s="79" t="n"/>
-      <c r="E19" s="79" t="n"/>
-      <c r="F19" s="79" t="n"/>
-      <c r="G19" s="79" t="n"/>
+      <c r="A19" s="82" t="n"/>
+      <c r="B19" s="82" t="n"/>
+      <c r="C19" s="82" t="n"/>
+      <c r="D19" s="82" t="n"/>
+      <c r="E19" s="82" t="n"/>
+      <c r="F19" s="82" t="n"/>
+      <c r="G19" s="82" t="n"/>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="79" t="n"/>
-      <c r="B20" s="82" t="inlineStr">
+      <c r="A20" s="82" t="n"/>
+      <c r="B20" s="85" t="inlineStr">
         <is>
           <t xml:space="preserve">  【 コンプライアンス 】</t>
         </is>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="79" t="n"/>
-      <c r="B21" s="91" t="inlineStr">
+      <c r="A21" s="82" t="n"/>
+      <c r="B21" s="94" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C21" s="84" t="inlineStr">
+      <c r="C21" s="87" t="inlineStr">
         <is>
           <t xml:space="preserve">  特定会社への誘導はない</t>
         </is>
       </c>
-      <c r="E21" s="92" t="n"/>
-      <c r="F21" s="86" t="n"/>
-      <c r="G21" s="86" t="n"/>
+      <c r="E21" s="95" t="n"/>
+      <c r="F21" s="89" t="n"/>
+      <c r="G21" s="89" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="79" t="n"/>
-      <c r="B22" s="91" t="inlineStr">
+      <c r="A22" s="82" t="n"/>
+      <c r="B22" s="94" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C22" s="84" t="inlineStr">
+      <c r="C22" s="87" t="inlineStr">
         <is>
           <t xml:space="preserve">  意向確認の同意を得た</t>
         </is>
       </c>
-      <c r="E22" s="92" t="n"/>
-      <c r="F22" s="86" t="n"/>
-      <c r="G22" s="86" t="n"/>
+      <c r="E22" s="95" t="n"/>
+      <c r="F22" s="89" t="n"/>
+      <c r="G22" s="89" t="n"/>
     </row>
     <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="79" t="n"/>
-      <c r="B23" s="91" t="inlineStr">
+      <c r="A23" s="82" t="n"/>
+      <c r="B23" s="94" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C23" s="84" t="inlineStr">
+      <c r="C23" s="87" t="inlineStr">
         <is>
           <t xml:space="preserve">  本シートを保管・アーカイブ予定</t>
         </is>
       </c>
-      <c r="E23" s="92" t="n"/>
-      <c r="F23" s="86" t="n"/>
-      <c r="G23" s="86" t="n"/>
+      <c r="E23" s="95" t="n"/>
+      <c r="F23" s="89" t="n"/>
+      <c r="G23" s="89" t="n"/>
     </row>
     <row r="24" ht="4" customHeight="1">
-      <c r="A24" s="79" t="n"/>
-      <c r="B24" s="79" t="n"/>
-      <c r="C24" s="79" t="n"/>
-      <c r="D24" s="79" t="n"/>
-      <c r="E24" s="79" t="n"/>
-      <c r="F24" s="79" t="n"/>
-      <c r="G24" s="79" t="n"/>
+      <c r="A24" s="82" t="n"/>
+      <c r="B24" s="82" t="n"/>
+      <c r="C24" s="82" t="n"/>
+      <c r="D24" s="82" t="n"/>
+      <c r="E24" s="82" t="n"/>
+      <c r="F24" s="82" t="n"/>
+      <c r="G24" s="82" t="n"/>
     </row>
     <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="79" t="n"/>
-      <c r="B25" s="79" t="n"/>
-      <c r="C25" s="79" t="n"/>
-      <c r="D25" s="79" t="n"/>
-      <c r="E25" s="79" t="n"/>
-      <c r="F25" s="79" t="n"/>
-      <c r="G25" s="79" t="n"/>
+      <c r="A25" s="82" t="n"/>
+      <c r="B25" s="82" t="n"/>
+      <c r="C25" s="82" t="n"/>
+      <c r="D25" s="82" t="n"/>
+      <c r="E25" s="82" t="n"/>
+      <c r="F25" s="82" t="n"/>
+      <c r="G25" s="82" t="n"/>
     </row>
     <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="79" t="n"/>
-      <c r="B26" s="79" t="n"/>
-      <c r="C26" s="79" t="n"/>
-      <c r="D26" s="79" t="n"/>
-      <c r="E26" s="79" t="n"/>
-      <c r="F26" s="79" t="n"/>
-      <c r="G26" s="79" t="n"/>
+      <c r="A26" s="82" t="n"/>
+      <c r="B26" s="82" t="n"/>
+      <c r="C26" s="82" t="n"/>
+      <c r="D26" s="82" t="n"/>
+      <c r="E26" s="82" t="n"/>
+      <c r="F26" s="82" t="n"/>
+      <c r="G26" s="82" t="n"/>
     </row>
     <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="79" t="n"/>
-      <c r="B27" s="79" t="n"/>
-      <c r="C27" s="79" t="n"/>
-      <c r="D27" s="79" t="n"/>
-      <c r="E27" s="79" t="n"/>
-      <c r="F27" s="79" t="n"/>
-      <c r="G27" s="79" t="n"/>
+      <c r="A27" s="82" t="n"/>
+      <c r="B27" s="82" t="n"/>
+      <c r="C27" s="82" t="n"/>
+      <c r="D27" s="82" t="n"/>
+      <c r="E27" s="82" t="n"/>
+      <c r="F27" s="82" t="n"/>
+      <c r="G27" s="82" t="n"/>
     </row>
     <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="79" t="n"/>
-      <c r="B28" s="79" t="n"/>
-      <c r="C28" s="79" t="n"/>
-      <c r="D28" s="79" t="n"/>
-      <c r="E28" s="79" t="n"/>
-      <c r="F28" s="79" t="n"/>
-      <c r="G28" s="79" t="n"/>
+      <c r="A28" s="82" t="n"/>
+      <c r="B28" s="82" t="n"/>
+      <c r="C28" s="82" t="n"/>
+      <c r="D28" s="82" t="n"/>
+      <c r="E28" s="82" t="n"/>
+      <c r="F28" s="82" t="n"/>
+      <c r="G28" s="82" t="n"/>
     </row>
     <row r="29" ht="16" customHeight="1">
-      <c r="A29" s="79" t="n"/>
-      <c r="B29" s="79" t="n"/>
-      <c r="C29" s="79" t="n"/>
-      <c r="D29" s="79" t="n"/>
-      <c r="E29" s="79" t="n"/>
-      <c r="F29" s="79" t="n"/>
-      <c r="G29" s="79" t="n"/>
+      <c r="A29" s="82" t="n"/>
+      <c r="B29" s="82" t="n"/>
+      <c r="C29" s="82" t="n"/>
+      <c r="D29" s="82" t="n"/>
+      <c r="E29" s="82" t="n"/>
+      <c r="F29" s="82" t="n"/>
+      <c r="G29" s="82" t="n"/>
     </row>
     <row r="30" ht="16" customHeight="1">
-      <c r="A30" s="79" t="n"/>
-      <c r="B30" s="79" t="n"/>
-      <c r="C30" s="79" t="n"/>
-      <c r="D30" s="79" t="n"/>
-      <c r="E30" s="79" t="n"/>
-      <c r="F30" s="79" t="n"/>
-      <c r="G30" s="79" t="n"/>
+      <c r="A30" s="82" t="n"/>
+      <c r="B30" s="82" t="n"/>
+      <c r="C30" s="82" t="n"/>
+      <c r="D30" s="82" t="n"/>
+      <c r="E30" s="82" t="n"/>
+      <c r="F30" s="82" t="n"/>
+      <c r="G30" s="82" t="n"/>
     </row>
     <row r="31" ht="16" customHeight="1">
-      <c r="A31" s="79" t="n"/>
-      <c r="B31" s="79" t="n"/>
-      <c r="C31" s="79" t="n"/>
-      <c r="D31" s="79" t="n"/>
-      <c r="E31" s="79" t="n"/>
-      <c r="F31" s="79" t="n"/>
-      <c r="G31" s="79" t="n"/>
+      <c r="A31" s="82" t="n"/>
+      <c r="B31" s="82" t="n"/>
+      <c r="C31" s="82" t="n"/>
+      <c r="D31" s="82" t="n"/>
+      <c r="E31" s="82" t="n"/>
+      <c r="F31" s="82" t="n"/>
+      <c r="G31" s="82" t="n"/>
     </row>
     <row r="32" ht="16" customHeight="1">
-      <c r="A32" s="79" t="n"/>
-      <c r="B32" s="79" t="n"/>
-      <c r="C32" s="79" t="n"/>
-      <c r="D32" s="79" t="n"/>
-      <c r="E32" s="79" t="n"/>
-      <c r="F32" s="79" t="n"/>
-      <c r="G32" s="79" t="n"/>
+      <c r="A32" s="82" t="n"/>
+      <c r="B32" s="82" t="n"/>
+      <c r="C32" s="82" t="n"/>
+      <c r="D32" s="82" t="n"/>
+      <c r="E32" s="82" t="n"/>
+      <c r="F32" s="82" t="n"/>
+      <c r="G32" s="82" t="n"/>
     </row>
     <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="79" t="n"/>
-      <c r="B33" s="79" t="n"/>
-      <c r="C33" s="79" t="n"/>
-      <c r="D33" s="79" t="n"/>
-      <c r="E33" s="79" t="n"/>
-      <c r="F33" s="79" t="n"/>
-      <c r="G33" s="79" t="n"/>
+      <c r="A33" s="82" t="n"/>
+      <c r="B33" s="82" t="n"/>
+      <c r="C33" s="82" t="n"/>
+      <c r="D33" s="82" t="n"/>
+      <c r="E33" s="82" t="n"/>
+      <c r="F33" s="82" t="n"/>
+      <c r="G33" s="82" t="n"/>
     </row>
     <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="79" t="n"/>
-      <c r="B34" s="79" t="n"/>
-      <c r="C34" s="79" t="n"/>
-      <c r="D34" s="79" t="n"/>
-      <c r="E34" s="79" t="n"/>
-      <c r="F34" s="79" t="n"/>
-      <c r="G34" s="79" t="n"/>
+      <c r="A34" s="82" t="n"/>
+      <c r="B34" s="82" t="n"/>
+      <c r="C34" s="82" t="n"/>
+      <c r="D34" s="82" t="n"/>
+      <c r="E34" s="82" t="n"/>
+      <c r="F34" s="82" t="n"/>
+      <c r="G34" s="82" t="n"/>
     </row>
     <row r="35" ht="16" customHeight="1">
-      <c r="A35" s="79" t="n"/>
-      <c r="B35" s="79" t="n"/>
-      <c r="C35" s="79" t="n"/>
-      <c r="D35" s="79" t="n"/>
-      <c r="E35" s="79" t="n"/>
-      <c r="F35" s="79" t="n"/>
-      <c r="G35" s="79" t="n"/>
+      <c r="A35" s="82" t="n"/>
+      <c r="B35" s="82" t="n"/>
+      <c r="C35" s="82" t="n"/>
+      <c r="D35" s="82" t="n"/>
+      <c r="E35" s="82" t="n"/>
+      <c r="F35" s="82" t="n"/>
+      <c r="G35" s="82" t="n"/>
     </row>
     <row r="36" ht="16" customHeight="1">
-      <c r="A36" s="79" t="n"/>
-      <c r="B36" s="79" t="n"/>
-      <c r="C36" s="79" t="n"/>
-      <c r="D36" s="79" t="n"/>
-      <c r="E36" s="79" t="n"/>
-      <c r="F36" s="79" t="n"/>
-      <c r="G36" s="79" t="n"/>
+      <c r="A36" s="82" t="n"/>
+      <c r="B36" s="82" t="n"/>
+      <c r="C36" s="82" t="n"/>
+      <c r="D36" s="82" t="n"/>
+      <c r="E36" s="82" t="n"/>
+      <c r="F36" s="82" t="n"/>
+      <c r="G36" s="82" t="n"/>
     </row>
     <row r="37" ht="16" customHeight="1">
-      <c r="A37" s="79" t="n"/>
-      <c r="B37" s="79" t="n"/>
-      <c r="C37" s="79" t="n"/>
-      <c r="D37" s="79" t="n"/>
-      <c r="E37" s="79" t="n"/>
-      <c r="F37" s="79" t="n"/>
-      <c r="G37" s="79" t="n"/>
+      <c r="A37" s="82" t="n"/>
+      <c r="B37" s="82" t="n"/>
+      <c r="C37" s="82" t="n"/>
+      <c r="D37" s="82" t="n"/>
+      <c r="E37" s="82" t="n"/>
+      <c r="F37" s="82" t="n"/>
+      <c r="G37" s="82" t="n"/>
     </row>
     <row r="38" ht="16" customHeight="1">
-      <c r="A38" s="79" t="n"/>
-      <c r="B38" s="79" t="n"/>
-      <c r="C38" s="79" t="n"/>
-      <c r="D38" s="79" t="n"/>
-      <c r="E38" s="79" t="n"/>
-      <c r="F38" s="79" t="n"/>
-      <c r="G38" s="79" t="n"/>
+      <c r="A38" s="82" t="n"/>
+      <c r="B38" s="82" t="n"/>
+      <c r="C38" s="82" t="n"/>
+      <c r="D38" s="82" t="n"/>
+      <c r="E38" s="82" t="n"/>
+      <c r="F38" s="82" t="n"/>
+      <c r="G38" s="82" t="n"/>
     </row>
     <row r="39" ht="16" customHeight="1">
-      <c r="A39" s="79" t="n"/>
-      <c r="B39" s="79" t="n"/>
-      <c r="C39" s="79" t="n"/>
-      <c r="D39" s="79" t="n"/>
-      <c r="E39" s="79" t="n"/>
-      <c r="F39" s="79" t="n"/>
-      <c r="G39" s="79" t="n"/>
+      <c r="A39" s="82" t="n"/>
+      <c r="B39" s="82" t="n"/>
+      <c r="C39" s="82" t="n"/>
+      <c r="D39" s="82" t="n"/>
+      <c r="E39" s="82" t="n"/>
+      <c r="F39" s="82" t="n"/>
+      <c r="G39" s="82" t="n"/>
     </row>
     <row r="40" ht="16" customHeight="1">
-      <c r="A40" s="79" t="n"/>
-      <c r="B40" s="79" t="n"/>
-      <c r="C40" s="79" t="n"/>
-      <c r="D40" s="79" t="n"/>
-      <c r="E40" s="79" t="n"/>
-      <c r="F40" s="79" t="n"/>
-      <c r="G40" s="79" t="n"/>
+      <c r="A40" s="82" t="n"/>
+      <c r="B40" s="82" t="n"/>
+      <c r="C40" s="82" t="n"/>
+      <c r="D40" s="82" t="n"/>
+      <c r="E40" s="82" t="n"/>
+      <c r="F40" s="82" t="n"/>
+      <c r="G40" s="82" t="n"/>
     </row>
     <row r="41" ht="16" customHeight="1">
-      <c r="A41" s="79" t="n"/>
-      <c r="B41" s="79" t="n"/>
-      <c r="C41" s="79" t="n"/>
-      <c r="D41" s="79" t="n"/>
-      <c r="E41" s="79" t="n"/>
-      <c r="F41" s="79" t="n"/>
-      <c r="G41" s="79" t="n"/>
+      <c r="A41" s="82" t="n"/>
+      <c r="B41" s="82" t="n"/>
+      <c r="C41" s="82" t="n"/>
+      <c r="D41" s="82" t="n"/>
+      <c r="E41" s="82" t="n"/>
+      <c r="F41" s="82" t="n"/>
+      <c r="G41" s="82" t="n"/>
     </row>
     <row r="42" ht="16" customHeight="1">
-      <c r="A42" s="79" t="n"/>
-      <c r="B42" s="79" t="n"/>
-      <c r="C42" s="79" t="n"/>
-      <c r="D42" s="79" t="n"/>
-      <c r="E42" s="79" t="n"/>
-      <c r="F42" s="79" t="n"/>
-      <c r="G42" s="79" t="n"/>
+      <c r="A42" s="82" t="n"/>
+      <c r="B42" s="82" t="n"/>
+      <c r="C42" s="82" t="n"/>
+      <c r="D42" s="82" t="n"/>
+      <c r="E42" s="82" t="n"/>
+      <c r="F42" s="82" t="n"/>
+      <c r="G42" s="82" t="n"/>
     </row>
     <row r="43" ht="16" customHeight="1">
-      <c r="A43" s="79" t="n"/>
-      <c r="B43" s="79" t="n"/>
-      <c r="C43" s="79" t="n"/>
-      <c r="D43" s="79" t="n"/>
-      <c r="E43" s="79" t="n"/>
-      <c r="F43" s="79" t="n"/>
-      <c r="G43" s="79" t="n"/>
+      <c r="A43" s="82" t="n"/>
+      <c r="B43" s="82" t="n"/>
+      <c r="C43" s="82" t="n"/>
+      <c r="D43" s="82" t="n"/>
+      <c r="E43" s="82" t="n"/>
+      <c r="F43" s="82" t="n"/>
+      <c r="G43" s="82" t="n"/>
     </row>
     <row r="44" ht="16" customHeight="1">
-      <c r="A44" s="79" t="n"/>
-      <c r="B44" s="79" t="n"/>
-      <c r="C44" s="79" t="n"/>
-      <c r="D44" s="79" t="n"/>
-      <c r="E44" s="79" t="n"/>
-      <c r="F44" s="79" t="n"/>
-      <c r="G44" s="79" t="n"/>
+      <c r="A44" s="82" t="n"/>
+      <c r="B44" s="82" t="n"/>
+      <c r="C44" s="82" t="n"/>
+      <c r="D44" s="82" t="n"/>
+      <c r="E44" s="82" t="n"/>
+      <c r="F44" s="82" t="n"/>
+      <c r="G44" s="82" t="n"/>
     </row>
     <row r="45" ht="16" customHeight="1">
-      <c r="A45" s="79" t="n"/>
-      <c r="B45" s="79" t="n"/>
-      <c r="C45" s="79" t="n"/>
-      <c r="D45" s="79" t="n"/>
-      <c r="E45" s="79" t="n"/>
-      <c r="F45" s="79" t="n"/>
-      <c r="G45" s="79" t="n"/>
+      <c r="A45" s="82" t="n"/>
+      <c r="B45" s="82" t="n"/>
+      <c r="C45" s="82" t="n"/>
+      <c r="D45" s="82" t="n"/>
+      <c r="E45" s="82" t="n"/>
+      <c r="F45" s="82" t="n"/>
+      <c r="G45" s="82" t="n"/>
     </row>
     <row r="46" ht="16" customHeight="1">
-      <c r="A46" s="79" t="n"/>
-      <c r="B46" s="79" t="n"/>
-      <c r="C46" s="79" t="n"/>
-      <c r="D46" s="79" t="n"/>
-      <c r="E46" s="79" t="n"/>
-      <c r="F46" s="79" t="n"/>
-      <c r="G46" s="79" t="n"/>
+      <c r="A46" s="82" t="n"/>
+      <c r="B46" s="82" t="n"/>
+      <c r="C46" s="82" t="n"/>
+      <c r="D46" s="82" t="n"/>
+      <c r="E46" s="82" t="n"/>
+      <c r="F46" s="82" t="n"/>
+      <c r="G46" s="82" t="n"/>
     </row>
     <row r="47" ht="16" customHeight="1">
-      <c r="A47" s="79" t="n"/>
-      <c r="B47" s="79" t="n"/>
-      <c r="C47" s="79" t="n"/>
-      <c r="D47" s="79" t="n"/>
-      <c r="E47" s="79" t="n"/>
-      <c r="F47" s="79" t="n"/>
-      <c r="G47" s="79" t="n"/>
+      <c r="A47" s="82" t="n"/>
+      <c r="B47" s="82" t="n"/>
+      <c r="C47" s="82" t="n"/>
+      <c r="D47" s="82" t="n"/>
+      <c r="E47" s="82" t="n"/>
+      <c r="F47" s="82" t="n"/>
+      <c r="G47" s="82" t="n"/>
     </row>
     <row r="48" ht="16" customHeight="1">
-      <c r="A48" s="79" t="n"/>
-      <c r="B48" s="79" t="n"/>
-      <c r="C48" s="79" t="n"/>
-      <c r="D48" s="79" t="n"/>
-      <c r="E48" s="79" t="n"/>
-      <c r="F48" s="79" t="n"/>
-      <c r="G48" s="79" t="n"/>
+      <c r="A48" s="82" t="n"/>
+      <c r="B48" s="82" t="n"/>
+      <c r="C48" s="82" t="n"/>
+      <c r="D48" s="82" t="n"/>
+      <c r="E48" s="82" t="n"/>
+      <c r="F48" s="82" t="n"/>
+      <c r="G48" s="82" t="n"/>
     </row>
     <row r="49" ht="16" customHeight="1">
-      <c r="A49" s="79" t="n"/>
-      <c r="B49" s="79" t="n"/>
-      <c r="C49" s="79" t="n"/>
-      <c r="D49" s="79" t="n"/>
-      <c r="E49" s="79" t="n"/>
-      <c r="F49" s="79" t="n"/>
-      <c r="G49" s="79" t="n"/>
+      <c r="A49" s="82" t="n"/>
+      <c r="B49" s="82" t="n"/>
+      <c r="C49" s="82" t="n"/>
+      <c r="D49" s="82" t="n"/>
+      <c r="E49" s="82" t="n"/>
+      <c r="F49" s="82" t="n"/>
+      <c r="G49" s="82" t="n"/>
     </row>
     <row r="50" ht="16" customHeight="1">
-      <c r="A50" s="79" t="n"/>
-      <c r="B50" s="79" t="n"/>
-      <c r="C50" s="79" t="n"/>
-      <c r="D50" s="79" t="n"/>
-      <c r="E50" s="79" t="n"/>
-      <c r="F50" s="79" t="n"/>
-      <c r="G50" s="79" t="n"/>
+      <c r="A50" s="82" t="n"/>
+      <c r="B50" s="82" t="n"/>
+      <c r="C50" s="82" t="n"/>
+      <c r="D50" s="82" t="n"/>
+      <c r="E50" s="82" t="n"/>
+      <c r="F50" s="82" t="n"/>
+      <c r="G50" s="82" t="n"/>
     </row>
     <row r="51" ht="16" customHeight="1">
-      <c r="A51" s="79" t="n"/>
-      <c r="B51" s="79" t="n"/>
-      <c r="C51" s="79" t="n"/>
-      <c r="D51" s="79" t="n"/>
-      <c r="E51" s="79" t="n"/>
-      <c r="F51" s="79" t="n"/>
-      <c r="G51" s="79" t="n"/>
+      <c r="A51" s="82" t="n"/>
+      <c r="B51" s="82" t="n"/>
+      <c r="C51" s="82" t="n"/>
+      <c r="D51" s="82" t="n"/>
+      <c r="E51" s="82" t="n"/>
+      <c r="F51" s="82" t="n"/>
+      <c r="G51" s="82" t="n"/>
     </row>
     <row r="52" ht="16" customHeight="1">
-      <c r="A52" s="79" t="n"/>
-      <c r="B52" s="79" t="n"/>
-      <c r="C52" s="79" t="n"/>
-      <c r="D52" s="79" t="n"/>
-      <c r="E52" s="79" t="n"/>
-      <c r="F52" s="79" t="n"/>
-      <c r="G52" s="79" t="n"/>
+      <c r="A52" s="82" t="n"/>
+      <c r="B52" s="82" t="n"/>
+      <c r="C52" s="82" t="n"/>
+      <c r="D52" s="82" t="n"/>
+      <c r="E52" s="82" t="n"/>
+      <c r="F52" s="82" t="n"/>
+      <c r="G52" s="82" t="n"/>
     </row>
     <row r="53" ht="16" customHeight="1">
-      <c r="A53" s="79" t="n"/>
-      <c r="B53" s="79" t="n"/>
-      <c r="C53" s="79" t="n"/>
-      <c r="D53" s="79" t="n"/>
-      <c r="E53" s="79" t="n"/>
-      <c r="F53" s="79" t="n"/>
-      <c r="G53" s="79" t="n"/>
+      <c r="A53" s="82" t="n"/>
+      <c r="B53" s="82" t="n"/>
+      <c r="C53" s="82" t="n"/>
+      <c r="D53" s="82" t="n"/>
+      <c r="E53" s="82" t="n"/>
+      <c r="F53" s="82" t="n"/>
+      <c r="G53" s="82" t="n"/>
     </row>
     <row r="54" ht="16" customHeight="1">
-      <c r="A54" s="79" t="n"/>
-      <c r="B54" s="79" t="n"/>
-      <c r="C54" s="79" t="n"/>
-      <c r="D54" s="79" t="n"/>
-      <c r="E54" s="79" t="n"/>
-      <c r="F54" s="79" t="n"/>
-      <c r="G54" s="79" t="n"/>
+      <c r="A54" s="82" t="n"/>
+      <c r="B54" s="82" t="n"/>
+      <c r="C54" s="82" t="n"/>
+      <c r="D54" s="82" t="n"/>
+      <c r="E54" s="82" t="n"/>
+      <c r="F54" s="82" t="n"/>
+      <c r="G54" s="82" t="n"/>
     </row>
     <row r="55" ht="16" customHeight="1">
-      <c r="A55" s="79" t="n"/>
-      <c r="B55" s="79" t="n"/>
-      <c r="C55" s="79" t="n"/>
-      <c r="D55" s="79" t="n"/>
-      <c r="E55" s="79" t="n"/>
-      <c r="F55" s="79" t="n"/>
-      <c r="G55" s="79" t="n"/>
+      <c r="A55" s="82" t="n"/>
+      <c r="B55" s="82" t="n"/>
+      <c r="C55" s="82" t="n"/>
+      <c r="D55" s="82" t="n"/>
+      <c r="E55" s="82" t="n"/>
+      <c r="F55" s="82" t="n"/>
+      <c r="G55" s="82" t="n"/>
     </row>
     <row r="56" ht="16" customHeight="1">
-      <c r="A56" s="79" t="n"/>
-      <c r="B56" s="79" t="n"/>
-      <c r="C56" s="79" t="n"/>
-      <c r="D56" s="79" t="n"/>
-      <c r="E56" s="79" t="n"/>
-      <c r="F56" s="79" t="n"/>
-      <c r="G56" s="79" t="n"/>
+      <c r="A56" s="82" t="n"/>
+      <c r="B56" s="82" t="n"/>
+      <c r="C56" s="82" t="n"/>
+      <c r="D56" s="82" t="n"/>
+      <c r="E56" s="82" t="n"/>
+      <c r="F56" s="82" t="n"/>
+      <c r="G56" s="82" t="n"/>
     </row>
     <row r="57" ht="16" customHeight="1">
-      <c r="A57" s="79" t="n"/>
-      <c r="B57" s="79" t="n"/>
-      <c r="C57" s="79" t="n"/>
-      <c r="D57" s="79" t="n"/>
-      <c r="E57" s="79" t="n"/>
-      <c r="F57" s="79" t="n"/>
-      <c r="G57" s="79" t="n"/>
+      <c r="A57" s="82" t="n"/>
+      <c r="B57" s="82" t="n"/>
+      <c r="C57" s="82" t="n"/>
+      <c r="D57" s="82" t="n"/>
+      <c r="E57" s="82" t="n"/>
+      <c r="F57" s="82" t="n"/>
+      <c r="G57" s="82" t="n"/>
     </row>
     <row r="58" ht="16" customHeight="1">
-      <c r="A58" s="79" t="n"/>
-      <c r="B58" s="79" t="n"/>
-      <c r="C58" s="79" t="n"/>
-      <c r="D58" s="79" t="n"/>
-      <c r="E58" s="79" t="n"/>
-      <c r="F58" s="79" t="n"/>
-      <c r="G58" s="79" t="n"/>
+      <c r="A58" s="82" t="n"/>
+      <c r="B58" s="82" t="n"/>
+      <c r="C58" s="82" t="n"/>
+      <c r="D58" s="82" t="n"/>
+      <c r="E58" s="82" t="n"/>
+      <c r="F58" s="82" t="n"/>
+      <c r="G58" s="82" t="n"/>
     </row>
     <row r="59" ht="16" customHeight="1">
-      <c r="A59" s="79" t="n"/>
-      <c r="B59" s="79" t="n"/>
-      <c r="C59" s="79" t="n"/>
-      <c r="D59" s="79" t="n"/>
-      <c r="E59" s="79" t="n"/>
-      <c r="F59" s="79" t="n"/>
-      <c r="G59" s="79" t="n"/>
+      <c r="A59" s="82" t="n"/>
+      <c r="B59" s="82" t="n"/>
+      <c r="C59" s="82" t="n"/>
+      <c r="D59" s="82" t="n"/>
+      <c r="E59" s="82" t="n"/>
+      <c r="F59" s="82" t="n"/>
+      <c r="G59" s="82" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="20">

</xml_diff>

<commit_message>
v4: 3-team review — legal compliance, bug fixes, design unification
Legal (Brain):
- Add opening statement per Insurance Business Act Art.294-3
- Rewrite 募集人ポイント: remove agent-convenience language
  ("担当者の手間が少ない" etc.) — was a比較推奨規制 violation risk
- Add coverage questions: 車両保険/運転者範囲/走行距離
- Add intent-contract matching confirmation step
- Checklist: replace "MSI必ず含める" with customer-intent-based
  selection criteria; add 2 new compliance items

Bugs (Director):
- Fix H20-H24 DV: change merge_cells F:H→F:G so H column is
  independent — previously DVs on merged child cells were silently
  ignored by Excel

Design (Designer):
- Drop H7 dropdown; H10 is now the single entry point
- Branch guide row: sz=8→9, height=20→24
- Sheet2: apply colored medium border to E+F+G input cells uniformly
- Extract hardcoded hex values to named constants

https://claude.ai/code/session_01AJdG4TQantm5HZTxDeQNzp
</commit_message>
<xml_diff>
--- a/intent_tool.xlsx
+++ b/intent_tool.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="31">
+  <fonts count="29">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,11 +45,6 @@
     </font>
     <font>
       <name val="Meiryo UI"/>
-      <color rgb="00000000"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Meiryo UI"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="11"/>
@@ -57,17 +52,6 @@
     <font>
       <name val="Meiryo UI"/>
       <b val="1"/>
-      <color rgb="001C3557"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Meiryo UI"/>
-      <b val="1"/>
-      <color rgb="00C5D8F5"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="Meiryo UI"/>
       <color rgb="00C5D8F5"/>
       <sz val="8"/>
     </font>
@@ -80,14 +64,14 @@
     <font>
       <name val="Meiryo UI"/>
       <b val="1"/>
-      <color rgb="001B5EB5"/>
-      <sz val="8"/>
+      <color rgb="00C0392B"/>
+      <sz val="9"/>
     </font>
     <font>
       <name val="Meiryo UI"/>
       <b val="1"/>
-      <color rgb="00C0392B"/>
-      <sz val="9"/>
+      <color rgb="001C3557"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Meiryo UI"/>
@@ -115,24 +99,18 @@
     <font>
       <name val="Meiryo UI"/>
       <b val="1"/>
-      <color rgb="002E7D5B"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="Meiryo UI"/>
-      <b val="1"/>
-      <color rgb="00C0392B"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="Meiryo UI"/>
-      <b val="1"/>
       <color rgb="00B8DEC9"/>
       <sz val="8"/>
     </font>
     <font>
       <name val="Meiryo UI"/>
       <color rgb="00B8DEC9"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Meiryo UI"/>
+      <b val="1"/>
+      <color rgb="002E7D5B"/>
       <sz val="8"/>
     </font>
     <font>
@@ -145,12 +123,6 @@
       <name val="Meiryo UI"/>
       <color rgb="001C3557"/>
       <sz val="9"/>
-    </font>
-    <font>
-      <name val="Meiryo UI"/>
-      <b val="1"/>
-      <color rgb="002E7D5B"/>
-      <sz val="11"/>
     </font>
     <font>
       <name val="Meiryo UI"/>
@@ -182,6 +154,23 @@
     </font>
     <font>
       <name val="Meiryo UI"/>
+      <b val="1"/>
+      <color rgb="00C0392B"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Meiryo UI"/>
+      <color rgb="009B2335"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Meiryo UI"/>
+      <b val="1"/>
+      <color rgb="0093B8DC"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Meiryo UI"/>
       <color rgb="00404B3A"/>
       <sz val="9"/>
     </font>
@@ -194,7 +183,7 @@
       <name val="Meiryo UI"/>
       <b val="1"/>
       <color rgb="00000000"/>
-      <sz val="10"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="24">
@@ -226,11 +215,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C0392B"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="001B5EB5"/>
       </patternFill>
     </fill>
@@ -241,17 +225,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00DCE8F9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00EBF2FC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DCE8F9"/>
+        <fgColor rgb="00FFF8E1"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF8E1"/>
+        <fgColor rgb="00C0392B"/>
       </patternFill>
     </fill>
     <fill>
@@ -291,7 +280,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEFEFE"/>
+        <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
@@ -315,7 +304,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -335,6 +324,20 @@
       </top>
       <bottom style="thin">
         <color rgb="00BFC5BB"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="00C0392B"/>
+      </left>
+      <right style="medium">
+        <color rgb="00C0392B"/>
+      </right>
+      <top style="medium">
+        <color rgb="00C0392B"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="00C0392B"/>
       </bottom>
     </border>
     <border>
@@ -451,20 +454,6 @@
     </border>
     <border>
       <left style="medium">
-        <color rgb="00C0392B"/>
-      </left>
-      <right style="medium">
-        <color rgb="00C0392B"/>
-      </right>
-      <top style="medium">
-        <color rgb="00C0392B"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="00C0392B"/>
-      </bottom>
-    </border>
-    <border>
-      <left style="medium">
         <color rgb="002E7D5B"/>
       </left>
       <right style="medium">
@@ -475,6 +464,20 @@
       </top>
       <bottom style="medium">
         <color rgb="002E7D5B"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="001E6644"/>
+      </left>
+      <right style="medium">
+        <color rgb="001E6644"/>
+      </right>
+      <top style="medium">
+        <color rgb="001E6644"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001E6644"/>
       </bottom>
     </border>
     <border>
@@ -493,6 +496,20 @@
     </border>
     <border>
       <left style="medium">
+        <color rgb="001C3557"/>
+      </left>
+      <right style="medium">
+        <color rgb="001C3557"/>
+      </right>
+      <top style="medium">
+        <color rgb="001C3557"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="001C3557"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium">
         <color rgb="007A8575"/>
       </left>
       <right style="medium">
@@ -505,25 +522,11 @@
         <color rgb="007A8575"/>
       </bottom>
     </border>
-    <border>
-      <left style="medium">
-        <color rgb="001E6644"/>
-      </left>
-      <right style="medium">
-        <color rgb="001E6644"/>
-      </right>
-      <top style="medium">
-        <color rgb="001E6644"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="001E6644"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="96">
+  <cellXfs count="87">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -535,245 +538,224 @@
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="17" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="14" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="14" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="15" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="13" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="17" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="17" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="5" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="20" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="14" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="20" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="20" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="25" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="18" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="29" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="22" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="5" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="5" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="5" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="5" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1141,13 +1123,13 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H129"/>
+  <dimension ref="A1:H149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2.5" customWidth="1" min="1" max="1"/>
     <col width="3" customWidth="1" min="2" max="2"/>
     <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
@@ -1157,14 +1139,14 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ■ 自動車保険　意向確認シート（トークスクリプト型）</t>
+          <t xml:space="preserve">  ■ 自動車保険　意向確認シート（トークスクリプト型）　改正保険業法対応版</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ※ 太字部分はお客様へ読み上げてください。黄色セルを入力・選択し、選択後は対応する下のグループ ＋ を展開してください。</t>
+          <t xml:space="preserve">  ※ 太字部分はお客様へ読み上げます。黄色セルを入力・選択し、STEP2は選択後に左端の ＋ ボタンで該当グループを展開してください。</t>
         </is>
       </c>
     </row>
@@ -1198,23 +1180,25 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>支店</t>
+          <t>支　店</t>
         </is>
       </c>
       <c r="G4" s="3" t="n"/>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>契約方法</t>
-        </is>
-      </c>
+      <c r="H4" s="3" t="n"/>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="3" t="n"/>
       <c r="B5" s="3" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="6" t="n"/>
-      <c r="F5" s="6" t="n"/>
+      <c r="C5" s="5" t="n"/>
+      <c r="D5" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>3</v>
+      </c>
       <c r="G5" s="3" t="n"/>
       <c r="H5" s="3" t="n"/>
     </row>
@@ -1230,140 +1214,142 @@
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="3" t="n"/>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  STEP 1　　契約方法の確認</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="n"/>
-      <c r="D7" s="8" t="n"/>
-      <c r="E7" s="8" t="n"/>
-      <c r="F7" s="8" t="n"/>
-      <c r="G7" s="9" t="inlineStr">
-        <is>
-          <t>契約方法を選択 ▼</t>
-        </is>
-      </c>
-      <c r="H7" s="10" t="n"/>
-    </row>
-    <row r="8" ht="18" customHeight="1">
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  STEP 1　　はじめに・契約方法の確認</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="n"/>
+      <c r="D7" s="7" t="n"/>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="7" t="n"/>
+      <c r="H7" s="8" t="n"/>
+    </row>
+    <row r="8" ht="55" customHeight="1">
       <c r="A8" s="3" t="n"/>
-      <c r="B8" s="11" t="inlineStr">
-        <is>
-          <t>📋 スクリプト</t>
-        </is>
-      </c>
-      <c r="C8" s="12" t="n"/>
-      <c r="D8" s="13" t="inlineStr"/>
-      <c r="E8" s="12" t="n"/>
-      <c r="F8" s="12" t="n"/>
-      <c r="G8" s="12" t="n"/>
-      <c r="H8" s="14" t="n"/>
-    </row>
-    <row r="9" ht="80" customHeight="1">
+      <c r="B8" s="9" t="inlineStr">
+        <is>
+          <t>📣 読み上げ①
+（開始前）</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="n"/>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>「本日は自動車保険のご案内をいたします。当社は複数の保険会社の商品を取り扱っており、お客様のご意向・ご状況に合った保険をご提案するために、まずいくつかお伺いします。
+ご確認いただいた内容は意向確認の記録として残させていただきます。よろしいですか？」</t>
+        </is>
+      </c>
+      <c r="E8" s="10" t="n"/>
+      <c r="F8" s="10" t="n"/>
+      <c r="G8" s="10" t="n"/>
+      <c r="H8" s="12" t="n"/>
+    </row>
+    <row r="9" ht="70" customHeight="1">
       <c r="A9" s="3" t="n"/>
-      <c r="B9" s="15" t="inlineStr">
-        <is>
-          <t>📣 読み上げ</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="n"/>
-      <c r="D9" s="16" t="inlineStr">
-        <is>
-          <t>「当社では●社の自動車保険を扱っています。
-そのうち 給与天引き（団体割引）が使えるのは 損保ジャパン・三井住友海上・東京海上 の3社です。
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>📣 読み上げ②
+（契約方法）</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="n"/>
+      <c r="D9" s="13" t="inlineStr">
+        <is>
+          <t>「当社では●社の自動車保険を扱っています。そのうち 給与天引き（団体割引）が使えるのは 損保ジャパン・三井住友海上・東京海上 の3社です。
 通販型のソニー損保 へのお取り次ぎも可能で、クレジットカード払いや口座振替の一般契約もご案内できます。
 どのご契約方法をご希望ですか？」</t>
         </is>
       </c>
-      <c r="E9" s="12" t="n"/>
-      <c r="F9" s="12" t="n"/>
-      <c r="G9" s="12" t="n"/>
-      <c r="H9" s="14" t="n"/>
+      <c r="E9" s="10" t="n"/>
+      <c r="F9" s="10" t="n"/>
+      <c r="G9" s="10" t="n"/>
+      <c r="H9" s="12" t="n"/>
     </row>
     <row r="10" ht="26" customHeight="1">
       <c r="A10" s="3" t="n"/>
-      <c r="B10" s="17" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t xml:space="preserve">  ▶ お客様のご希望の契約方法（右の黄色セルで選択してください）</t>
         </is>
       </c>
-      <c r="C10" s="12" t="n"/>
-      <c r="D10" s="12" t="n"/>
-      <c r="E10" s="12" t="n"/>
-      <c r="F10" s="12" t="n"/>
-      <c r="G10" s="18" t="inlineStr">
+      <c r="C10" s="10" t="n"/>
+      <c r="D10" s="10" t="n"/>
+      <c r="E10" s="10" t="n"/>
+      <c r="F10" s="10" t="n"/>
+      <c r="G10" s="15" t="inlineStr">
         <is>
           <t>契約方法 →</t>
         </is>
       </c>
-      <c r="H10" s="10" t="n"/>
+      <c r="H10" s="16" t="n"/>
     </row>
     <row r="11" ht="20" customHeight="1">
       <c r="A11" s="3" t="n"/>
-      <c r="B11" s="19" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C11" s="20" t="inlineStr">
+      <c r="C11" s="18" t="inlineStr">
         <is>
           <t>給与天引き（団体割引）</t>
         </is>
       </c>
-      <c r="D11" s="21" t="inlineStr">
+      <c r="D11" s="19" t="inlineStr">
         <is>
           <t>→ 下のグループ「①②」を展開</t>
         </is>
       </c>
-      <c r="E11" s="12" t="n"/>
-      <c r="F11" s="12" t="n"/>
-      <c r="G11" s="12" t="n"/>
-      <c r="H11" s="22" t="n"/>
+      <c r="E11" s="10" t="n"/>
+      <c r="F11" s="10" t="n"/>
+      <c r="G11" s="10" t="n"/>
+      <c r="H11" s="12" t="n"/>
     </row>
     <row r="12" ht="20" customHeight="1">
       <c r="A12" s="3" t="n"/>
-      <c r="B12" s="23" t="inlineStr">
+      <c r="B12" s="20" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C12" s="24" t="inlineStr">
+      <c r="C12" s="21" t="inlineStr">
         <is>
           <t>一般契約（クレカ・口振）</t>
         </is>
       </c>
-      <c r="D12" s="25" t="inlineStr">
+      <c r="D12" s="22" t="inlineStr">
         <is>
           <t>→ 下のグループ「①②」を展開</t>
         </is>
       </c>
-      <c r="E12" s="12" t="n"/>
-      <c r="F12" s="12" t="n"/>
-      <c r="G12" s="12" t="n"/>
-      <c r="H12" s="26" t="n"/>
+      <c r="E12" s="10" t="n"/>
+      <c r="F12" s="10" t="n"/>
+      <c r="G12" s="10" t="n"/>
+      <c r="H12" s="12" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="3" t="n"/>
-      <c r="B13" s="27" t="inlineStr">
+      <c r="B13" s="23" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C13" s="28" t="inlineStr">
+      <c r="C13" s="24" t="inlineStr">
         <is>
           <t>通販型（ソニー損保）</t>
         </is>
       </c>
-      <c r="D13" s="29" t="inlineStr">
+      <c r="D13" s="25" t="inlineStr">
         <is>
           <t>→ 下のグループ「③」を展開</t>
         </is>
       </c>
-      <c r="E13" s="30" t="n"/>
-      <c r="F13" s="30" t="n"/>
-      <c r="G13" s="30" t="n"/>
-      <c r="H13" s="31" t="n"/>
+      <c r="E13" s="26" t="n"/>
+      <c r="F13" s="26" t="n"/>
+      <c r="G13" s="26" t="n"/>
+      <c r="H13" s="27" t="n"/>
     </row>
     <row r="14" ht="5" customHeight="1">
       <c r="A14" s="3" t="n"/>
@@ -1375,590 +1361,648 @@
       <c r="G14" s="3" t="n"/>
       <c r="H14" s="3" t="n"/>
     </row>
-    <row r="15" ht="20" customHeight="1">
+    <row r="15" ht="24" customHeight="1">
       <c r="A15" s="3" t="n"/>
-      <c r="B15" s="32" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ▼  ①② 給与天引き・一般契約 ─── 下のグループ「＋」で展開</t>
-        </is>
-      </c>
-      <c r="F15" s="33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ▼  ③ 通販型 ─── 下のグループ「＋」で展開</t>
+      <c r="B15" s="28" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ▼  ①② 給与天引き・一般契約 ─── 下のグループ ＋ で展開</t>
+        </is>
+      </c>
+      <c r="F15" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ▼  ③ 通販型 ─── 下のグループ ＋ で展開</t>
         </is>
       </c>
     </row>
     <row r="16" hidden="1" outlineLevel="1" ht="22" customHeight="1">
       <c r="A16" s="3" t="n"/>
-      <c r="B16" s="34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  STEP 2　　意向確認（重視事項）　　給与天引き・一般契約の方</t>
-        </is>
-      </c>
-      <c r="C16" s="8" t="n"/>
-      <c r="D16" s="8" t="n"/>
-      <c r="E16" s="8" t="n"/>
-      <c r="F16" s="8" t="n"/>
-      <c r="G16" s="8" t="n"/>
-      <c r="H16" s="35" t="n"/>
+      <c r="B16" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  STEP 2　　意向確認（重視事項・補償内容）　　給与天引き・一般契約の方</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="n"/>
+      <c r="D16" s="7" t="n"/>
+      <c r="E16" s="7" t="n"/>
+      <c r="F16" s="7" t="n"/>
+      <c r="G16" s="7" t="n"/>
+      <c r="H16" s="8" t="n"/>
     </row>
     <row r="17" hidden="1" outlineLevel="1" ht="18" customHeight="1">
       <c r="A17" s="3" t="n"/>
-      <c r="B17" s="36" t="inlineStr">
+      <c r="B17" s="31" t="inlineStr">
         <is>
           <t>📋 スクリプト</t>
         </is>
       </c>
-      <c r="C17" s="12" t="n"/>
-      <c r="D17" s="37" t="inlineStr"/>
-      <c r="E17" s="12" t="n"/>
-      <c r="F17" s="12" t="n"/>
-      <c r="G17" s="12" t="n"/>
-      <c r="H17" s="14" t="n"/>
-    </row>
-    <row r="18" hidden="1" outlineLevel="1" ht="60" customHeight="1">
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="32" t="inlineStr"/>
+      <c r="E17" s="10" t="n"/>
+      <c r="F17" s="10" t="n"/>
+      <c r="G17" s="10" t="n"/>
+      <c r="H17" s="12" t="n"/>
+    </row>
+    <row r="18" hidden="1" outlineLevel="1" ht="55" customHeight="1">
       <c r="A18" s="3" t="n"/>
-      <c r="B18" s="38" t="inlineStr">
+      <c r="B18" s="33" t="inlineStr">
         <is>
           <t>📣 読み上げ</t>
         </is>
       </c>
-      <c r="C18" s="12" t="n"/>
-      <c r="D18" s="39" t="inlineStr">
-        <is>
-          <t>「自動車保険でいちばん大切にしていることを教えていただけますか？
-いくつかお伺いしてもよいでしょうか？当てはまるものに○をつけてください。（複数回答可）」</t>
-        </is>
-      </c>
-      <c r="E18" s="12" t="n"/>
-      <c r="F18" s="12" t="n"/>
-      <c r="G18" s="12" t="n"/>
-      <c r="H18" s="14" t="n"/>
-    </row>
-    <row r="19" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="C18" s="10" t="n"/>
+      <c r="D18" s="34" t="inlineStr">
+        <is>
+          <t>「自動車保険でいちばん大切にしていることを教えていただけますか？いくつかお伺いしてもよいでしょうか？
+当てはまるものに○をつけてください。（複数回答可）」</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="n"/>
+      <c r="F18" s="10" t="n"/>
+      <c r="G18" s="10" t="n"/>
+      <c r="H18" s="12" t="n"/>
+    </row>
+    <row r="19" hidden="1" outlineLevel="1" ht="18" customHeight="1">
       <c r="A19" s="3" t="n"/>
-      <c r="B19" s="36" t="inlineStr">
-        <is>
-          <t>重視項目</t>
-        </is>
-      </c>
-      <c r="C19" s="12" t="n"/>
-      <c r="D19" s="40" t="inlineStr">
-        <is>
-          <t>お客様選択</t>
-        </is>
-      </c>
-      <c r="E19" s="12" t="n"/>
-      <c r="F19" s="40" t="inlineStr">
+      <c r="B19" s="31" t="inlineStr">
+        <is>
+          <t>重視事項
+（複数可）</t>
+        </is>
+      </c>
+      <c r="C19" s="10" t="n"/>
+      <c r="D19" s="35" t="inlineStr">
+        <is>
+          <t>お客様の重視事項</t>
+        </is>
+      </c>
+      <c r="E19" s="10" t="n"/>
+      <c r="F19" s="10" t="n"/>
+      <c r="G19" s="35" t="inlineStr">
         <is>
           <t>各社の強み（参考）</t>
         </is>
       </c>
-      <c r="G19" s="12" t="n"/>
-      <c r="H19" s="14" t="n"/>
+      <c r="H19" s="12" t="n"/>
     </row>
     <row r="20" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A20" s="3" t="n"/>
-      <c r="B20" s="41" t="inlineStr">
+      <c r="B20" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">  ①</t>
         </is>
       </c>
-      <c r="C20" s="42" t="inlineStr">
+      <c r="C20" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">  保険料をできるだけ抑えたい</t>
         </is>
       </c>
-      <c r="D20" s="12" t="n"/>
-      <c r="E20" s="12" t="n"/>
-      <c r="F20" s="43" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  損保ジャパン（多様なプラン）／三井住友海上（ネット割引あり）</t>
-        </is>
-      </c>
-      <c r="G20" s="12" t="n"/>
-      <c r="H20" s="44" t="n"/>
+      <c r="D20" s="10" t="n"/>
+      <c r="E20" s="10" t="n"/>
+      <c r="F20" s="10" t="n"/>
+      <c r="G20" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  損保ジャパン（多様なプラン）／三井住友海上（ネット割引）</t>
+        </is>
+      </c>
+      <c r="H20" s="16" t="n"/>
     </row>
     <row r="21" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A21" s="3" t="n"/>
-      <c r="B21" s="41" t="inlineStr">
+      <c r="B21" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">  ②</t>
         </is>
       </c>
-      <c r="C21" s="42" t="inlineStr">
+      <c r="C21" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">  補償をしっかり充実させたい</t>
         </is>
       </c>
-      <c r="D21" s="12" t="n"/>
-      <c r="E21" s="12" t="n"/>
-      <c r="F21" s="43" t="inlineStr">
+      <c r="D21" s="10" t="n"/>
+      <c r="E21" s="10" t="n"/>
+      <c r="F21" s="10" t="n"/>
+      <c r="G21" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  東京海上（総合型・特約充実）／損保ジャパン（幅広い特約）</t>
         </is>
       </c>
-      <c r="G21" s="12" t="n"/>
-      <c r="H21" s="44" t="n"/>
+      <c r="H21" s="16" t="n"/>
     </row>
     <row r="22" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A22" s="3" t="n"/>
-      <c r="B22" s="41" t="inlineStr">
+      <c r="B22" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">  ③</t>
         </is>
       </c>
-      <c r="C22" s="42" t="inlineStr">
+      <c r="C22" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">  事故時の対応・サポートを重視したい</t>
         </is>
       </c>
-      <c r="D22" s="12" t="n"/>
-      <c r="E22" s="12" t="n"/>
-      <c r="F22" s="43" t="inlineStr">
+      <c r="D22" s="10" t="n"/>
+      <c r="E22" s="10" t="n"/>
+      <c r="F22" s="10" t="n"/>
+      <c r="G22" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  三井住友海上（示談交渉◎）／東京海上（専任担当）</t>
         </is>
       </c>
-      <c r="G22" s="12" t="n"/>
-      <c r="H22" s="44" t="n"/>
+      <c r="H22" s="16" t="n"/>
     </row>
     <row r="23" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A23" s="3" t="n"/>
-      <c r="B23" s="41" t="inlineStr">
+      <c r="B23" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">  ④</t>
         </is>
       </c>
-      <c r="C23" s="42" t="inlineStr">
+      <c r="C23" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">  手続きが簡単・わかりやすいものがいい</t>
         </is>
       </c>
-      <c r="D23" s="12" t="n"/>
-      <c r="E23" s="12" t="n"/>
-      <c r="F23" s="43" t="inlineStr">
+      <c r="D23" s="10" t="n"/>
+      <c r="E23" s="10" t="n"/>
+      <c r="F23" s="10" t="n"/>
+      <c r="G23" s="38" t="inlineStr">
         <is>
           <t xml:space="preserve">  三井住友海上（シンプル設計・見積り速い）</t>
         </is>
       </c>
-      <c r="G23" s="12" t="n"/>
-      <c r="H23" s="44" t="n"/>
+      <c r="H23" s="16" t="n"/>
     </row>
     <row r="24" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A24" s="3" t="n"/>
-      <c r="B24" s="45" t="inlineStr">
+      <c r="B24" s="36" t="inlineStr">
         <is>
           <t xml:space="preserve">  ⑤</t>
         </is>
       </c>
-      <c r="C24" s="46" t="inlineStr">
+      <c r="C24" s="37" t="inlineStr">
         <is>
           <t xml:space="preserve">  担当者に相談しながら決めたい</t>
         </is>
       </c>
-      <c r="D24" s="30" t="n"/>
-      <c r="E24" s="30" t="n"/>
-      <c r="F24" s="47" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  3社すべて対応可。担当者によるサポートが手厚い</t>
-        </is>
-      </c>
-      <c r="G24" s="30" t="n"/>
-      <c r="H24" s="48" t="n"/>
-    </row>
-    <row r="25" hidden="1" outlineLevel="1" ht="18" customHeight="1">
+      <c r="D24" s="10" t="n"/>
+      <c r="E24" s="10" t="n"/>
+      <c r="F24" s="10" t="n"/>
+      <c r="G24" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  3社すべて対応可。担当者によるサポート</t>
+        </is>
+      </c>
+      <c r="H24" s="16" t="n"/>
+    </row>
+    <row r="25" hidden="1" outlineLevel="1" ht="5" customHeight="1">
       <c r="A25" s="3" t="n"/>
-      <c r="B25" s="3" t="n"/>
-      <c r="C25" s="3" t="n"/>
-      <c r="D25" s="3" t="n"/>
-      <c r="E25" s="3" t="n"/>
-      <c r="F25" s="3" t="n"/>
-      <c r="G25" s="3" t="n"/>
-      <c r="H25" s="3" t="n"/>
-    </row>
-    <row r="26" hidden="1" outlineLevel="1" ht="22" customHeight="1">
+      <c r="B25" s="39" t="n"/>
+      <c r="C25" s="40" t="n"/>
+      <c r="D25" s="40" t="n"/>
+      <c r="E25" s="40" t="n"/>
+      <c r="F25" s="40" t="n"/>
+      <c r="G25" s="40" t="n"/>
+      <c r="H25" s="41" t="n"/>
+    </row>
+    <row r="26" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A26" s="3" t="n"/>
-      <c r="B26" s="49" t="inlineStr">
+      <c r="B26" s="42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  補償内容の確認（意向把握の必須事項）</t>
+        </is>
+      </c>
+      <c r="C26" s="10" t="n"/>
+      <c r="D26" s="10" t="n"/>
+      <c r="E26" s="10" t="n"/>
+      <c r="F26" s="10" t="n"/>
+      <c r="G26" s="10" t="n"/>
+      <c r="H26" s="12" t="n"/>
+    </row>
+    <row r="27" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A27" s="3" t="n"/>
+      <c r="B27" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ⑥</t>
+        </is>
+      </c>
+      <c r="C27" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  車両保険の加入希望</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="n"/>
+      <c r="E27" s="10" t="n"/>
+      <c r="F27" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  車両保険あり・なしで保険料が大きく変わります</t>
+        </is>
+      </c>
+      <c r="G27" s="10" t="n"/>
+      <c r="H27" s="16" t="n"/>
+    </row>
+    <row r="28" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A28" s="3" t="n"/>
+      <c r="B28" s="43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ⑦</t>
+        </is>
+      </c>
+      <c r="C28" s="37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  運転者の範囲</t>
+        </is>
+      </c>
+      <c r="D28" s="10" t="n"/>
+      <c r="E28" s="10" t="n"/>
+      <c r="F28" s="38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  限定なしは保険料が高くなる場合があります</t>
+        </is>
+      </c>
+      <c r="G28" s="10" t="n"/>
+      <c r="H28" s="16" t="n"/>
+    </row>
+    <row r="29" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A29" s="3" t="n"/>
+      <c r="B29" s="44" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ⑧</t>
+        </is>
+      </c>
+      <c r="C29" s="45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  年間走行距離の目安</t>
+        </is>
+      </c>
+      <c r="D29" s="26" t="n"/>
+      <c r="E29" s="26" t="n"/>
+      <c r="F29" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  距離が多いほどリスクが高まる場合があります</t>
+        </is>
+      </c>
+      <c r="G29" s="26" t="n"/>
+      <c r="H29" s="47" t="n"/>
+    </row>
+    <row r="30" hidden="1" outlineLevel="1" ht="5" customHeight="1">
+      <c r="A30" s="3" t="n"/>
+      <c r="B30" s="3" t="n"/>
+      <c r="C30" s="3" t="n"/>
+      <c r="D30" s="3" t="n"/>
+      <c r="E30" s="3" t="n"/>
+      <c r="F30" s="3" t="n"/>
+      <c r="G30" s="3" t="n"/>
+      <c r="H30" s="3" t="n"/>
+    </row>
+    <row r="31" hidden="1" outlineLevel="1" ht="22" customHeight="1">
+      <c r="A31" s="3" t="n"/>
+      <c r="B31" s="48" t="inlineStr">
         <is>
           <t xml:space="preserve">  STEP 2-2　　3社ご提案（意向確認結果をふまえて）</t>
         </is>
       </c>
-      <c r="C26" s="8" t="n"/>
-      <c r="D26" s="8" t="n"/>
-      <c r="E26" s="8" t="n"/>
-      <c r="F26" s="8" t="n"/>
-      <c r="G26" s="8" t="n"/>
-      <c r="H26" s="35" t="n"/>
-    </row>
-    <row r="27" hidden="1" outlineLevel="1" ht="18" customHeight="1">
-      <c r="A27" s="3" t="n"/>
-      <c r="B27" s="36" t="inlineStr">
+      <c r="C31" s="7" t="n"/>
+      <c r="D31" s="7" t="n"/>
+      <c r="E31" s="7" t="n"/>
+      <c r="F31" s="7" t="n"/>
+      <c r="G31" s="7" t="n"/>
+      <c r="H31" s="8" t="n"/>
+    </row>
+    <row r="32" hidden="1" outlineLevel="1" ht="18" customHeight="1">
+      <c r="A32" s="3" t="n"/>
+      <c r="B32" s="31" t="inlineStr">
         <is>
           <t>📣 読み上げ
 + ポイント</t>
         </is>
       </c>
-      <c r="C27" s="12" t="n"/>
-      <c r="D27" s="50" t="inlineStr">
-        <is>
-          <t>「ありがとうございます。いただいたご希望をもとに、損保ジャパン・三井住友海上・東京海上 の3社でお見積りをご用意します。
-─── 募集人ポイント ────────────────────────────────────────────────────────────
-三井住友海上はシンプル設計で見積り・手続きが速く、担当者の手間が少ないです。
-お客様には保険料もご提示しやすい選択肢です。必ず3社セットでお見せしましょう。
-────────────────────────────────────────────────────────────────────────────」</t>
-        </is>
-      </c>
-      <c r="E27" s="12" t="n"/>
-      <c r="F27" s="12" t="n"/>
-      <c r="G27" s="12" t="n"/>
-      <c r="H27" s="14" t="n"/>
-    </row>
-    <row r="28" hidden="1" outlineLevel="1" ht="60" customHeight="1">
-      <c r="A28" s="3" t="n"/>
-      <c r="B28" s="51" t="inlineStr">
+      <c r="C32" s="10" t="n"/>
+      <c r="D32" s="49" t="inlineStr">
+        <is>
+          <t>「ありがとうございます。いただいたご意向をもとに、損保ジャパン・三井住友海上・東京海上の3社でお見積りをご用意します。
+─── 募集人ポイント（顧客の意向に基づく推奨根拠を説明してください）──────────────────
+・保険料重視 → 三井住友海上のシンプルプランが競争力あり。ネット割引も活用可
+・補償充実重視 → 東京海上の総合型、または損保ジャパンの幅広い特約構成
+・事故対応重視 → 三井住友海上の示談交渉サービス、東京海上の専任担当制度
+・手続き簡便重視 → 三井住友海上のシンプル設計はお客様にとって分かりやすい
+必ず3社のお見積りをお客様にご提示し、推奨理由をご説明ください。」</t>
+        </is>
+      </c>
+      <c r="E32" s="10" t="n"/>
+      <c r="F32" s="10" t="n"/>
+      <c r="G32" s="10" t="n"/>
+      <c r="H32" s="12" t="n"/>
+    </row>
+    <row r="33" hidden="1" outlineLevel="1" ht="68" customHeight="1">
+      <c r="A33" s="3" t="n"/>
+      <c r="B33" s="50" t="inlineStr">
         <is>
           <t>会　社</t>
         </is>
       </c>
-      <c r="C28" s="12" t="n"/>
-      <c r="D28" s="52" t="inlineStr">
+      <c r="C33" s="10" t="n"/>
+      <c r="D33" s="51" t="inlineStr">
         <is>
           <t>主な強み・特徴</t>
         </is>
       </c>
-      <c r="E28" s="12" t="n"/>
-      <c r="F28" s="52" t="inlineStr">
-        <is>
-          <t>MSI提案の一言</t>
-        </is>
-      </c>
-      <c r="G28" s="12" t="n"/>
-      <c r="H28" s="53" t="inlineStr">
+      <c r="E33" s="10" t="n"/>
+      <c r="F33" s="51" t="inlineStr">
+        <is>
+          <t>顧客への一言</t>
+        </is>
+      </c>
+      <c r="G33" s="10" t="n"/>
+      <c r="H33" s="52" t="inlineStr">
         <is>
           <t>提案</t>
         </is>
       </c>
     </row>
-    <row r="29" hidden="1" outlineLevel="1" ht="18" customHeight="1">
-      <c r="A29" s="3" t="n"/>
-      <c r="B29" s="54" t="inlineStr">
+    <row r="34" hidden="1" outlineLevel="1" ht="18" customHeight="1">
+      <c r="A34" s="3" t="n"/>
+      <c r="B34" s="53" t="inlineStr">
         <is>
           <t xml:space="preserve">  損保ジャパン</t>
         </is>
       </c>
-      <c r="C29" s="12" t="n"/>
-      <c r="D29" s="55" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  取引歴が長く慣れている。多彩なプラン・特約</t>
-        </is>
-      </c>
-      <c r="E29" s="12" t="n"/>
-      <c r="F29" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  慣れ親しんだ会社。実績・信頼で推せます</t>
-        </is>
-      </c>
-      <c r="G29" s="12" t="n"/>
-      <c r="H29" s="57" t="n"/>
-    </row>
-    <row r="30" hidden="1" outlineLevel="1" ht="18" customHeight="1">
-      <c r="A30" s="3" t="n"/>
-      <c r="B30" s="58" t="inlineStr">
+      <c r="C34" s="10" t="n"/>
+      <c r="D34" s="54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  取引歴が長く多彩なプラン・特約</t>
+        </is>
+      </c>
+      <c r="E34" s="10" t="n"/>
+      <c r="F34" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  慣れ親しんだ信頼の1社。特約の選択肢が豊富</t>
+        </is>
+      </c>
+      <c r="G34" s="10" t="n"/>
+      <c r="H34" s="16" t="n"/>
+    </row>
+    <row r="35" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A35" s="3" t="n"/>
+      <c r="B35" s="56" t="inlineStr">
         <is>
           <t xml:space="preserve">  三井住友海上</t>
         </is>
       </c>
-      <c r="C30" s="12" t="n"/>
-      <c r="D30" s="21" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  シンプル設計・見積り速い・ネット割引あり</t>
-        </is>
-      </c>
-      <c r="E30" s="12" t="n"/>
-      <c r="F30" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  手続きが楽で保険料も競争力あり。比較必須</t>
-        </is>
-      </c>
-      <c r="G30" s="12" t="n"/>
-      <c r="H30" s="59" t="n"/>
-    </row>
-    <row r="31" hidden="1" outlineLevel="1" ht="18" customHeight="1">
-      <c r="A31" s="3" t="n"/>
-      <c r="B31" s="60" t="inlineStr">
+      <c r="C35" s="10" t="n"/>
+      <c r="D35" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  シンプル設計・ネット割引・見積り速い</t>
+        </is>
+      </c>
+      <c r="E35" s="10" t="n"/>
+      <c r="F35" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  保険料を重視される方、手続きの明快さを求める方に</t>
+        </is>
+      </c>
+      <c r="G35" s="10" t="n"/>
+      <c r="H35" s="16" t="n"/>
+    </row>
+    <row r="36" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A36" s="3" t="n"/>
+      <c r="B36" s="57" t="inlineStr">
         <is>
           <t xml:space="preserve">  東京海上日動</t>
         </is>
       </c>
-      <c r="C31" s="12" t="n"/>
-      <c r="D31" s="25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  業界最大手。補償・サービスの充実度が高い</t>
-        </is>
-      </c>
-      <c r="E31" s="12" t="n"/>
-      <c r="F31" s="56" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  手厚い補償を重視するお客様に有効</t>
-        </is>
-      </c>
-      <c r="G31" s="12" t="n"/>
-      <c r="H31" s="61" t="n"/>
-    </row>
-    <row r="32" hidden="1" outlineLevel="1" ht="18" customHeight="1">
-      <c r="A32" s="3" t="n"/>
-      <c r="B32" s="62" t="n"/>
-      <c r="C32" s="63" t="n"/>
-      <c r="D32" s="63" t="n"/>
-      <c r="E32" s="63" t="n"/>
-      <c r="F32" s="63" t="n"/>
-      <c r="G32" s="63" t="n"/>
-      <c r="H32" s="64" t="n"/>
-    </row>
-    <row r="33" hidden="1" outlineLevel="1" ht="18" customHeight="1">
-      <c r="A33" s="3" t="n"/>
-      <c r="B33" s="65" t="n"/>
-      <c r="C33" s="66" t="n"/>
-      <c r="D33" s="66" t="n"/>
-      <c r="E33" s="66" t="n"/>
-      <c r="F33" s="66" t="n"/>
-      <c r="G33" s="66" t="n"/>
-      <c r="H33" s="67" t="n"/>
-    </row>
-    <row r="34" hidden="1" outlineLevel="1" ht="5" customHeight="1">
-      <c r="A34" s="3" t="n"/>
-      <c r="B34" s="3" t="n"/>
-      <c r="C34" s="3" t="n"/>
-      <c r="D34" s="3" t="n"/>
-      <c r="E34" s="3" t="n"/>
-      <c r="F34" s="3" t="n"/>
-      <c r="G34" s="3" t="n"/>
-      <c r="H34" s="3" t="n"/>
-    </row>
-    <row r="35" ht="5" customHeight="1">
-      <c r="A35" s="3" t="n"/>
-      <c r="B35" s="3" t="n"/>
-      <c r="C35" s="3" t="n"/>
-      <c r="D35" s="3" t="n"/>
-      <c r="E35" s="3" t="n"/>
-      <c r="F35" s="3" t="n"/>
-      <c r="G35" s="3" t="n"/>
-      <c r="H35" s="3" t="n"/>
-    </row>
-    <row r="36" hidden="1" outlineLevel="1" ht="22" customHeight="1">
-      <c r="A36" s="3" t="n"/>
-      <c r="B36" s="68" t="inlineStr">
+      <c r="C36" s="10" t="n"/>
+      <c r="D36" s="22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  業界最大手・補償充実・専任担当制度あり</t>
+        </is>
+      </c>
+      <c r="E36" s="10" t="n"/>
+      <c r="F36" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  手厚い補償・事故後のサポートを重視される方に</t>
+        </is>
+      </c>
+      <c r="G36" s="10" t="n"/>
+      <c r="H36" s="16" t="n"/>
+    </row>
+    <row r="37" hidden="1" outlineLevel="1" ht="20" customHeight="1">
+      <c r="A37" s="3" t="n"/>
+      <c r="B37" s="58" t="n"/>
+      <c r="C37" s="59" t="n"/>
+      <c r="D37" s="59" t="n"/>
+      <c r="E37" s="59" t="n"/>
+      <c r="F37" s="59" t="n"/>
+      <c r="G37" s="59" t="n"/>
+      <c r="H37" s="60" t="n"/>
+    </row>
+    <row r="38" hidden="1" outlineLevel="1" ht="5" customHeight="1">
+      <c r="A38" s="3" t="n"/>
+      <c r="B38" s="3" t="n"/>
+      <c r="C38" s="3" t="n"/>
+      <c r="D38" s="3" t="n"/>
+      <c r="E38" s="3" t="n"/>
+      <c r="F38" s="3" t="n"/>
+      <c r="G38" s="3" t="n"/>
+      <c r="H38" s="3" t="n"/>
+    </row>
+    <row r="39" ht="16" customHeight="1">
+      <c r="A39" s="3" t="n"/>
+      <c r="B39" s="3" t="n"/>
+      <c r="C39" s="3" t="n"/>
+      <c r="D39" s="3" t="n"/>
+      <c r="E39" s="3" t="n"/>
+      <c r="F39" s="3" t="n"/>
+      <c r="G39" s="3" t="n"/>
+      <c r="H39" s="3" t="n"/>
+    </row>
+    <row r="40" hidden="1" outlineLevel="1" ht="22" customHeight="1">
+      <c r="A40" s="3" t="n"/>
+      <c r="B40" s="61" t="inlineStr">
         <is>
           <t xml:space="preserve">  STEP 2　　ソニー損保ご案内　　通販型をご希望の方</t>
         </is>
       </c>
-      <c r="C36" s="8" t="n"/>
-      <c r="D36" s="8" t="n"/>
-      <c r="E36" s="8" t="n"/>
-      <c r="F36" s="8" t="n"/>
-      <c r="G36" s="8" t="n"/>
-      <c r="H36" s="35" t="n"/>
-    </row>
-    <row r="37" hidden="1" outlineLevel="1" ht="18" customHeight="1">
-      <c r="A37" s="3" t="n"/>
-      <c r="B37" s="69" t="inlineStr">
-        <is>
-          <t>📋 スクリプト</t>
-        </is>
-      </c>
-      <c r="C37" s="12" t="n"/>
-      <c r="D37" s="70" t="inlineStr"/>
-      <c r="E37" s="12" t="n"/>
-      <c r="F37" s="12" t="n"/>
-      <c r="G37" s="12" t="n"/>
-      <c r="H37" s="14" t="n"/>
-    </row>
-    <row r="38" hidden="1" outlineLevel="1" ht="65" customHeight="1">
-      <c r="A38" s="3" t="n"/>
-      <c r="B38" s="71" t="inlineStr">
-        <is>
-          <t>📣 読み上げ①</t>
-        </is>
-      </c>
-      <c r="C38" s="12" t="n"/>
-      <c r="D38" s="72" t="inlineStr">
-        <is>
-          <t>「それではソニー損保をご案内しますので、お客様のご状況を確認させてください。
-ソニー損保はインターネットでお客様ご自身に直接ご契約いただく通販型です。手続きはお客様側のご対応となりますが、よろしいでしょうか？」</t>
-        </is>
-      </c>
-      <c r="E38" s="12" t="n"/>
-      <c r="F38" s="12" t="n"/>
-      <c r="G38" s="12" t="n"/>
-      <c r="H38" s="14" t="n"/>
-    </row>
-    <row r="39" hidden="1" outlineLevel="1" ht="65" customHeight="1">
-      <c r="A39" s="3" t="n"/>
-      <c r="B39" s="71" t="inlineStr">
-        <is>
-          <t>📣 読み上げ②
-（留意点）</t>
-        </is>
-      </c>
-      <c r="C39" s="12" t="n"/>
-      <c r="D39" s="72" t="inlineStr">
-        <is>
-          <t>「保険料面ではメリットが出る場合もありますが、事故時のサポートはコールセンター対応が基本となります。
-当社担当者が直接サポートすることは難しくなりますが、それでもよろしいでしょうか？
-ご希望でしたら、ソニー損保のサイトをご一緒に確認しながら手続きをご案内します。」</t>
-        </is>
-      </c>
-      <c r="E39" s="12" t="n"/>
-      <c r="F39" s="12" t="n"/>
-      <c r="G39" s="12" t="n"/>
-      <c r="H39" s="14" t="n"/>
-    </row>
-    <row r="40" hidden="1" outlineLevel="1" ht="20" customHeight="1">
-      <c r="A40" s="3" t="n"/>
-      <c r="B40" s="69" t="inlineStr">
-        <is>
-          <t>✏️ お客様の意向</t>
-        </is>
-      </c>
-      <c r="C40" s="12" t="n"/>
-      <c r="D40" s="73" t="inlineStr">
-        <is>
-          <t>ソニー損保で進める</t>
-        </is>
-      </c>
-      <c r="E40" s="12" t="n"/>
-      <c r="F40" s="12" t="n"/>
-      <c r="G40" s="12" t="n"/>
-      <c r="H40" s="57" t="n"/>
+      <c r="C40" s="7" t="n"/>
+      <c r="D40" s="7" t="n"/>
+      <c r="E40" s="7" t="n"/>
+      <c r="F40" s="7" t="n"/>
+      <c r="G40" s="7" t="n"/>
+      <c r="H40" s="8" t="n"/>
     </row>
     <row r="41" hidden="1" outlineLevel="1" ht="18" customHeight="1">
       <c r="A41" s="3" t="n"/>
-      <c r="B41" s="74" t="inlineStr"/>
-      <c r="C41" s="12" t="n"/>
-      <c r="D41" s="63" t="n"/>
-      <c r="E41" s="63" t="n"/>
-      <c r="F41" s="63" t="n"/>
-      <c r="G41" s="63" t="n"/>
-      <c r="H41" s="64" t="n"/>
-    </row>
-    <row r="42" hidden="1" outlineLevel="1" ht="18" customHeight="1">
+      <c r="B41" s="62" t="inlineStr">
+        <is>
+          <t>📋 スクリプト</t>
+        </is>
+      </c>
+      <c r="C41" s="10" t="n"/>
+      <c r="D41" s="63" t="inlineStr"/>
+      <c r="E41" s="10" t="n"/>
+      <c r="F41" s="10" t="n"/>
+      <c r="G41" s="10" t="n"/>
+      <c r="H41" s="12" t="n"/>
+    </row>
+    <row r="42" hidden="1" outlineLevel="1" ht="60" customHeight="1">
       <c r="A42" s="3" t="n"/>
-      <c r="B42" s="75" t="inlineStr"/>
-      <c r="C42" s="30" t="n"/>
-      <c r="D42" s="66" t="n"/>
-      <c r="E42" s="66" t="n"/>
-      <c r="F42" s="66" t="n"/>
-      <c r="G42" s="66" t="n"/>
-      <c r="H42" s="67" t="n"/>
-    </row>
-    <row r="43" hidden="1" outlineLevel="1" ht="5" customHeight="1">
+      <c r="B42" s="64" t="inlineStr">
+        <is>
+          <t>📣 読み上げ①</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="n"/>
+      <c r="D42" s="65" t="inlineStr">
+        <is>
+          <t>「それではソニー損保をご案内しますので、お客様のご状況を確認させてください。
+ソニー損保はインターネットでお客様ご自身に直接ご契約いただく通販型です。当社（代理店）が契約を代理するものではなく、申込内容・告知内容はお客様ご自身でご入力・ご確認いただきます。手続きはお客様側のご対応となりますが、よろしいでしょうか？」</t>
+        </is>
+      </c>
+      <c r="E42" s="10" t="n"/>
+      <c r="F42" s="10" t="n"/>
+      <c r="G42" s="10" t="n"/>
+      <c r="H42" s="12" t="n"/>
+    </row>
+    <row r="43" hidden="1" outlineLevel="1" ht="60" customHeight="1">
       <c r="A43" s="3" t="n"/>
-      <c r="B43" s="3" t="n"/>
-      <c r="C43" s="3" t="n"/>
-      <c r="D43" s="3" t="n"/>
-      <c r="E43" s="3" t="n"/>
-      <c r="F43" s="3" t="n"/>
-      <c r="G43" s="3" t="n"/>
-      <c r="H43" s="3" t="n"/>
-    </row>
-    <row r="44" hidden="1" outlineLevel="1" ht="16" customHeight="1">
+      <c r="B43" s="64" t="inlineStr">
+        <is>
+          <t>📣 読み上げ②
+（留意事項）</t>
+        </is>
+      </c>
+      <c r="C43" s="10" t="n"/>
+      <c r="D43" s="65" t="inlineStr">
+        <is>
+          <t>「事故時のサポートはソニー損保のコールセンター対応が基本となり、当社担当者が直接サポートすることは難しくなります。
+ご契約後の変更・事故対応についてもソニー損保に直接ご連絡いただくことになります。
+この点をご了解いただいたうえでご希望ですか？」</t>
+        </is>
+      </c>
+      <c r="E43" s="10" t="n"/>
+      <c r="F43" s="10" t="n"/>
+      <c r="G43" s="10" t="n"/>
+      <c r="H43" s="12" t="n"/>
+    </row>
+    <row r="44" hidden="1" outlineLevel="1" ht="22" customHeight="1">
       <c r="A44" s="3" t="n"/>
-      <c r="B44" s="3" t="n"/>
-      <c r="C44" s="3" t="n"/>
-      <c r="D44" s="3" t="n"/>
-      <c r="E44" s="3" t="n"/>
-      <c r="F44" s="3" t="n"/>
-      <c r="G44" s="3" t="n"/>
-      <c r="H44" s="3" t="n"/>
-    </row>
-    <row r="45" ht="16" customHeight="1">
+      <c r="B44" s="62" t="inlineStr">
+        <is>
+          <t>✏️ お客様確認</t>
+        </is>
+      </c>
+      <c r="C44" s="10" t="n"/>
+      <c r="D44" s="54" t="inlineStr">
+        <is>
+          <t>通販型の特性（直接契約・コールセンター）を理解の上、ソニー損保を希望する</t>
+        </is>
+      </c>
+      <c r="E44" s="10" t="n"/>
+      <c r="F44" s="66" t="inlineStr">
+        <is>
+          <t>← お客様の意向を選択</t>
+        </is>
+      </c>
+      <c r="G44" s="10" t="n"/>
+      <c r="H44" s="16" t="n"/>
+    </row>
+    <row r="45" hidden="1" outlineLevel="1" ht="20" customHeight="1">
       <c r="A45" s="3" t="n"/>
-      <c r="B45" s="3" t="n"/>
-      <c r="C45" s="3" t="n"/>
-      <c r="D45" s="3" t="n"/>
-      <c r="E45" s="3" t="n"/>
-      <c r="F45" s="3" t="n"/>
-      <c r="G45" s="3" t="n"/>
-      <c r="H45" s="3" t="n"/>
-    </row>
-    <row r="46" ht="20" customHeight="1">
+      <c r="B45" s="58" t="n"/>
+      <c r="C45" s="59" t="n"/>
+      <c r="D45" s="59" t="n"/>
+      <c r="E45" s="59" t="n"/>
+      <c r="F45" s="59" t="n"/>
+      <c r="G45" s="59" t="n"/>
+      <c r="H45" s="60" t="n"/>
+    </row>
+    <row r="46" hidden="1" outlineLevel="1" ht="5" customHeight="1">
       <c r="A46" s="3" t="n"/>
-      <c r="B46" s="76" t="inlineStr">
+      <c r="B46" s="3" t="n"/>
+      <c r="C46" s="3" t="n"/>
+      <c r="D46" s="3" t="n"/>
+      <c r="E46" s="3" t="n"/>
+      <c r="F46" s="3" t="n"/>
+      <c r="G46" s="3" t="n"/>
+      <c r="H46" s="3" t="n"/>
+    </row>
+    <row r="47" ht="16" customHeight="1">
+      <c r="A47" s="3" t="n"/>
+      <c r="B47" s="3" t="n"/>
+      <c r="C47" s="3" t="n"/>
+      <c r="D47" s="3" t="n"/>
+      <c r="E47" s="3" t="n"/>
+      <c r="F47" s="3" t="n"/>
+      <c r="G47" s="3" t="n"/>
+      <c r="H47" s="3" t="n"/>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="3" t="n"/>
+      <c r="B48" s="67" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ■ 意向と最終選択の確認（契約前に必ず実施）</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="n"/>
+      <c r="D48" s="7" t="n"/>
+      <c r="E48" s="7" t="n"/>
+      <c r="F48" s="7" t="n"/>
+      <c r="G48" s="7" t="n"/>
+      <c r="H48" s="8" t="n"/>
+    </row>
+    <row r="49" ht="40" customHeight="1">
+      <c r="A49" s="3" t="n"/>
+      <c r="B49" s="68" t="inlineStr">
+        <is>
+          <t>📣 確認・記録</t>
+        </is>
+      </c>
+      <c r="C49" s="26" t="n"/>
+      <c r="D49" s="69" t="inlineStr">
+        <is>
+          <t>「本日ご提案した○○（会社名）の○○プランは、先ほどお伺いしたご意向（○○を重視）に沿ったものです。ご確認いただけますか？」
+→ 異なる商品をご選択の場合は、右の欄にその理由を記録してください。</t>
+        </is>
+      </c>
+      <c r="E49" s="26" t="n"/>
+      <c r="F49" s="26" t="n"/>
+      <c r="G49" s="26" t="n"/>
+      <c r="H49" s="70" t="n"/>
+    </row>
+    <row r="50" ht="5" customHeight="1">
+      <c r="A50" s="3" t="n"/>
+      <c r="B50" s="3" t="n"/>
+      <c r="C50" s="3" t="n"/>
+      <c r="D50" s="3" t="n"/>
+      <c r="E50" s="3" t="n"/>
+      <c r="F50" s="3" t="n"/>
+      <c r="G50" s="3" t="n"/>
+      <c r="H50" s="3" t="n"/>
+    </row>
+    <row r="51" ht="20" customHeight="1">
+      <c r="A51" s="3" t="n"/>
+      <c r="B51" s="71" t="inlineStr">
         <is>
           <t xml:space="preserve">  📝 面談メモ・お客様の声</t>
         </is>
       </c>
-      <c r="C46" s="8" t="n"/>
-      <c r="D46" s="8" t="n"/>
-      <c r="E46" s="8" t="n"/>
-      <c r="F46" s="8" t="n"/>
-      <c r="G46" s="8" t="n"/>
-      <c r="H46" s="35" t="n"/>
-    </row>
-    <row r="47" ht="80" customHeight="1">
-      <c r="A47" s="3" t="n"/>
-      <c r="B47" s="77" t="n"/>
-      <c r="C47" s="12" t="n"/>
-      <c r="D47" s="12" t="n"/>
-      <c r="E47" s="12" t="n"/>
-      <c r="F47" s="12" t="n"/>
-      <c r="G47" s="12" t="n"/>
-      <c r="H47" s="14" t="n"/>
-    </row>
-    <row r="48" ht="5" customHeight="1">
-      <c r="A48" s="3" t="n"/>
-      <c r="B48" s="62" t="n"/>
-      <c r="C48" s="63" t="n"/>
-      <c r="D48" s="63" t="n"/>
-      <c r="E48" s="63" t="n"/>
-      <c r="F48" s="63" t="n"/>
-      <c r="G48" s="63" t="n"/>
-      <c r="H48" s="64" t="n"/>
-    </row>
-    <row r="49" ht="20" customHeight="1">
-      <c r="A49" s="3" t="n"/>
-      <c r="B49" s="78" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  📌 次回アクション</t>
-        </is>
-      </c>
-      <c r="C49" s="12" t="n"/>
-      <c r="D49" s="12" t="n"/>
-      <c r="E49" s="12" t="n"/>
-      <c r="F49" s="12" t="n"/>
-      <c r="G49" s="12" t="n"/>
-      <c r="H49" s="14" t="n"/>
-    </row>
-    <row r="50" ht="30" customHeight="1">
-      <c r="A50" s="3" t="n"/>
-      <c r="B50" s="79" t="n"/>
-      <c r="C50" s="30" t="n"/>
-      <c r="D50" s="30" t="n"/>
-      <c r="E50" s="30" t="n"/>
-      <c r="F50" s="30" t="n"/>
-      <c r="G50" s="30" t="n"/>
-      <c r="H50" s="80" t="n"/>
-    </row>
-    <row r="51" ht="5" customHeight="1">
-      <c r="A51" s="3" t="n"/>
-      <c r="B51" s="3" t="n"/>
-      <c r="C51" s="3" t="n"/>
-      <c r="D51" s="3" t="n"/>
-      <c r="E51" s="3" t="n"/>
-      <c r="F51" s="3" t="n"/>
-      <c r="G51" s="3" t="n"/>
-      <c r="H51" s="3" t="n"/>
-    </row>
-    <row r="52" ht="16" customHeight="1">
+      <c r="C51" s="7" t="n"/>
+      <c r="D51" s="7" t="n"/>
+      <c r="E51" s="7" t="n"/>
+      <c r="F51" s="7" t="n"/>
+      <c r="G51" s="7" t="n"/>
+      <c r="H51" s="8" t="n"/>
+    </row>
+    <row r="52" ht="75" customHeight="1">
       <c r="A52" s="3" t="n"/>
-      <c r="B52" s="81" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ＊本シートは比較推奨規制対応の意向確認記録として活用してください。面談後は保存・アーカイブをお願いします。</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="16" customHeight="1">
+      <c r="B52" s="72" t="n"/>
+      <c r="C52" s="26" t="n"/>
+      <c r="D52" s="26" t="n"/>
+      <c r="E52" s="26" t="n"/>
+      <c r="F52" s="26" t="n"/>
+      <c r="G52" s="26" t="n"/>
+      <c r="H52" s="27" t="n"/>
+    </row>
+    <row r="53" ht="5" customHeight="1">
       <c r="A53" s="3" t="n"/>
       <c r="B53" s="3" t="n"/>
       <c r="C53" s="3" t="n"/>
@@ -1968,27 +2012,31 @@
       <c r="G53" s="3" t="n"/>
       <c r="H53" s="3" t="n"/>
     </row>
-    <row r="54" ht="16" customHeight="1">
+    <row r="54" ht="20" customHeight="1">
       <c r="A54" s="3" t="n"/>
-      <c r="B54" s="3" t="n"/>
-      <c r="C54" s="3" t="n"/>
-      <c r="D54" s="3" t="n"/>
-      <c r="E54" s="3" t="n"/>
-      <c r="F54" s="3" t="n"/>
-      <c r="G54" s="3" t="n"/>
-      <c r="H54" s="3" t="n"/>
-    </row>
-    <row r="55" ht="16" customHeight="1">
+      <c r="B54" s="71" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  📌 次回アクション</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="n"/>
+      <c r="D54" s="7" t="n"/>
+      <c r="E54" s="7" t="n"/>
+      <c r="F54" s="7" t="n"/>
+      <c r="G54" s="7" t="n"/>
+      <c r="H54" s="8" t="n"/>
+    </row>
+    <row r="55" ht="30" customHeight="1">
       <c r="A55" s="3" t="n"/>
-      <c r="B55" s="3" t="n"/>
-      <c r="C55" s="3" t="n"/>
-      <c r="D55" s="3" t="n"/>
-      <c r="E55" s="3" t="n"/>
-      <c r="F55" s="3" t="n"/>
-      <c r="G55" s="3" t="n"/>
-      <c r="H55" s="3" t="n"/>
-    </row>
-    <row r="56" ht="16" customHeight="1">
+      <c r="B55" s="72" t="n"/>
+      <c r="C55" s="26" t="n"/>
+      <c r="D55" s="26" t="n"/>
+      <c r="E55" s="26" t="n"/>
+      <c r="F55" s="26" t="n"/>
+      <c r="G55" s="26" t="n"/>
+      <c r="H55" s="27" t="n"/>
+    </row>
+    <row r="56" ht="5" customHeight="1">
       <c r="A56" s="3" t="n"/>
       <c r="B56" s="3" t="n"/>
       <c r="C56" s="3" t="n"/>
@@ -2000,13 +2048,11 @@
     </row>
     <row r="57" ht="16" customHeight="1">
       <c r="A57" s="3" t="n"/>
-      <c r="B57" s="3" t="n"/>
-      <c r="C57" s="3" t="n"/>
-      <c r="D57" s="3" t="n"/>
-      <c r="E57" s="3" t="n"/>
-      <c r="F57" s="3" t="n"/>
-      <c r="G57" s="3" t="n"/>
-      <c r="H57" s="3" t="n"/>
+      <c r="B57" s="73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ＊本シートは比較推奨規制対応の意向確認記録として活用してください。面談後は必ず保存・アーカイブをお願いします。</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="16" customHeight="1">
       <c r="A58" s="3" t="n"/>
@@ -2728,84 +2774,301 @@
       <c r="G129" s="3" t="n"/>
       <c r="H129" s="3" t="n"/>
     </row>
+    <row r="130" ht="16" customHeight="1">
+      <c r="A130" s="3" t="n"/>
+      <c r="B130" s="3" t="n"/>
+      <c r="C130" s="3" t="n"/>
+      <c r="D130" s="3" t="n"/>
+      <c r="E130" s="3" t="n"/>
+      <c r="F130" s="3" t="n"/>
+      <c r="G130" s="3" t="n"/>
+      <c r="H130" s="3" t="n"/>
+    </row>
+    <row r="131" ht="16" customHeight="1">
+      <c r="A131" s="3" t="n"/>
+      <c r="B131" s="3" t="n"/>
+      <c r="C131" s="3" t="n"/>
+      <c r="D131" s="3" t="n"/>
+      <c r="E131" s="3" t="n"/>
+      <c r="F131" s="3" t="n"/>
+      <c r="G131" s="3" t="n"/>
+      <c r="H131" s="3" t="n"/>
+    </row>
+    <row r="132" ht="16" customHeight="1">
+      <c r="A132" s="3" t="n"/>
+      <c r="B132" s="3" t="n"/>
+      <c r="C132" s="3" t="n"/>
+      <c r="D132" s="3" t="n"/>
+      <c r="E132" s="3" t="n"/>
+      <c r="F132" s="3" t="n"/>
+      <c r="G132" s="3" t="n"/>
+      <c r="H132" s="3" t="n"/>
+    </row>
+    <row r="133" ht="16" customHeight="1">
+      <c r="A133" s="3" t="n"/>
+      <c r="B133" s="3" t="n"/>
+      <c r="C133" s="3" t="n"/>
+      <c r="D133" s="3" t="n"/>
+      <c r="E133" s="3" t="n"/>
+      <c r="F133" s="3" t="n"/>
+      <c r="G133" s="3" t="n"/>
+      <c r="H133" s="3" t="n"/>
+    </row>
+    <row r="134" ht="16" customHeight="1">
+      <c r="A134" s="3" t="n"/>
+      <c r="B134" s="3" t="n"/>
+      <c r="C134" s="3" t="n"/>
+      <c r="D134" s="3" t="n"/>
+      <c r="E134" s="3" t="n"/>
+      <c r="F134" s="3" t="n"/>
+      <c r="G134" s="3" t="n"/>
+      <c r="H134" s="3" t="n"/>
+    </row>
+    <row r="135" ht="16" customHeight="1">
+      <c r="A135" s="3" t="n"/>
+      <c r="B135" s="3" t="n"/>
+      <c r="C135" s="3" t="n"/>
+      <c r="D135" s="3" t="n"/>
+      <c r="E135" s="3" t="n"/>
+      <c r="F135" s="3" t="n"/>
+      <c r="G135" s="3" t="n"/>
+      <c r="H135" s="3" t="n"/>
+    </row>
+    <row r="136" ht="16" customHeight="1">
+      <c r="A136" s="3" t="n"/>
+      <c r="B136" s="3" t="n"/>
+      <c r="C136" s="3" t="n"/>
+      <c r="D136" s="3" t="n"/>
+      <c r="E136" s="3" t="n"/>
+      <c r="F136" s="3" t="n"/>
+      <c r="G136" s="3" t="n"/>
+      <c r="H136" s="3" t="n"/>
+    </row>
+    <row r="137" ht="16" customHeight="1">
+      <c r="A137" s="3" t="n"/>
+      <c r="B137" s="3" t="n"/>
+      <c r="C137" s="3" t="n"/>
+      <c r="D137" s="3" t="n"/>
+      <c r="E137" s="3" t="n"/>
+      <c r="F137" s="3" t="n"/>
+      <c r="G137" s="3" t="n"/>
+      <c r="H137" s="3" t="n"/>
+    </row>
+    <row r="138" ht="16" customHeight="1">
+      <c r="A138" s="3" t="n"/>
+      <c r="B138" s="3" t="n"/>
+      <c r="C138" s="3" t="n"/>
+      <c r="D138" s="3" t="n"/>
+      <c r="E138" s="3" t="n"/>
+      <c r="F138" s="3" t="n"/>
+      <c r="G138" s="3" t="n"/>
+      <c r="H138" s="3" t="n"/>
+    </row>
+    <row r="139" ht="16" customHeight="1">
+      <c r="A139" s="3" t="n"/>
+      <c r="B139" s="3" t="n"/>
+      <c r="C139" s="3" t="n"/>
+      <c r="D139" s="3" t="n"/>
+      <c r="E139" s="3" t="n"/>
+      <c r="F139" s="3" t="n"/>
+      <c r="G139" s="3" t="n"/>
+      <c r="H139" s="3" t="n"/>
+    </row>
+    <row r="140" ht="16" customHeight="1">
+      <c r="A140" s="3" t="n"/>
+      <c r="B140" s="3" t="n"/>
+      <c r="C140" s="3" t="n"/>
+      <c r="D140" s="3" t="n"/>
+      <c r="E140" s="3" t="n"/>
+      <c r="F140" s="3" t="n"/>
+      <c r="G140" s="3" t="n"/>
+      <c r="H140" s="3" t="n"/>
+    </row>
+    <row r="141" ht="16" customHeight="1">
+      <c r="A141" s="3" t="n"/>
+      <c r="B141" s="3" t="n"/>
+      <c r="C141" s="3" t="n"/>
+      <c r="D141" s="3" t="n"/>
+      <c r="E141" s="3" t="n"/>
+      <c r="F141" s="3" t="n"/>
+      <c r="G141" s="3" t="n"/>
+      <c r="H141" s="3" t="n"/>
+    </row>
+    <row r="142" ht="16" customHeight="1">
+      <c r="A142" s="3" t="n"/>
+      <c r="B142" s="3" t="n"/>
+      <c r="C142" s="3" t="n"/>
+      <c r="D142" s="3" t="n"/>
+      <c r="E142" s="3" t="n"/>
+      <c r="F142" s="3" t="n"/>
+      <c r="G142" s="3" t="n"/>
+      <c r="H142" s="3" t="n"/>
+    </row>
+    <row r="143" ht="16" customHeight="1">
+      <c r="A143" s="3" t="n"/>
+      <c r="B143" s="3" t="n"/>
+      <c r="C143" s="3" t="n"/>
+      <c r="D143" s="3" t="n"/>
+      <c r="E143" s="3" t="n"/>
+      <c r="F143" s="3" t="n"/>
+      <c r="G143" s="3" t="n"/>
+      <c r="H143" s="3" t="n"/>
+    </row>
+    <row r="144" ht="16" customHeight="1">
+      <c r="A144" s="3" t="n"/>
+      <c r="B144" s="3" t="n"/>
+      <c r="C144" s="3" t="n"/>
+      <c r="D144" s="3" t="n"/>
+      <c r="E144" s="3" t="n"/>
+      <c r="F144" s="3" t="n"/>
+      <c r="G144" s="3" t="n"/>
+      <c r="H144" s="3" t="n"/>
+    </row>
+    <row r="145" ht="16" customHeight="1">
+      <c r="A145" s="3" t="n"/>
+      <c r="B145" s="3" t="n"/>
+      <c r="C145" s="3" t="n"/>
+      <c r="D145" s="3" t="n"/>
+      <c r="E145" s="3" t="n"/>
+      <c r="F145" s="3" t="n"/>
+      <c r="G145" s="3" t="n"/>
+      <c r="H145" s="3" t="n"/>
+    </row>
+    <row r="146" ht="16" customHeight="1">
+      <c r="A146" s="3" t="n"/>
+      <c r="B146" s="3" t="n"/>
+      <c r="C146" s="3" t="n"/>
+      <c r="D146" s="3" t="n"/>
+      <c r="E146" s="3" t="n"/>
+      <c r="F146" s="3" t="n"/>
+      <c r="G146" s="3" t="n"/>
+      <c r="H146" s="3" t="n"/>
+    </row>
+    <row r="147" ht="16" customHeight="1">
+      <c r="A147" s="3" t="n"/>
+      <c r="B147" s="3" t="n"/>
+      <c r="C147" s="3" t="n"/>
+      <c r="D147" s="3" t="n"/>
+      <c r="E147" s="3" t="n"/>
+      <c r="F147" s="3" t="n"/>
+      <c r="G147" s="3" t="n"/>
+      <c r="H147" s="3" t="n"/>
+    </row>
+    <row r="148" ht="16" customHeight="1">
+      <c r="A148" s="3" t="n"/>
+      <c r="B148" s="3" t="n"/>
+      <c r="C148" s="3" t="n"/>
+      <c r="D148" s="3" t="n"/>
+      <c r="E148" s="3" t="n"/>
+      <c r="F148" s="3" t="n"/>
+      <c r="G148" s="3" t="n"/>
+      <c r="H148" s="3" t="n"/>
+    </row>
+    <row r="149" ht="16" customHeight="1">
+      <c r="A149" s="3" t="n"/>
+      <c r="B149" s="3" t="n"/>
+      <c r="C149" s="3" t="n"/>
+      <c r="D149" s="3" t="n"/>
+      <c r="E149" s="3" t="n"/>
+      <c r="F149" s="3" t="n"/>
+      <c r="G149" s="3" t="n"/>
+      <c r="H149" s="3" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="63">
-    <mergeCell ref="F20:H20"/>
-    <mergeCell ref="B7:F7"/>
-    <mergeCell ref="C20:E20"/>
-    <mergeCell ref="F21:H21"/>
+  <mergeCells count="71">
+    <mergeCell ref="C23:F23"/>
+    <mergeCell ref="B40:H40"/>
     <mergeCell ref="F29:G29"/>
-    <mergeCell ref="D12:G12"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="B49:H49"/>
-    <mergeCell ref="C22:E22"/>
+    <mergeCell ref="G20"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="B55:H55"/>
     <mergeCell ref="B15:E15"/>
-    <mergeCell ref="B31:C31"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="B18:C18"/>
-    <mergeCell ref="C21:E21"/>
-    <mergeCell ref="B27:C27"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="F23:H23"/>
-    <mergeCell ref="B36:H36"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="B50:H50"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="F22:H22"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="B51:H51"/>
+    <mergeCell ref="G22"/>
+    <mergeCell ref="B43:C43"/>
     <mergeCell ref="B26:H26"/>
-    <mergeCell ref="C23:E23"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="D27:H27"/>
-    <mergeCell ref="B47:H47"/>
+    <mergeCell ref="C27:E27"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="D11:H11"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="G21"/>
     <mergeCell ref="B16:H16"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="B7:H7"/>
     <mergeCell ref="B17:C17"/>
+    <mergeCell ref="C24:F24"/>
+    <mergeCell ref="D32:H32"/>
     <mergeCell ref="B8:C8"/>
+    <mergeCell ref="D41:H41"/>
+    <mergeCell ref="B54:H54"/>
+    <mergeCell ref="F35:G35"/>
     <mergeCell ref="D17:H17"/>
-    <mergeCell ref="B46:H46"/>
-    <mergeCell ref="D40:G40"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B31:H31"/>
+    <mergeCell ref="G23"/>
+    <mergeCell ref="C28:E28"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="D43:H43"/>
     <mergeCell ref="B52:H52"/>
     <mergeCell ref="B10:F10"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="B19:C19"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="D37:H37"/>
+    <mergeCell ref="C20:F20"/>
+    <mergeCell ref="B34:C34"/>
+    <mergeCell ref="B48:H48"/>
     <mergeCell ref="F28:G28"/>
-    <mergeCell ref="D11:G11"/>
-    <mergeCell ref="D13:G13"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="D49:G49"/>
     <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="G10"/>
+    <mergeCell ref="F27:G27"/>
     <mergeCell ref="D18:H18"/>
+    <mergeCell ref="B49:C49"/>
     <mergeCell ref="D9:H9"/>
-    <mergeCell ref="C24:E24"/>
-    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="C22:F22"/>
+    <mergeCell ref="D12:H12"/>
+    <mergeCell ref="D19:F19"/>
     <mergeCell ref="D8:H8"/>
-    <mergeCell ref="D39:H39"/>
-    <mergeCell ref="F19:H19"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="D38:H38"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="B57:H57"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="D42:H42"/>
+    <mergeCell ref="C21:F21"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="G24"/>
+    <mergeCell ref="C29:E29"/>
     <mergeCell ref="B41:C41"/>
+    <mergeCell ref="F44:G44"/>
     <mergeCell ref="F15:H15"/>
-    <mergeCell ref="F24:H24"/>
+    <mergeCell ref="B35:C35"/>
+    <mergeCell ref="D35:E35"/>
   </mergeCells>
-  <dataValidations count="4">
-    <dataValidation sqref="H7 H10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+  <dataValidations count="7">
+    <dataValidation sqref="H10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"①給与天引き（団体割引）,②一般契約（クレカ・口振）,③通販型（ソニー損保）"</formula1>
     </dataValidation>
     <dataValidation sqref="H20 H21 H22 H23 H24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"○,−"</formula1>
     </dataValidation>
-    <dataValidation sqref="H29 H30 H31" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H27" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"ご希望あり,検討中,不要"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H28" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"本人のみ,家族限定,限定なし"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"5,000km未満,〜10,000km,10,000km超"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H34 H35 H36" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"◎提案する,○提案する,△保留,×見送り"</formula1>
     </dataValidation>
-    <dataValidation sqref="H40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"はい（取り次ぎ確定）,再検討（3社も比較）,見送り"</formula1>
+    <dataValidation sqref="H44" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"はい（取り次ぎ確定）,再検討（3社比較に戻る）,見送り"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2818,7 +3081,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G59"/>
+  <dimension ref="A1:G69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2833,635 +3096,732 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ■ 比較推奨チェックリスト（金融庁指針対応）</t>
+          <t xml:space="preserve">  ■ 比較推奨チェックリスト（改正保険業法対応・金融庁指針準拠）</t>
         </is>
       </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">  面談前後に確認し、すべて「✅ 済」になっていることを確認してください。</t>
+          <t xml:space="preserve">  面談後に全項目を確認し、すべて「✅ 済」になっていることを確認してください。</t>
         </is>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="82" t="n"/>
-      <c r="B3" s="82" t="n"/>
-      <c r="C3" s="83" t="inlineStr">
+      <c r="A3" s="74" t="n"/>
+      <c r="B3" s="74" t="n"/>
+      <c r="C3" s="75" t="inlineStr">
         <is>
           <t xml:space="preserve">  確認項目</t>
         </is>
       </c>
-      <c r="E3" s="84" t="inlineStr">
+      <c r="E3" s="76" t="inlineStr">
         <is>
           <t>SJ</t>
         </is>
       </c>
-      <c r="F3" s="84" t="inlineStr">
+      <c r="F3" s="76" t="inlineStr">
         <is>
           <t>MSI</t>
         </is>
       </c>
-      <c r="G3" s="84" t="inlineStr">
+      <c r="G3" s="76" t="inlineStr">
         <is>
           <t>TN</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="A4" s="82" t="n"/>
-      <c r="B4" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  【 事前確認 】</t>
+      <c r="A4" s="74" t="n"/>
+      <c r="B4" s="77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  【 ① 事前確認（意向把握） 】</t>
         </is>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="82" t="n"/>
-      <c r="B5" s="86" t="inlineStr">
+      <c r="A5" s="74" t="n"/>
+      <c r="B5" s="78" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C5" s="87" t="inlineStr">
+      <c r="C5" s="79" t="inlineStr">
         <is>
           <t xml:space="preserve">  お客様の意向（重視事項）を確認した</t>
         </is>
       </c>
-      <c r="E5" s="88" t="n"/>
-      <c r="F5" s="89" t="n"/>
-      <c r="G5" s="89" t="n"/>
+      <c r="E5" s="80" t="n"/>
+      <c r="F5" s="80" t="n"/>
+      <c r="G5" s="80" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="82" t="n"/>
-      <c r="B6" s="86" t="inlineStr">
+      <c r="A6" s="74" t="n"/>
+      <c r="B6" s="78" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C6" s="87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  複数社（原則3社）の見積りを取得した</t>
-        </is>
-      </c>
-      <c r="E6" s="88" t="n"/>
-      <c r="F6" s="89" t="n"/>
-      <c r="G6" s="89" t="n"/>
+      <c r="C6" s="79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  補償内容の希望（車両保険・運転者範囲等）を確認した</t>
+        </is>
+      </c>
+      <c r="E6" s="80" t="n"/>
+      <c r="F6" s="80" t="n"/>
+      <c r="G6" s="80" t="n"/>
     </row>
     <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="82" t="n"/>
-      <c r="B7" s="86" t="inlineStr">
+      <c r="A7" s="74" t="n"/>
+      <c r="B7" s="78" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C7" s="87" t="inlineStr">
+      <c r="C7" s="79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  複数社（3社）の見積りを取得した</t>
+        </is>
+      </c>
+      <c r="E7" s="80" t="n"/>
+      <c r="F7" s="80" t="n"/>
+      <c r="G7" s="80" t="n"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="74" t="n"/>
+      <c r="B8" s="78" t="inlineStr">
+        <is>
+          <t>▸</t>
+        </is>
+      </c>
+      <c r="C8" s="79" t="inlineStr">
         <is>
           <t xml:space="preserve">  各社の保険料・補償内容を比較説明した</t>
         </is>
       </c>
-      <c r="E7" s="88" t="n"/>
-      <c r="F7" s="89" t="n"/>
-      <c r="G7" s="89" t="n"/>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="82" t="n"/>
-      <c r="B8" s="86" t="inlineStr">
+      <c r="E8" s="80" t="n"/>
+      <c r="F8" s="80" t="n"/>
+      <c r="G8" s="80" t="n"/>
+    </row>
+    <row r="9" ht="4" customHeight="1">
+      <c r="A9" s="74" t="n"/>
+      <c r="B9" s="74" t="n"/>
+      <c r="C9" s="74" t="n"/>
+      <c r="D9" s="74" t="n"/>
+      <c r="E9" s="74" t="n"/>
+      <c r="F9" s="74" t="n"/>
+      <c r="G9" s="74" t="n"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="74" t="n"/>
+      <c r="B10" s="77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  【 ② 比較推奨の実施 】</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="74" t="n"/>
+      <c r="B11" s="81" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C8" s="87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  比較に用いた基準・理由を説明できる</t>
-        </is>
-      </c>
-      <c r="E8" s="88" t="n"/>
-      <c r="F8" s="89" t="n"/>
-      <c r="G8" s="89" t="n"/>
-    </row>
-    <row r="9" ht="4" customHeight="1">
-      <c r="A9" s="82" t="n"/>
-      <c r="B9" s="82" t="n"/>
-      <c r="C9" s="82" t="n"/>
-      <c r="D9" s="82" t="n"/>
-      <c r="E9" s="82" t="n"/>
-      <c r="F9" s="82" t="n"/>
-      <c r="G9" s="82" t="n"/>
-    </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="A10" s="82" t="n"/>
-      <c r="B10" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  【 三井住友海上の提案 】</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="82" t="n"/>
-      <c r="B11" s="90" t="inlineStr">
+      <c r="C11" s="79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  お客様の意向に照らして比較対象3社を選定し、選定理由を説明できる</t>
+        </is>
+      </c>
+      <c r="E11" s="82" t="n"/>
+      <c r="F11" s="82" t="n"/>
+      <c r="G11" s="82" t="n"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="74" t="n"/>
+      <c r="B12" s="81" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C11" s="87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  三井住友海上の見積りを必ず含めた</t>
-        </is>
-      </c>
-      <c r="E11" s="91" t="n"/>
-      <c r="F11" s="89" t="n"/>
-      <c r="G11" s="89" t="n"/>
-    </row>
-    <row r="12" ht="20" customHeight="1">
-      <c r="A12" s="82" t="n"/>
-      <c r="B12" s="90" t="inlineStr">
+      <c r="C12" s="79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  各社の特徴・強みをお客様の意向と紐づけて説明した</t>
+        </is>
+      </c>
+      <c r="E12" s="82" t="n"/>
+      <c r="F12" s="82" t="n"/>
+      <c r="G12" s="82" t="n"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="74" t="n"/>
+      <c r="B13" s="81" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C12" s="87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  損保ジャパンとの比較ポイントを説明した</t>
-        </is>
-      </c>
-      <c r="E12" s="91" t="n"/>
-      <c r="F12" s="89" t="n"/>
-      <c r="G12" s="89" t="n"/>
-    </row>
-    <row r="13" ht="20" customHeight="1">
-      <c r="A13" s="82" t="n"/>
-      <c r="B13" s="90" t="inlineStr">
+      <c r="C13" s="79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  推奨・非推奨の根拠が顧客の意向に基づいていることを確認した</t>
+        </is>
+      </c>
+      <c r="E13" s="82" t="n"/>
+      <c r="F13" s="82" t="n"/>
+      <c r="G13" s="82" t="n"/>
+    </row>
+    <row r="14" ht="4" customHeight="1">
+      <c r="A14" s="74" t="n"/>
+      <c r="B14" s="74" t="n"/>
+      <c r="C14" s="74" t="n"/>
+      <c r="D14" s="74" t="n"/>
+      <c r="E14" s="74" t="n"/>
+      <c r="F14" s="74" t="n"/>
+      <c r="G14" s="74" t="n"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="74" t="n"/>
+      <c r="B15" s="77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  【 ③ 推奨根拠の記録 】</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="74" t="n"/>
+      <c r="B16" s="83" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C13" s="87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  MSIを選ばない場合、理由を記録した</t>
-        </is>
-      </c>
-      <c r="E13" s="91" t="n"/>
-      <c r="F13" s="89" t="n"/>
-      <c r="G13" s="89" t="n"/>
-    </row>
-    <row r="14" ht="4" customHeight="1">
-      <c r="A14" s="82" t="n"/>
-      <c r="B14" s="82" t="n"/>
-      <c r="C14" s="82" t="n"/>
-      <c r="D14" s="82" t="n"/>
-      <c r="E14" s="82" t="n"/>
-      <c r="F14" s="82" t="n"/>
-      <c r="G14" s="82" t="n"/>
-    </row>
-    <row r="15" ht="20" customHeight="1">
-      <c r="A15" s="82" t="n"/>
-      <c r="B15" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  【 推奨根拠の記録 】</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="A16" s="82" t="n"/>
-      <c r="B16" s="92" t="inlineStr">
+      <c r="C16" s="79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  推奨する会社・商品とその理由を記録した</t>
+        </is>
+      </c>
+      <c r="E16" s="84" t="n"/>
+      <c r="F16" s="84" t="n"/>
+      <c r="G16" s="84" t="n"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="74" t="n"/>
+      <c r="B17" s="83" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C16" s="87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  推奨する会社・商品とその理由を記録した</t>
-        </is>
-      </c>
-      <c r="E16" s="93" t="n"/>
-      <c r="F16" s="89" t="n"/>
-      <c r="G16" s="89" t="n"/>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="A17" s="82" t="n"/>
-      <c r="B17" s="92" t="inlineStr">
+      <c r="C17" s="79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  お客様が選んだ会社・商品を記録した</t>
+        </is>
+      </c>
+      <c r="E17" s="84" t="n"/>
+      <c r="F17" s="84" t="n"/>
+      <c r="G17" s="84" t="n"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="74" t="n"/>
+      <c r="B18" s="83" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C17" s="87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  お客様が選んだ会社・商品を記録した</t>
-        </is>
-      </c>
-      <c r="E17" s="93" t="n"/>
-      <c r="F17" s="89" t="n"/>
-      <c r="G17" s="89" t="n"/>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="A18" s="82" t="n"/>
-      <c r="B18" s="92" t="inlineStr">
+      <c r="C18" s="79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  意向と異なる商品を選択した場合、その理由を確認・記録した</t>
+        </is>
+      </c>
+      <c r="E18" s="84" t="n"/>
+      <c r="F18" s="84" t="n"/>
+      <c r="G18" s="84" t="n"/>
+    </row>
+    <row r="19" ht="4" customHeight="1">
+      <c r="A19" s="74" t="n"/>
+      <c r="B19" s="74" t="n"/>
+      <c r="C19" s="74" t="n"/>
+      <c r="D19" s="74" t="n"/>
+      <c r="E19" s="74" t="n"/>
+      <c r="F19" s="74" t="n"/>
+      <c r="G19" s="74" t="n"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="74" t="n"/>
+      <c r="B20" s="77" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  【 ④ コンプライアンス 】</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="74" t="n"/>
+      <c r="B21" s="85" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C18" s="87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  意向と選択が異なる場合、経緯を記録した</t>
-        </is>
-      </c>
-      <c r="E18" s="93" t="n"/>
-      <c r="F18" s="89" t="n"/>
-      <c r="G18" s="89" t="n"/>
-    </row>
-    <row r="19" ht="4" customHeight="1">
-      <c r="A19" s="82" t="n"/>
-      <c r="B19" s="82" t="n"/>
-      <c r="C19" s="82" t="n"/>
-      <c r="D19" s="82" t="n"/>
-      <c r="E19" s="82" t="n"/>
-      <c r="F19" s="82" t="n"/>
-      <c r="G19" s="82" t="n"/>
-    </row>
-    <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="82" t="n"/>
-      <c r="B20" s="85" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  【 コンプライアンス 】</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="82" t="n"/>
-      <c r="B21" s="94" t="inlineStr">
+      <c r="C21" s="79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  特定会社への一方的な誘導はなく、公平な比較を実施した</t>
+        </is>
+      </c>
+      <c r="E21" s="86" t="n"/>
+      <c r="F21" s="86" t="n"/>
+      <c r="G21" s="86" t="n"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="74" t="n"/>
+      <c r="B22" s="85" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C21" s="87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  特定会社への誘導はない</t>
-        </is>
-      </c>
-      <c r="E21" s="95" t="n"/>
-      <c r="F21" s="89" t="n"/>
-      <c r="G21" s="89" t="n"/>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="82" t="n"/>
-      <c r="B22" s="94" t="inlineStr">
+      <c r="C22" s="79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  意向確認の内容をお客様に読み上げ・確認いただいた</t>
+        </is>
+      </c>
+      <c r="E22" s="86" t="n"/>
+      <c r="F22" s="86" t="n"/>
+      <c r="G22" s="86" t="n"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="74" t="n"/>
+      <c r="B23" s="85" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C22" s="87" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  意向確認の同意を得た</t>
-        </is>
-      </c>
-      <c r="E22" s="95" t="n"/>
-      <c r="F22" s="89" t="n"/>
-      <c r="G22" s="89" t="n"/>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="82" t="n"/>
-      <c r="B23" s="94" t="inlineStr">
+      <c r="C23" s="79" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  推奨内容がお客様の意向に沿うことを口頭で説明した</t>
+        </is>
+      </c>
+      <c r="E23" s="86" t="n"/>
+      <c r="F23" s="86" t="n"/>
+      <c r="G23" s="86" t="n"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="74" t="n"/>
+      <c r="B24" s="85" t="inlineStr">
         <is>
           <t>▸</t>
         </is>
       </c>
-      <c r="C23" s="87" t="inlineStr">
+      <c r="C24" s="79" t="inlineStr">
         <is>
           <t xml:space="preserve">  本シートを保管・アーカイブ予定</t>
         </is>
       </c>
-      <c r="E23" s="95" t="n"/>
-      <c r="F23" s="89" t="n"/>
-      <c r="G23" s="89" t="n"/>
-    </row>
-    <row r="24" ht="4" customHeight="1">
-      <c r="A24" s="82" t="n"/>
-      <c r="B24" s="82" t="n"/>
-      <c r="C24" s="82" t="n"/>
-      <c r="D24" s="82" t="n"/>
-      <c r="E24" s="82" t="n"/>
-      <c r="F24" s="82" t="n"/>
-      <c r="G24" s="82" t="n"/>
-    </row>
-    <row r="25" ht="16" customHeight="1">
-      <c r="A25" s="82" t="n"/>
-      <c r="B25" s="82" t="n"/>
-      <c r="C25" s="82" t="n"/>
-      <c r="D25" s="82" t="n"/>
-      <c r="E25" s="82" t="n"/>
-      <c r="F25" s="82" t="n"/>
-      <c r="G25" s="82" t="n"/>
-    </row>
-    <row r="26" ht="16" customHeight="1">
-      <c r="A26" s="82" t="n"/>
-      <c r="B26" s="82" t="n"/>
-      <c r="C26" s="82" t="n"/>
-      <c r="D26" s="82" t="n"/>
-      <c r="E26" s="82" t="n"/>
-      <c r="F26" s="82" t="n"/>
-      <c r="G26" s="82" t="n"/>
+      <c r="E24" s="86" t="n"/>
+      <c r="F24" s="86" t="n"/>
+      <c r="G24" s="86" t="n"/>
+    </row>
+    <row r="25" ht="4" customHeight="1">
+      <c r="A25" s="74" t="n"/>
+      <c r="B25" s="74" t="n"/>
+      <c r="C25" s="74" t="n"/>
+      <c r="D25" s="74" t="n"/>
+      <c r="E25" s="74" t="n"/>
+      <c r="F25" s="74" t="n"/>
+      <c r="G25" s="74" t="n"/>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="74" t="n"/>
+      <c r="B26" s="73" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ＊推奨根拠は必ず「顧客の意向との対応関係」で記録してください（保険業法施行規則第227条の2）。</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="16" customHeight="1">
-      <c r="A27" s="82" t="n"/>
-      <c r="B27" s="82" t="n"/>
-      <c r="C27" s="82" t="n"/>
-      <c r="D27" s="82" t="n"/>
-      <c r="E27" s="82" t="n"/>
-      <c r="F27" s="82" t="n"/>
-      <c r="G27" s="82" t="n"/>
+      <c r="A27" s="74" t="n"/>
+      <c r="B27" s="74" t="n"/>
+      <c r="C27" s="74" t="n"/>
+      <c r="D27" s="74" t="n"/>
+      <c r="E27" s="74" t="n"/>
+      <c r="F27" s="74" t="n"/>
+      <c r="G27" s="74" t="n"/>
     </row>
     <row r="28" ht="16" customHeight="1">
-      <c r="A28" s="82" t="n"/>
-      <c r="B28" s="82" t="n"/>
-      <c r="C28" s="82" t="n"/>
-      <c r="D28" s="82" t="n"/>
-      <c r="E28" s="82" t="n"/>
-      <c r="F28" s="82" t="n"/>
-      <c r="G28" s="82" t="n"/>
+      <c r="A28" s="74" t="n"/>
+      <c r="B28" s="74" t="n"/>
+      <c r="C28" s="74" t="n"/>
+      <c r="D28" s="74" t="n"/>
+      <c r="E28" s="74" t="n"/>
+      <c r="F28" s="74" t="n"/>
+      <c r="G28" s="74" t="n"/>
     </row>
     <row r="29" ht="16" customHeight="1">
-      <c r="A29" s="82" t="n"/>
-      <c r="B29" s="82" t="n"/>
-      <c r="C29" s="82" t="n"/>
-      <c r="D29" s="82" t="n"/>
-      <c r="E29" s="82" t="n"/>
-      <c r="F29" s="82" t="n"/>
-      <c r="G29" s="82" t="n"/>
+      <c r="A29" s="74" t="n"/>
+      <c r="B29" s="74" t="n"/>
+      <c r="C29" s="74" t="n"/>
+      <c r="D29" s="74" t="n"/>
+      <c r="E29" s="74" t="n"/>
+      <c r="F29" s="74" t="n"/>
+      <c r="G29" s="74" t="n"/>
     </row>
     <row r="30" ht="16" customHeight="1">
-      <c r="A30" s="82" t="n"/>
-      <c r="B30" s="82" t="n"/>
-      <c r="C30" s="82" t="n"/>
-      <c r="D30" s="82" t="n"/>
-      <c r="E30" s="82" t="n"/>
-      <c r="F30" s="82" t="n"/>
-      <c r="G30" s="82" t="n"/>
+      <c r="A30" s="74" t="n"/>
+      <c r="B30" s="74" t="n"/>
+      <c r="C30" s="74" t="n"/>
+      <c r="D30" s="74" t="n"/>
+      <c r="E30" s="74" t="n"/>
+      <c r="F30" s="74" t="n"/>
+      <c r="G30" s="74" t="n"/>
     </row>
     <row r="31" ht="16" customHeight="1">
-      <c r="A31" s="82" t="n"/>
-      <c r="B31" s="82" t="n"/>
-      <c r="C31" s="82" t="n"/>
-      <c r="D31" s="82" t="n"/>
-      <c r="E31" s="82" t="n"/>
-      <c r="F31" s="82" t="n"/>
-      <c r="G31" s="82" t="n"/>
+      <c r="A31" s="74" t="n"/>
+      <c r="B31" s="74" t="n"/>
+      <c r="C31" s="74" t="n"/>
+      <c r="D31" s="74" t="n"/>
+      <c r="E31" s="74" t="n"/>
+      <c r="F31" s="74" t="n"/>
+      <c r="G31" s="74" t="n"/>
     </row>
     <row r="32" ht="16" customHeight="1">
-      <c r="A32" s="82" t="n"/>
-      <c r="B32" s="82" t="n"/>
-      <c r="C32" s="82" t="n"/>
-      <c r="D32" s="82" t="n"/>
-      <c r="E32" s="82" t="n"/>
-      <c r="F32" s="82" t="n"/>
-      <c r="G32" s="82" t="n"/>
+      <c r="A32" s="74" t="n"/>
+      <c r="B32" s="74" t="n"/>
+      <c r="C32" s="74" t="n"/>
+      <c r="D32" s="74" t="n"/>
+      <c r="E32" s="74" t="n"/>
+      <c r="F32" s="74" t="n"/>
+      <c r="G32" s="74" t="n"/>
     </row>
     <row r="33" ht="16" customHeight="1">
-      <c r="A33" s="82" t="n"/>
-      <c r="B33" s="82" t="n"/>
-      <c r="C33" s="82" t="n"/>
-      <c r="D33" s="82" t="n"/>
-      <c r="E33" s="82" t="n"/>
-      <c r="F33" s="82" t="n"/>
-      <c r="G33" s="82" t="n"/>
+      <c r="A33" s="74" t="n"/>
+      <c r="B33" s="74" t="n"/>
+      <c r="C33" s="74" t="n"/>
+      <c r="D33" s="74" t="n"/>
+      <c r="E33" s="74" t="n"/>
+      <c r="F33" s="74" t="n"/>
+      <c r="G33" s="74" t="n"/>
     </row>
     <row r="34" ht="16" customHeight="1">
-      <c r="A34" s="82" t="n"/>
-      <c r="B34" s="82" t="n"/>
-      <c r="C34" s="82" t="n"/>
-      <c r="D34" s="82" t="n"/>
-      <c r="E34" s="82" t="n"/>
-      <c r="F34" s="82" t="n"/>
-      <c r="G34" s="82" t="n"/>
+      <c r="A34" s="74" t="n"/>
+      <c r="B34" s="74" t="n"/>
+      <c r="C34" s="74" t="n"/>
+      <c r="D34" s="74" t="n"/>
+      <c r="E34" s="74" t="n"/>
+      <c r="F34" s="74" t="n"/>
+      <c r="G34" s="74" t="n"/>
     </row>
     <row r="35" ht="16" customHeight="1">
-      <c r="A35" s="82" t="n"/>
-      <c r="B35" s="82" t="n"/>
-      <c r="C35" s="82" t="n"/>
-      <c r="D35" s="82" t="n"/>
-      <c r="E35" s="82" t="n"/>
-      <c r="F35" s="82" t="n"/>
-      <c r="G35" s="82" t="n"/>
+      <c r="A35" s="74" t="n"/>
+      <c r="B35" s="74" t="n"/>
+      <c r="C35" s="74" t="n"/>
+      <c r="D35" s="74" t="n"/>
+      <c r="E35" s="74" t="n"/>
+      <c r="F35" s="74" t="n"/>
+      <c r="G35" s="74" t="n"/>
     </row>
     <row r="36" ht="16" customHeight="1">
-      <c r="A36" s="82" t="n"/>
-      <c r="B36" s="82" t="n"/>
-      <c r="C36" s="82" t="n"/>
-      <c r="D36" s="82" t="n"/>
-      <c r="E36" s="82" t="n"/>
-      <c r="F36" s="82" t="n"/>
-      <c r="G36" s="82" t="n"/>
+      <c r="A36" s="74" t="n"/>
+      <c r="B36" s="74" t="n"/>
+      <c r="C36" s="74" t="n"/>
+      <c r="D36" s="74" t="n"/>
+      <c r="E36" s="74" t="n"/>
+      <c r="F36" s="74" t="n"/>
+      <c r="G36" s="74" t="n"/>
     </row>
     <row r="37" ht="16" customHeight="1">
-      <c r="A37" s="82" t="n"/>
-      <c r="B37" s="82" t="n"/>
-      <c r="C37" s="82" t="n"/>
-      <c r="D37" s="82" t="n"/>
-      <c r="E37" s="82" t="n"/>
-      <c r="F37" s="82" t="n"/>
-      <c r="G37" s="82" t="n"/>
+      <c r="A37" s="74" t="n"/>
+      <c r="B37" s="74" t="n"/>
+      <c r="C37" s="74" t="n"/>
+      <c r="D37" s="74" t="n"/>
+      <c r="E37" s="74" t="n"/>
+      <c r="F37" s="74" t="n"/>
+      <c r="G37" s="74" t="n"/>
     </row>
     <row r="38" ht="16" customHeight="1">
-      <c r="A38" s="82" t="n"/>
-      <c r="B38" s="82" t="n"/>
-      <c r="C38" s="82" t="n"/>
-      <c r="D38" s="82" t="n"/>
-      <c r="E38" s="82" t="n"/>
-      <c r="F38" s="82" t="n"/>
-      <c r="G38" s="82" t="n"/>
+      <c r="A38" s="74" t="n"/>
+      <c r="B38" s="74" t="n"/>
+      <c r="C38" s="74" t="n"/>
+      <c r="D38" s="74" t="n"/>
+      <c r="E38" s="74" t="n"/>
+      <c r="F38" s="74" t="n"/>
+      <c r="G38" s="74" t="n"/>
     </row>
     <row r="39" ht="16" customHeight="1">
-      <c r="A39" s="82" t="n"/>
-      <c r="B39" s="82" t="n"/>
-      <c r="C39" s="82" t="n"/>
-      <c r="D39" s="82" t="n"/>
-      <c r="E39" s="82" t="n"/>
-      <c r="F39" s="82" t="n"/>
-      <c r="G39" s="82" t="n"/>
+      <c r="A39" s="74" t="n"/>
+      <c r="B39" s="74" t="n"/>
+      <c r="C39" s="74" t="n"/>
+      <c r="D39" s="74" t="n"/>
+      <c r="E39" s="74" t="n"/>
+      <c r="F39" s="74" t="n"/>
+      <c r="G39" s="74" t="n"/>
     </row>
     <row r="40" ht="16" customHeight="1">
-      <c r="A40" s="82" t="n"/>
-      <c r="B40" s="82" t="n"/>
-      <c r="C40" s="82" t="n"/>
-      <c r="D40" s="82" t="n"/>
-      <c r="E40" s="82" t="n"/>
-      <c r="F40" s="82" t="n"/>
-      <c r="G40" s="82" t="n"/>
+      <c r="A40" s="74" t="n"/>
+      <c r="B40" s="74" t="n"/>
+      <c r="C40" s="74" t="n"/>
+      <c r="D40" s="74" t="n"/>
+      <c r="E40" s="74" t="n"/>
+      <c r="F40" s="74" t="n"/>
+      <c r="G40" s="74" t="n"/>
     </row>
     <row r="41" ht="16" customHeight="1">
-      <c r="A41" s="82" t="n"/>
-      <c r="B41" s="82" t="n"/>
-      <c r="C41" s="82" t="n"/>
-      <c r="D41" s="82" t="n"/>
-      <c r="E41" s="82" t="n"/>
-      <c r="F41" s="82" t="n"/>
-      <c r="G41" s="82" t="n"/>
+      <c r="A41" s="74" t="n"/>
+      <c r="B41" s="74" t="n"/>
+      <c r="C41" s="74" t="n"/>
+      <c r="D41" s="74" t="n"/>
+      <c r="E41" s="74" t="n"/>
+      <c r="F41" s="74" t="n"/>
+      <c r="G41" s="74" t="n"/>
     </row>
     <row r="42" ht="16" customHeight="1">
-      <c r="A42" s="82" t="n"/>
-      <c r="B42" s="82" t="n"/>
-      <c r="C42" s="82" t="n"/>
-      <c r="D42" s="82" t="n"/>
-      <c r="E42" s="82" t="n"/>
-      <c r="F42" s="82" t="n"/>
-      <c r="G42" s="82" t="n"/>
+      <c r="A42" s="74" t="n"/>
+      <c r="B42" s="74" t="n"/>
+      <c r="C42" s="74" t="n"/>
+      <c r="D42" s="74" t="n"/>
+      <c r="E42" s="74" t="n"/>
+      <c r="F42" s="74" t="n"/>
+      <c r="G42" s="74" t="n"/>
     </row>
     <row r="43" ht="16" customHeight="1">
-      <c r="A43" s="82" t="n"/>
-      <c r="B43" s="82" t="n"/>
-      <c r="C43" s="82" t="n"/>
-      <c r="D43" s="82" t="n"/>
-      <c r="E43" s="82" t="n"/>
-      <c r="F43" s="82" t="n"/>
-      <c r="G43" s="82" t="n"/>
+      <c r="A43" s="74" t="n"/>
+      <c r="B43" s="74" t="n"/>
+      <c r="C43" s="74" t="n"/>
+      <c r="D43" s="74" t="n"/>
+      <c r="E43" s="74" t="n"/>
+      <c r="F43" s="74" t="n"/>
+      <c r="G43" s="74" t="n"/>
     </row>
     <row r="44" ht="16" customHeight="1">
-      <c r="A44" s="82" t="n"/>
-      <c r="B44" s="82" t="n"/>
-      <c r="C44" s="82" t="n"/>
-      <c r="D44" s="82" t="n"/>
-      <c r="E44" s="82" t="n"/>
-      <c r="F44" s="82" t="n"/>
-      <c r="G44" s="82" t="n"/>
+      <c r="A44" s="74" t="n"/>
+      <c r="B44" s="74" t="n"/>
+      <c r="C44" s="74" t="n"/>
+      <c r="D44" s="74" t="n"/>
+      <c r="E44" s="74" t="n"/>
+      <c r="F44" s="74" t="n"/>
+      <c r="G44" s="74" t="n"/>
     </row>
     <row r="45" ht="16" customHeight="1">
-      <c r="A45" s="82" t="n"/>
-      <c r="B45" s="82" t="n"/>
-      <c r="C45" s="82" t="n"/>
-      <c r="D45" s="82" t="n"/>
-      <c r="E45" s="82" t="n"/>
-      <c r="F45" s="82" t="n"/>
-      <c r="G45" s="82" t="n"/>
+      <c r="A45" s="74" t="n"/>
+      <c r="B45" s="74" t="n"/>
+      <c r="C45" s="74" t="n"/>
+      <c r="D45" s="74" t="n"/>
+      <c r="E45" s="74" t="n"/>
+      <c r="F45" s="74" t="n"/>
+      <c r="G45" s="74" t="n"/>
     </row>
     <row r="46" ht="16" customHeight="1">
-      <c r="A46" s="82" t="n"/>
-      <c r="B46" s="82" t="n"/>
-      <c r="C46" s="82" t="n"/>
-      <c r="D46" s="82" t="n"/>
-      <c r="E46" s="82" t="n"/>
-      <c r="F46" s="82" t="n"/>
-      <c r="G46" s="82" t="n"/>
+      <c r="A46" s="74" t="n"/>
+      <c r="B46" s="74" t="n"/>
+      <c r="C46" s="74" t="n"/>
+      <c r="D46" s="74" t="n"/>
+      <c r="E46" s="74" t="n"/>
+      <c r="F46" s="74" t="n"/>
+      <c r="G46" s="74" t="n"/>
     </row>
     <row r="47" ht="16" customHeight="1">
-      <c r="A47" s="82" t="n"/>
-      <c r="B47" s="82" t="n"/>
-      <c r="C47" s="82" t="n"/>
-      <c r="D47" s="82" t="n"/>
-      <c r="E47" s="82" t="n"/>
-      <c r="F47" s="82" t="n"/>
-      <c r="G47" s="82" t="n"/>
+      <c r="A47" s="74" t="n"/>
+      <c r="B47" s="74" t="n"/>
+      <c r="C47" s="74" t="n"/>
+      <c r="D47" s="74" t="n"/>
+      <c r="E47" s="74" t="n"/>
+      <c r="F47" s="74" t="n"/>
+      <c r="G47" s="74" t="n"/>
     </row>
     <row r="48" ht="16" customHeight="1">
-      <c r="A48" s="82" t="n"/>
-      <c r="B48" s="82" t="n"/>
-      <c r="C48" s="82" t="n"/>
-      <c r="D48" s="82" t="n"/>
-      <c r="E48" s="82" t="n"/>
-      <c r="F48" s="82" t="n"/>
-      <c r="G48" s="82" t="n"/>
+      <c r="A48" s="74" t="n"/>
+      <c r="B48" s="74" t="n"/>
+      <c r="C48" s="74" t="n"/>
+      <c r="D48" s="74" t="n"/>
+      <c r="E48" s="74" t="n"/>
+      <c r="F48" s="74" t="n"/>
+      <c r="G48" s="74" t="n"/>
     </row>
     <row r="49" ht="16" customHeight="1">
-      <c r="A49" s="82" t="n"/>
-      <c r="B49" s="82" t="n"/>
-      <c r="C49" s="82" t="n"/>
-      <c r="D49" s="82" t="n"/>
-      <c r="E49" s="82" t="n"/>
-      <c r="F49" s="82" t="n"/>
-      <c r="G49" s="82" t="n"/>
+      <c r="A49" s="74" t="n"/>
+      <c r="B49" s="74" t="n"/>
+      <c r="C49" s="74" t="n"/>
+      <c r="D49" s="74" t="n"/>
+      <c r="E49" s="74" t="n"/>
+      <c r="F49" s="74" t="n"/>
+      <c r="G49" s="74" t="n"/>
     </row>
     <row r="50" ht="16" customHeight="1">
-      <c r="A50" s="82" t="n"/>
-      <c r="B50" s="82" t="n"/>
-      <c r="C50" s="82" t="n"/>
-      <c r="D50" s="82" t="n"/>
-      <c r="E50" s="82" t="n"/>
-      <c r="F50" s="82" t="n"/>
-      <c r="G50" s="82" t="n"/>
+      <c r="A50" s="74" t="n"/>
+      <c r="B50" s="74" t="n"/>
+      <c r="C50" s="74" t="n"/>
+      <c r="D50" s="74" t="n"/>
+      <c r="E50" s="74" t="n"/>
+      <c r="F50" s="74" t="n"/>
+      <c r="G50" s="74" t="n"/>
     </row>
     <row r="51" ht="16" customHeight="1">
-      <c r="A51" s="82" t="n"/>
-      <c r="B51" s="82" t="n"/>
-      <c r="C51" s="82" t="n"/>
-      <c r="D51" s="82" t="n"/>
-      <c r="E51" s="82" t="n"/>
-      <c r="F51" s="82" t="n"/>
-      <c r="G51" s="82" t="n"/>
+      <c r="A51" s="74" t="n"/>
+      <c r="B51" s="74" t="n"/>
+      <c r="C51" s="74" t="n"/>
+      <c r="D51" s="74" t="n"/>
+      <c r="E51" s="74" t="n"/>
+      <c r="F51" s="74" t="n"/>
+      <c r="G51" s="74" t="n"/>
     </row>
     <row r="52" ht="16" customHeight="1">
-      <c r="A52" s="82" t="n"/>
-      <c r="B52" s="82" t="n"/>
-      <c r="C52" s="82" t="n"/>
-      <c r="D52" s="82" t="n"/>
-      <c r="E52" s="82" t="n"/>
-      <c r="F52" s="82" t="n"/>
-      <c r="G52" s="82" t="n"/>
+      <c r="A52" s="74" t="n"/>
+      <c r="B52" s="74" t="n"/>
+      <c r="C52" s="74" t="n"/>
+      <c r="D52" s="74" t="n"/>
+      <c r="E52" s="74" t="n"/>
+      <c r="F52" s="74" t="n"/>
+      <c r="G52" s="74" t="n"/>
     </row>
     <row r="53" ht="16" customHeight="1">
-      <c r="A53" s="82" t="n"/>
-      <c r="B53" s="82" t="n"/>
-      <c r="C53" s="82" t="n"/>
-      <c r="D53" s="82" t="n"/>
-      <c r="E53" s="82" t="n"/>
-      <c r="F53" s="82" t="n"/>
-      <c r="G53" s="82" t="n"/>
+      <c r="A53" s="74" t="n"/>
+      <c r="B53" s="74" t="n"/>
+      <c r="C53" s="74" t="n"/>
+      <c r="D53" s="74" t="n"/>
+      <c r="E53" s="74" t="n"/>
+      <c r="F53" s="74" t="n"/>
+      <c r="G53" s="74" t="n"/>
     </row>
     <row r="54" ht="16" customHeight="1">
-      <c r="A54" s="82" t="n"/>
-      <c r="B54" s="82" t="n"/>
-      <c r="C54" s="82" t="n"/>
-      <c r="D54" s="82" t="n"/>
-      <c r="E54" s="82" t="n"/>
-      <c r="F54" s="82" t="n"/>
-      <c r="G54" s="82" t="n"/>
+      <c r="A54" s="74" t="n"/>
+      <c r="B54" s="74" t="n"/>
+      <c r="C54" s="74" t="n"/>
+      <c r="D54" s="74" t="n"/>
+      <c r="E54" s="74" t="n"/>
+      <c r="F54" s="74" t="n"/>
+      <c r="G54" s="74" t="n"/>
     </row>
     <row r="55" ht="16" customHeight="1">
-      <c r="A55" s="82" t="n"/>
-      <c r="B55" s="82" t="n"/>
-      <c r="C55" s="82" t="n"/>
-      <c r="D55" s="82" t="n"/>
-      <c r="E55" s="82" t="n"/>
-      <c r="F55" s="82" t="n"/>
-      <c r="G55" s="82" t="n"/>
+      <c r="A55" s="74" t="n"/>
+      <c r="B55" s="74" t="n"/>
+      <c r="C55" s="74" t="n"/>
+      <c r="D55" s="74" t="n"/>
+      <c r="E55" s="74" t="n"/>
+      <c r="F55" s="74" t="n"/>
+      <c r="G55" s="74" t="n"/>
     </row>
     <row r="56" ht="16" customHeight="1">
-      <c r="A56" s="82" t="n"/>
-      <c r="B56" s="82" t="n"/>
-      <c r="C56" s="82" t="n"/>
-      <c r="D56" s="82" t="n"/>
-      <c r="E56" s="82" t="n"/>
-      <c r="F56" s="82" t="n"/>
-      <c r="G56" s="82" t="n"/>
+      <c r="A56" s="74" t="n"/>
+      <c r="B56" s="74" t="n"/>
+      <c r="C56" s="74" t="n"/>
+      <c r="D56" s="74" t="n"/>
+      <c r="E56" s="74" t="n"/>
+      <c r="F56" s="74" t="n"/>
+      <c r="G56" s="74" t="n"/>
     </row>
     <row r="57" ht="16" customHeight="1">
-      <c r="A57" s="82" t="n"/>
-      <c r="B57" s="82" t="n"/>
-      <c r="C57" s="82" t="n"/>
-      <c r="D57" s="82" t="n"/>
-      <c r="E57" s="82" t="n"/>
-      <c r="F57" s="82" t="n"/>
-      <c r="G57" s="82" t="n"/>
+      <c r="A57" s="74" t="n"/>
+      <c r="B57" s="74" t="n"/>
+      <c r="C57" s="74" t="n"/>
+      <c r="D57" s="74" t="n"/>
+      <c r="E57" s="74" t="n"/>
+      <c r="F57" s="74" t="n"/>
+      <c r="G57" s="74" t="n"/>
     </row>
     <row r="58" ht="16" customHeight="1">
-      <c r="A58" s="82" t="n"/>
-      <c r="B58" s="82" t="n"/>
-      <c r="C58" s="82" t="n"/>
-      <c r="D58" s="82" t="n"/>
-      <c r="E58" s="82" t="n"/>
-      <c r="F58" s="82" t="n"/>
-      <c r="G58" s="82" t="n"/>
+      <c r="A58" s="74" t="n"/>
+      <c r="B58" s="74" t="n"/>
+      <c r="C58" s="74" t="n"/>
+      <c r="D58" s="74" t="n"/>
+      <c r="E58" s="74" t="n"/>
+      <c r="F58" s="74" t="n"/>
+      <c r="G58" s="74" t="n"/>
     </row>
     <row r="59" ht="16" customHeight="1">
-      <c r="A59" s="82" t="n"/>
-      <c r="B59" s="82" t="n"/>
-      <c r="C59" s="82" t="n"/>
-      <c r="D59" s="82" t="n"/>
-      <c r="E59" s="82" t="n"/>
-      <c r="F59" s="82" t="n"/>
-      <c r="G59" s="82" t="n"/>
+      <c r="A59" s="74" t="n"/>
+      <c r="B59" s="74" t="n"/>
+      <c r="C59" s="74" t="n"/>
+      <c r="D59" s="74" t="n"/>
+      <c r="E59" s="74" t="n"/>
+      <c r="F59" s="74" t="n"/>
+      <c r="G59" s="74" t="n"/>
+    </row>
+    <row r="60" ht="16" customHeight="1">
+      <c r="A60" s="74" t="n"/>
+      <c r="B60" s="74" t="n"/>
+      <c r="C60" s="74" t="n"/>
+      <c r="D60" s="74" t="n"/>
+      <c r="E60" s="74" t="n"/>
+      <c r="F60" s="74" t="n"/>
+      <c r="G60" s="74" t="n"/>
+    </row>
+    <row r="61" ht="16" customHeight="1">
+      <c r="A61" s="74" t="n"/>
+      <c r="B61" s="74" t="n"/>
+      <c r="C61" s="74" t="n"/>
+      <c r="D61" s="74" t="n"/>
+      <c r="E61" s="74" t="n"/>
+      <c r="F61" s="74" t="n"/>
+      <c r="G61" s="74" t="n"/>
+    </row>
+    <row r="62" ht="16" customHeight="1">
+      <c r="A62" s="74" t="n"/>
+      <c r="B62" s="74" t="n"/>
+      <c r="C62" s="74" t="n"/>
+      <c r="D62" s="74" t="n"/>
+      <c r="E62" s="74" t="n"/>
+      <c r="F62" s="74" t="n"/>
+      <c r="G62" s="74" t="n"/>
+    </row>
+    <row r="63" ht="16" customHeight="1">
+      <c r="A63" s="74" t="n"/>
+      <c r="B63" s="74" t="n"/>
+      <c r="C63" s="74" t="n"/>
+      <c r="D63" s="74" t="n"/>
+      <c r="E63" s="74" t="n"/>
+      <c r="F63" s="74" t="n"/>
+      <c r="G63" s="74" t="n"/>
+    </row>
+    <row r="64" ht="16" customHeight="1">
+      <c r="A64" s="74" t="n"/>
+      <c r="B64" s="74" t="n"/>
+      <c r="C64" s="74" t="n"/>
+      <c r="D64" s="74" t="n"/>
+      <c r="E64" s="74" t="n"/>
+      <c r="F64" s="74" t="n"/>
+      <c r="G64" s="74" t="n"/>
+    </row>
+    <row r="65" ht="16" customHeight="1">
+      <c r="A65" s="74" t="n"/>
+      <c r="B65" s="74" t="n"/>
+      <c r="C65" s="74" t="n"/>
+      <c r="D65" s="74" t="n"/>
+      <c r="E65" s="74" t="n"/>
+      <c r="F65" s="74" t="n"/>
+      <c r="G65" s="74" t="n"/>
+    </row>
+    <row r="66" ht="16" customHeight="1">
+      <c r="A66" s="74" t="n"/>
+      <c r="B66" s="74" t="n"/>
+      <c r="C66" s="74" t="n"/>
+      <c r="D66" s="74" t="n"/>
+      <c r="E66" s="74" t="n"/>
+      <c r="F66" s="74" t="n"/>
+      <c r="G66" s="74" t="n"/>
+    </row>
+    <row r="67" ht="16" customHeight="1">
+      <c r="A67" s="74" t="n"/>
+      <c r="B67" s="74" t="n"/>
+      <c r="C67" s="74" t="n"/>
+      <c r="D67" s="74" t="n"/>
+      <c r="E67" s="74" t="n"/>
+      <c r="F67" s="74" t="n"/>
+      <c r="G67" s="74" t="n"/>
+    </row>
+    <row r="68" ht="16" customHeight="1">
+      <c r="A68" s="74" t="n"/>
+      <c r="B68" s="74" t="n"/>
+      <c r="C68" s="74" t="n"/>
+      <c r="D68" s="74" t="n"/>
+      <c r="E68" s="74" t="n"/>
+      <c r="F68" s="74" t="n"/>
+      <c r="G68" s="74" t="n"/>
+    </row>
+    <row r="69" ht="16" customHeight="1">
+      <c r="A69" s="74" t="n"/>
+      <c r="B69" s="74" t="n"/>
+      <c r="C69" s="74" t="n"/>
+      <c r="D69" s="74" t="n"/>
+      <c r="E69" s="74" t="n"/>
+      <c r="F69" s="74" t="n"/>
+      <c r="G69" s="74" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="22">
     <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C24:D24"/>
     <mergeCell ref="C5:D5"/>
     <mergeCell ref="B10:G10"/>
     <mergeCell ref="C16:D16"/>
@@ -3473,6 +3833,7 @@
     <mergeCell ref="C21:D21"/>
     <mergeCell ref="C11:D11"/>
     <mergeCell ref="B4:G4"/>
+    <mergeCell ref="B26:G26"/>
     <mergeCell ref="C17:D17"/>
     <mergeCell ref="C23:D23"/>
     <mergeCell ref="C8:D8"/>
@@ -3483,7 +3844,7 @@
     <mergeCell ref="C3:D3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="E5 E6 E7 E8 E11 E12 E13 E16 E17 E18 E21 E22 E23 F5 F6 F7 F8 F11 F12 F13 F16 F17 F18 F21 F22 F23 G5 G6 G7 G8 G11 G12 G13 G16 G17 G18 G21 G22 G23" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="E5 E6 E7 E8 E11 E12 E13 E16 E17 E18 E21 E22 E23 E24 F5 F6 F7 F8 F11 F12 F13 F16 F17 F18 F21 F22 F23 F24 G5 G6 G7 G8 G11 G12 G13 G16 G17 G18 G21 G22 G23 G24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"✅ 済,⬜ 未,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>